<commit_message>
Génère les tables B'c et h_w du SiC et complète l'onglet SiC du classeur
- sic_bprime.py : équilibre à assemblage fixé résolu en potentiels
  élémentaires là où plusieurs solides coexistent (SiC + C(gr),
  SiC + SiO2(L) + Si(L)) et où Mutation++ ne converge pas ; les 4725
  points de la grille sont des équilibres strictement stables.
- Tables sic_bprime_table.csv, _bc_table.csv, _hw_table.csv (format et
  unités SI identiques au carbone et à la silice), _phases.csv
  (assemblage retenu en chaque point) et figure.
- README : choix du suivi sur N, méthode de calcul, régimes, domaine de
  validité de l'approche à l'équilibre.
- Classeur : valeurs calculées dans l'onglet SiC (comparaison des suivis
  N/Si/C, régimes à 1 atm), classeur régénéré et vérifié (638 formules,
  0 erreur).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TcAV8aPzoBRqLK16FKxnci
</commit_message>
<xml_diff>
--- a/mise_en_donnees_xlsx/mise_en_donnees_materiaux.xlsx
+++ b/mise_en_donnees_xlsx/mise_en_donnees_materiaux.xlsx
@@ -17,6 +17,7 @@
     <sheet name="Liège-phénolique" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Carbone" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Silice" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="SiC" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -178,7 +179,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -279,6 +280,7 @@
     <xf numFmtId="165" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -645,7 +647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I54"/>
+  <dimension ref="A1:I55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4.5" customWidth="1" min="1" max="1"/>
@@ -676,7 +678,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Fichier(s) XML : data/mixtures/ — 9 matériaux, 17 fichiers de mélange</t>
+          <t>Fichier(s) XML : data/mixtures/ — 10 matériaux, 18 fichiers de mélange</t>
         </is>
       </c>
     </row>
@@ -1017,97 +1019,106 @@
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="12" t="inlineStr">
-        <is>
-          <t>Les colonnes « gaz » sont des liens vers la ligne « valeur portée dans le XML » de chaque onglet. Le graphite et la silice n'ont pas de gaz de pyrolyse (k = 0). TACOT et CPh70 portent RIGOUREUSEMENT la même composition : leurs fichiers XML sont identiques, seul k les distingue — c'est la démonstration de l'onglet CPh70.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Carbure de silicium SiC</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t>Si:1.0, C:1.0</t>
+        </is>
+      </c>
+      <c r="H20" s="8">
+        <f>'SiC'!C69</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>Les colonnes « gaz » sont des liens vers la ligne « valeur portée dans le XML » de chaque onglet. Le graphite, la silice et le SiC n'ont pas de gaz de pyrolyse (k = 0). TACOT et CPh70 portent RIGOUREUSEMENT la même composition : leurs fichiers XML sont identiques, seul k les distingue — c'est la démonstration de l'onglet CPh70.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>§3 — LES TROIS SEULES DONNÉES QUE CONSOMME LE CALCUL</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="B23" s="6" t="inlineStr">
+    <row r="24">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>Composition</t>
         </is>
       </c>
-      <c r="D23" s="6" t="inlineStr">
+      <c r="D24" s="6" t="inlineStr">
         <is>
           <t>Rôle dans le bilan</t>
         </is>
       </c>
-      <c r="E23" s="6" t="inlineStr">
+      <c r="E24" s="6" t="inlineStr">
         <is>
           <t>Option</t>
         </is>
       </c>
-      <c r="F23" s="6" t="inlineStr">
+      <c r="F24" s="6" t="inlineStr">
         <is>
           <t>Comment on l'obtient</t>
         </is>
       </c>
-      <c r="G23" s="6" t="inlineStr"/>
-      <c r="H23" s="6" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="B24" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>bord de couche limite</t>
-        </is>
-      </c>
-      <c r="D24" s="7" t="inlineStr">
-        <is>
-          <t>Y_e</t>
-        </is>
-      </c>
-      <c r="E24" s="14" t="inlineStr">
-        <is>
-          <t>-bl</t>
-        </is>
-      </c>
-      <c r="F24" s="11" t="inlineStr">
-        <is>
-          <t>l'atmosphère : air N:0.79 O:0.21 · Mars · Titan…</t>
-        </is>
-      </c>
-      <c r="G24" s="15" t="inlineStr"/>
-      <c r="H24" s="15" t="inlineStr"/>
+      <c r="G24" s="6" t="inlineStr"/>
+      <c r="H24" s="6" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="B25" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>gaz de pyrolyse</t>
+          <t>bord de couche limite</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>Y_g</t>
+          <t>Y_e</t>
         </is>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>-py</t>
+          <t>-bl</t>
         </is>
       </c>
       <c r="F25" s="11" t="inlineStr">
         <is>
-          <t>c'est TOUT l'objet de ce classeur — quatre routes possibles, §4</t>
+          <t>l'atmosphère : air N:0.79 O:0.21 · Mars · Titan…</t>
         </is>
       </c>
       <c r="G25" s="15" t="inlineStr"/>
@@ -1115,127 +1126,125 @@
     </row>
     <row r="26">
       <c r="B26" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>char</t>
+          <t>gaz de pyrolyse</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Y_c</t>
+          <t>Y_g</t>
         </is>
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
-          <t>-char + -char-elem</t>
+          <t>-py</t>
         </is>
       </c>
       <c r="F26" s="11" t="inlineStr">
         <is>
-          <t>C:1.0 si tous les constituants carbonisent vers le carbone ; sinon pondérer par les masses de char</t>
+          <t>c'est TOUT l'objet de ce classeur — quatre routes possibles, §4</t>
         </is>
       </c>
       <c r="G26" s="15" t="inlineStr"/>
       <c r="H26" s="15" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="B27" s="12" t="inlineStr">
+      <c r="B27" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>char</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Y_c</t>
+        </is>
+      </c>
+      <c r="E27" s="14" t="inlineStr">
+        <is>
+          <t>-char + -char-elem</t>
+        </is>
+      </c>
+      <c r="F27" s="11" t="inlineStr">
+        <is>
+          <t>C:1.0 si tous les constituants carbonisent vers le carbone ; sinon pondérer par les masses de char</t>
+        </is>
+      </c>
+      <c r="G27" s="15" t="inlineStr"/>
+      <c r="H27" s="15" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="12" t="inlineStr">
         <is>
           <t>Plus T, P et B'g. Rien d'autre : cf. src/apps/bprime.cpp:304-330. Sans -char/-char-elem, bprime utilise un char de carbone pur intégré ; les deux options vont toujours ensemble.</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="4" t="inlineStr">
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>§4 — LES QUATRE ROUTES DE CALCUL DU GAZ DE PYROLYSE</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="B30" s="6" t="inlineStr">
+    <row r="31">
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="C30" s="6" t="inlineStr">
+      <c r="C31" s="6" t="inlineStr">
         <is>
           <t>Matériau</t>
         </is>
       </c>
-      <c r="D30" s="6" t="inlineStr">
+      <c r="D31" s="6" t="inlineStr">
         <is>
           <t>Donnée primaire</t>
         </is>
       </c>
-      <c r="E30" s="6" t="inlineStr">
+      <c r="E31" s="6" t="inlineStr">
         <is>
           <t>Passage à l'élémentaire</t>
         </is>
       </c>
-      <c r="F30" s="6" t="inlineStr">
+      <c r="F31" s="6" t="inlineStr">
         <is>
           <t>Point critique</t>
         </is>
       </c>
-      <c r="G30" s="6" t="inlineStr"/>
-      <c r="H30" s="6" t="inlineStr"/>
-    </row>
-    <row r="31" ht="28" customHeight="1">
-      <c r="B31" s="16" t="inlineStr">
-        <is>
-          <t>A — sommation atomique</t>
-        </is>
-      </c>
-      <c r="C31" s="17" t="inlineStr">
-        <is>
-          <t>TACOT, CPh70</t>
-        </is>
-      </c>
-      <c r="D31" s="17" t="inlineStr">
-        <is>
-          <t>spéciation moléculaire mesurée (7 espèces)</t>
-        </is>
-      </c>
-      <c r="E31" s="18" t="inlineStr">
-        <is>
-          <t>n_E = Σ_j ν_E,j · x_j</t>
-        </is>
-      </c>
-      <c r="F31" s="19" t="inlineStr">
-        <is>
-          <t>la renormalisation : somme réelle des colonnes (100.30), pas les totaux imprimés (100.0)</t>
-        </is>
-      </c>
-      <c r="G31" s="15" t="inlineStr"/>
-      <c r="H31" s="15" t="inlineStr"/>
+      <c r="G31" s="6" t="inlineStr"/>
+      <c r="H31" s="6" t="inlineStr"/>
     </row>
     <row r="32" ht="28" customHeight="1">
       <c r="B32" s="16" t="inlineStr">
         <is>
-          <t>B — conversion directe</t>
+          <t>A — sommation atomique</t>
         </is>
       </c>
       <c r="C32" s="17" t="inlineStr">
         <is>
-          <t>ZURAM</t>
+          <t>TACOT, CPh70</t>
         </is>
       </c>
       <c r="D32" s="17" t="inlineStr">
         <is>
-          <t>composition élémentaire MASSIQUE mesurée</t>
+          <t>spéciation moléculaire mesurée (7 espèces)</t>
         </is>
       </c>
       <c r="E32" s="18" t="inlineStr">
         <is>
-          <t>x_E = (y_E/M_E) / Σ (y_j/M_j)</t>
+          <t>n_E = Σ_j ν_E,j · x_j</t>
         </is>
       </c>
       <c r="F32" s="19" t="inlineStr">
         <is>
-          <t>traçabilité limitée à 3 décimales ; la source primaire VKI n'est pas publique</t>
+          <t>la renormalisation : somme réelle des colonnes (100.30), pas les totaux imprimés (100.0)</t>
         </is>
       </c>
       <c r="G32" s="15" t="inlineStr"/>
@@ -1244,27 +1253,27 @@
     <row r="33" ht="28" customHeight="1">
       <c r="B33" s="16" t="inlineStr">
         <is>
-          <t>C — fermeture élémentaire</t>
+          <t>B — conversion directe</t>
         </is>
       </c>
       <c r="C33" s="17" t="inlineStr">
         <is>
-          <t>SC-1008</t>
+          <t>ZURAM</t>
         </is>
       </c>
       <c r="D33" s="17" t="inlineStr">
         <is>
-          <t>motif chimique idéalisé + rendement en char</t>
+          <t>composition élémentaire MASSIQUE mesurée</t>
         </is>
       </c>
       <c r="E33" s="18" t="inlineStr">
         <is>
-          <t>n_E(gaz) = n_E(résine) − n_E(char)</t>
+          <t>x_E = (y_E/M_E) / Σ (y_j/M_j)</t>
         </is>
       </c>
       <c r="F33" s="19" t="inlineStr">
         <is>
-          <t>le rendement en char entre DANS la chaîne : ±0.05 sur Y déplace le carbone de ~12 %</t>
+          <t>traçabilité limitée à 3 décimales ; la source primaire VKI n'est pas publique</t>
         </is>
       </c>
       <c r="G33" s="15" t="inlineStr"/>
@@ -1273,27 +1282,27 @@
     <row r="34" ht="28" customHeight="1">
       <c r="B34" s="16" t="inlineStr">
         <is>
-          <t>D — fermeture sur DEUX constituants</t>
+          <t>C — fermeture élémentaire</t>
         </is>
       </c>
       <c r="C34" s="17" t="inlineStr">
         <is>
-          <t>Liège/phénolique</t>
+          <t>SC-1008</t>
         </is>
       </c>
       <c r="D34" s="17" t="inlineStr">
         <is>
-          <t>analyses des deux constituants + rendements</t>
+          <t>motif chimique idéalisé + rendement en char</t>
         </is>
       </c>
       <c r="E34" s="18" t="inlineStr">
         <is>
-          <t>n_E(gaz) = Σ_i [n_E(i) − n_E(char,i)]</t>
+          <t>n_E(gaz) = n_E(résine) − n_E(char)</t>
         </is>
       </c>
       <c r="F34" s="19" t="inlineStr">
         <is>
-          <t>le renfort pyrolyse : le rapport renfort/résine entre dans la table B'</t>
+          <t>le rendement en char entre DANS la chaîne : ±0.05 sur Y déplace le carbone de ~12 %</t>
         </is>
       </c>
       <c r="G34" s="15" t="inlineStr"/>
@@ -1302,85 +1311,93 @@
     <row r="35" ht="28" customHeight="1">
       <c r="B35" s="16" t="inlineStr">
         <is>
-          <t>E — stœchiométrie directe</t>
+          <t>D — fermeture sur DEUX constituants</t>
         </is>
       </c>
       <c r="C35" s="17" t="inlineStr">
         <is>
-          <t>Carbone, Silice</t>
+          <t>Liège/phénolique</t>
         </is>
       </c>
       <c r="D35" s="17" t="inlineStr">
         <is>
-          <t>la formule du solide</t>
+          <t>analyses des deux constituants + rendements</t>
         </is>
       </c>
       <c r="E35" s="18" t="inlineStr">
         <is>
-          <t>aucun gaz de pyrolyse (B'g = 0)</t>
+          <t>n_E(gaz) = Σ_i [n_E(i) − n_E(char,i)]</t>
         </is>
       </c>
       <c r="F35" s="19" t="inlineStr">
         <is>
-          <t>le char EST le matériau ; pour la silice, -char-elem devient Si</t>
+          <t>le renfort pyrolyse : le rapport renfort/résine entre dans la table B'</t>
         </is>
       </c>
       <c r="G35" s="15" t="inlineStr"/>
       <c r="H35" s="15" t="inlineStr"/>
     </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="4" t="inlineStr">
+    <row r="36" ht="28" customHeight="1">
+      <c r="B36" s="16" t="inlineStr">
+        <is>
+          <t>E — stœchiométrie directe</t>
+        </is>
+      </c>
+      <c r="C36" s="17" t="inlineStr">
+        <is>
+          <t>Carbone, Silice, SiC</t>
+        </is>
+      </c>
+      <c r="D36" s="17" t="inlineStr">
+        <is>
+          <t>la formule du solide</t>
+        </is>
+      </c>
+      <c r="E36" s="18" t="inlineStr">
+        <is>
+          <t>aucun gaz de pyrolyse (B'g = 0)</t>
+        </is>
+      </c>
+      <c r="F36" s="19" t="inlineStr">
+        <is>
+          <t>le char EST le matériau ; -char-elem Si pour la silice, N pour le SiC (char non congruent)</t>
+        </is>
+      </c>
+      <c r="G36" s="15" t="inlineStr"/>
+      <c r="H36" s="15" t="inlineStr"/>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>§5 — CE QUI N'ENTRE PAS DANS LE XML</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="B38" s="6" t="inlineStr">
+    <row r="39">
+      <c r="B39" s="6" t="inlineStr">
         <is>
           <t>Donnée</t>
         </is>
       </c>
-      <c r="C38" s="6" t="inlineStr">
+      <c r="C39" s="6" t="inlineStr">
         <is>
           <t>Dans le XML ?</t>
         </is>
       </c>
-      <c r="D38" s="6" t="inlineStr">
+      <c r="D39" s="6" t="inlineStr">
         <is>
           <t>Où elle sert vraiment</t>
         </is>
       </c>
-      <c r="E38" s="6" t="inlineStr"/>
-      <c r="F38" s="6" t="inlineStr"/>
-      <c r="G38" s="6" t="inlineStr"/>
-      <c r="H38" s="6" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="B39" s="7" t="inlineStr">
-        <is>
-          <t>masse volumique ρ_v, ρ_c</t>
-        </is>
-      </c>
-      <c r="C39" s="13" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="D39" s="11" t="inlineStr">
-        <is>
-          <t>solveur de réponse matériau ; récession ṡ = B'c·ṁe/ρ_c</t>
-        </is>
-      </c>
-      <c r="E39" s="15" t="inlineStr"/>
-      <c r="F39" s="15" t="inlineStr"/>
-      <c r="G39" s="15" t="inlineStr"/>
-      <c r="H39" s="15" t="inlineStr"/>
+      <c r="E39" s="6" t="inlineStr"/>
+      <c r="F39" s="6" t="inlineStr"/>
+      <c r="G39" s="6" t="inlineStr"/>
+      <c r="H39" s="6" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>porosité</t>
+          <t>masse volumique ρ_v, ρ_c</t>
         </is>
       </c>
       <c r="C40" s="13" t="inlineStr">
@@ -1390,7 +1407,7 @@
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>conduction, perméabilité</t>
+          <t>solveur de réponse matériau ; récession ṡ = B'c·ṁe/ρ_c</t>
         </is>
       </c>
       <c r="E40" s="15" t="inlineStr"/>
@@ -1401,17 +1418,17 @@
     <row r="41">
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>rapport fibres/résine</t>
+          <t>porosité</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
         <is>
-          <t>non *</t>
+          <t>non</t>
         </is>
       </c>
       <c r="D41" s="11" t="inlineStr">
         <is>
-          <t>fixe la QUANTITÉ de gaz (donc B'g), pas sa composition</t>
+          <t>conduction, perméabilité</t>
         </is>
       </c>
       <c r="E41" s="15" t="inlineStr"/>
@@ -1422,7 +1439,7 @@
     <row r="42">
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>rendement en char</t>
+          <t>rapport fibres/résine</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
@@ -1432,7 +1449,7 @@
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>idem — mais il entre dans le CALCUL du gaz pour les routes C et D</t>
+          <t>fixe la QUANTITÉ de gaz (donc B'g), pas sa composition</t>
         </is>
       </c>
       <c r="E42" s="15" t="inlineStr"/>
@@ -1443,17 +1460,17 @@
     <row r="43">
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>cinétique de pyrolyse</t>
+          <t>rendement en char</t>
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr">
         <is>
-          <t>non</t>
+          <t>non *</t>
         </is>
       </c>
       <c r="D43" s="11" t="inlineStr">
         <is>
-          <t>fixe B'g au cours du temps</t>
+          <t>idem — mais il entre dans le CALCUL du gaz pour les routes C et D</t>
         </is>
       </c>
       <c r="E43" s="15" t="inlineStr"/>
@@ -1462,109 +1479,130 @@
       <c r="H43" s="15" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="B44" s="12" t="inlineStr">
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>cinétique de pyrolyse</t>
+        </is>
+      </c>
+      <c r="C44" s="13" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="D44" s="11" t="inlineStr">
+        <is>
+          <t>fixe B'g au cours du temps</t>
+        </is>
+      </c>
+      <c r="E44" s="15" t="inlineStr"/>
+      <c r="F44" s="15" t="inlineStr"/>
+      <c r="G44" s="15" t="inlineStr"/>
+      <c r="H44" s="15" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="B45" s="12" t="inlineStr">
         <is>
           <t>* sauf si les constituants donnent des chars de compositions élémentaires DIFFÉRENTES (fibres de silice + résine phénolique), ou si le renfort pyrolyse (liège) : le rapport entre alors dans Y_c et/ou Y_g, et la table change. Le bilan de masse de surface est écrit sur des fractions massiques élémentaires, donc normalisées : les grandeurs VOLUMIQUES n'y ont structurellement aucune place.</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="4" t="inlineStr">
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="4" t="inlineStr">
         <is>
           <t>§6 — RECETTE POUR UN NOUVEAU MATÉRIAU</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="B47" s="5" t="inlineStr">
-        <is>
-          <t>Atmosphère → composition -bl (air, Mars, Titan…).</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>Résine → composition du gaz de pyrolyse par l'une des quatre routes du §4 → composition -py.</t>
+          <t>Atmosphère → composition -bl (air, Mars, Titan…).</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>Char → C:1.0 si tous les constituants carbonisent vers le carbone ; sinon pondérer par les masses de char de chaque constituant.</t>
+          <t>Résine → composition du gaz de pyrolyse par l'une des quatre routes du §4 → composition -py.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>Espèces → tous les produits attendus des éléments présents, PLUS la ou les phases condensées.</t>
+          <t>Char → C:1.0 si tous les constituants carbonisent vers le carbone ; sinon pondérer par les masses de char de chaque constituant.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>Vérifier : checkmix (noms, phases), puis un run court.</t>
+          <t>Espèces → tous les produits attendus des éléments présents, PLUS la ou les phases condensées.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>Vérifier : checkmix (noms, phases), puis un run court.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="B52" s="5" t="inlineStr">
-        <is>
-          <t>Contrôler la physique : à 300 K et B'g = 0 dans l'air, un char carboné doit donner B'c ≈ 0.0874 (limite C + O2 → CO2, indépendante de la pression). Une valeur ≈ 200 signale l'absence de C(gr).</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="30" customHeight="1">
-      <c r="B54" s="5" t="inlineStr">
-        <is>
-          <t>Documents de référence du dépôt : tacot_bprime/mise_en_donnees_xml.md (mécanique du fichier XML et règles du parseur) · resine_tacot.md · zuram_bprime/resine_zuram.md · sc1008_bprime/resine_sc1008.md · cork_bprime/mise_en_donnees_cork.md · tacot_bprime/cph70_vs_tacot.md · carbon_bprime/bprime_carbon_physique.md.</t>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>Contrôler la physique : à 300 K et B'g = 0 dans l'air, un char carboné doit donner B'c ≈ 0.0874 (limite C + O2 → CO2, indépendante de la pression). Une valeur ≈ 200 signale l'absence de C(gr). Pour un char multi-élément susceptible de laisser un autre solide à la paroi (SiC), suivre le bilan sur N (-char-elem N).</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="30" customHeight="1">
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>Documents de référence du dépôt : tacot_bprime/mise_en_donnees_xml.md (mécanique du fichier XML et règles du parseur) · resine_tacot.md · zuram_bprime/resine_zuram.md · sc1008_bprime/resine_sc1008.md · cork_bprime/mise_en_donnees_cork.md · tacot_bprime/cph70_vs_tacot.md · carbon_bprime/bprime_carbon_physique.md · sic_bprime/README.md.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="22">
     <mergeCell ref="B7:I7"/>
-    <mergeCell ref="A37:I37"/>
-    <mergeCell ref="A46:I46"/>
-    <mergeCell ref="B47:I47"/>
-    <mergeCell ref="B54:I54"/>
     <mergeCell ref="A3:I3"/>
-    <mergeCell ref="B27:I27"/>
     <mergeCell ref="B52:I52"/>
+    <mergeCell ref="B21:I21"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="B48:I48"/>
+    <mergeCell ref="A47:I47"/>
     <mergeCell ref="A5:I5"/>
-    <mergeCell ref="A22:I22"/>
+    <mergeCell ref="A23:I23"/>
     <mergeCell ref="B8:I8"/>
-    <mergeCell ref="A29:I29"/>
-    <mergeCell ref="B44:I44"/>
+    <mergeCell ref="A38:I38"/>
+    <mergeCell ref="B53:I53"/>
     <mergeCell ref="A10:I10"/>
+    <mergeCell ref="B28:I28"/>
     <mergeCell ref="B49:I49"/>
+    <mergeCell ref="A30:I30"/>
+    <mergeCell ref="B55:I55"/>
     <mergeCell ref="B6:I6"/>
     <mergeCell ref="B51:I51"/>
-    <mergeCell ref="B20:I20"/>
     <mergeCell ref="A1:I1"/>
+    <mergeCell ref="B45:I45"/>
     <mergeCell ref="B50:I50"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1602,7 +1640,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Le seul matériau du dépôt dont le char n'est pas du carbone : montre comment se remplit une composition à plusieurs éléments</t>
+          <t>Premier char du dépôt qui n'est pas du carbone (avec le SiC) : montre comment se remplit une composition à plusieurs éléments</t>
         </is>
       </c>
     </row>
@@ -2233,6 +2271,1182 @@
     <mergeCell ref="A45:I45"/>
     <mergeCell ref="B35:I35"/>
     <mergeCell ref="B50:I50"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="007030A0"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I88"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4.5" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="72" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Carbure de silicium SiC — char multi-élément NON congruent</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Char à deux éléments qui peut laisser à la paroi SiO2, Si liquide ou carbone : le bilan est suivi sur l'azote de l'air</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Fichier(s) XML : data/mixtures/sic-air.xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>§0 — FICHE D'IDENTITÉ</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="35" t="inlineStr">
+        <is>
+          <t>Matériau</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="inlineStr">
+        <is>
+          <t>carbure de silicium massif β-SiC (dense, fritté ou CVD)</t>
+        </is>
+      </c>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>sic_bprime/sic_bprime.py · sic_bprime/README.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="35" t="inlineStr">
+        <is>
+          <t>Système chimique</t>
+        </is>
+      </c>
+      <c r="C7" s="30" t="inlineStr">
+        <is>
+          <t>Si-C-N-O : 5 espèces d'air + 6 gaz carbonés + 10 gaz siliciés (SiO, SiO2, SiC, SiC2, Si2C, SiN…) + 9 phases condensées</t>
+        </is>
+      </c>
+      <c r="I7" s="12" t="inlineStr">
+        <is>
+          <t>30 espèces au total</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="35" t="inlineStr">
+        <is>
+          <t>Phases condensées</t>
+        </is>
+      </c>
+      <c r="C8" s="30" t="inlineStr">
+        <is>
+          <t>C(gr) · Si(cr), Si(L) · SiC(b), SiC(L) · SiO2(a-qz), SiO2(b-qz), SiO2(b-crt), SiO2(L)</t>
+        </is>
+      </c>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>une seule forme de chaque famille est valide à une température donnée</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="35" t="inlineStr">
+        <is>
+          <t>Binaire</t>
+        </is>
+      </c>
+      <c r="C9" s="30" t="inlineStr">
+        <is>
+          <t>bprime généralisé : -char sic -char-elem N</t>
+        </is>
+      </c>
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>aucun binaire dédié (contrairement à bprime_silica)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="35" t="inlineStr">
+        <is>
+          <t>Compositions du XML</t>
+        </is>
+      </c>
+      <c r="C10" s="30" t="inlineStr">
+        <is>
+          <t>air (-bl) · sic (char, -char)</t>
+        </is>
+      </c>
+      <c r="I10" s="12" t="inlineStr"/>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>§1 — HYPOTHÈSES</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="A13" s="20" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Le char est le SiC lui-même, de stœchiométrie Si:C = 1:1 exacte.</t>
+        </is>
+      </c>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>Matériau monolithique : pas de résine, donc pas de gaz de pyrolyse (B'g = 0) et pas de fermeture élémentaire à faire.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="26" customHeight="1">
+      <c r="A14" s="20" t="inlineStr">
+        <is>
+          <t>H2</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>L'élément du bilan est l'AZOTE de l'air, pas Si ni C.</t>
+        </is>
+      </c>
+      <c r="I14" s="12" t="inlineStr">
+        <is>
+          <t>Le SiC ne se consomme pas toujours en bloc : selon (T_w, P) il laisse de la silice (oxydation passive), du silicium liquide ou un résidu de carbone (décomposition SiC → Si(g) + C(gr)). Suivre Si ou C donne alors un B'c faux — nul, ou négatif puis écrêté, alors que le matériau se décompose (§5). N est inerte et absent de toute phase condensée : son bilan donne la masse NETTE gazéifiée par la paroi. Pour le carbone et la silice, dont le char est la seule phase condensée, le résultat est identique à celui du suivi sur C ou sur Si.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>H3</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Toutes les phases condensées du système Si-C-O figurent dans &lt;species&gt;, sauf Si3N4.</t>
+        </is>
+      </c>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>Même exigence que C(gr) pour le carbone : sans SiO2 condensée, l'oxydation passive disparaît ; sans C(gr), le résidu de décomposition ne peut pas se former. Si3N4(cr) est écarté : il bloque le solveur, et la nitruration du SiC sous air est cinétiquement inhibée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="26" customHeight="1">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Équilibre thermochimique à la paroi, vérifié point par point.</t>
+        </is>
+      </c>
+      <c r="I16" s="12" t="inlineStr">
+        <is>
+          <t>Le solveur multiphase boucle sur ~7 % des points (frontières de phases). Chaque point est contrôlé : aucune phase absente ne doit avoir une force motrice g°/RT − Σ a·λ négative. Sinon les assemblages de phases sont énumérés et celui qui vérifie ce critère est retenu (équilibre vrai). Là où plusieurs solides coexistent (SiC + C(gr), SiC + SiO2 + Si(L)), l'équilibre à assemblage fixé est résolu directement en potentiels élémentaires. Bilan : 4387 points directs, 289 par énumération, 49 à assemblage fixé, tous strictement stables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>§2 — DONNÉES D'ENTRÉE</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="35" t="inlineStr">
+        <is>
+          <t>stœchiométrie — ν_Si</t>
+        </is>
+      </c>
+      <c r="C19" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="12" t="inlineStr">
+        <is>
+          <t>SiC</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="35" t="inlineStr">
+        <is>
+          <t>stœchiométrie — ν_C</t>
+        </is>
+      </c>
+      <c r="C20" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" s="12" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="35" t="inlineStr">
+        <is>
+          <t>fraction massique d'oxygène de l'air</t>
+        </is>
+      </c>
+      <c r="C21" s="50">
+        <f>Constantes!D19</f>
+        <v>0.23290921795842306</v>
+      </c>
+      <c r="I21" s="12" t="inlineStr">
+        <is>
+          <t>y_O calculé au §2 de l'onglet Constantes</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="35" t="inlineStr">
+        <is>
+          <t>fraction massique d'azote de l'air</t>
+        </is>
+      </c>
+      <c r="C22" s="50">
+        <f>Constantes!C19</f>
+        <v>0.7670907820415769</v>
+      </c>
+      <c r="I22" s="12" t="inlineStr">
+        <is>
+          <t>y_N — l'élément de suivi du bilan (H2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="35" t="inlineStr">
+        <is>
+          <t>masse volumique du SiC [kg/m³]</t>
+        </is>
+      </c>
+      <c r="C23" s="30" t="n">
+        <v>3210</v>
+      </c>
+      <c r="I23" s="12" t="inlineStr">
+        <is>
+          <t>β-SiC dense — n'entre que dans la récession</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>§3 — CALCUL PAS À PAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="20" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="B26" s="20" t="inlineStr">
+        <is>
+          <t>Étape 1 — masse molaire du motif</t>
+        </is>
+      </c>
+      <c r="I26" s="27" t="inlineStr">
+        <is>
+          <t>M = ν_Si·M_Si + ν_C·M_C</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="35" t="inlineStr">
+        <is>
+          <t>M(SiC) [g/mol]</t>
+        </is>
+      </c>
+      <c r="C27" s="70">
+        <f>C19*Constantes!$C$11+C20*Constantes!$C$7</f>
+        <v>40.0965</v>
+      </c>
+      <c r="I27" s="12" t="inlineStr">
+        <is>
+          <t>attendu 40.10 g/mol</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="20" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="B28" s="20" t="inlineStr">
+        <is>
+          <t>Étape 2 — composition élémentaire, en molaire puis en massique</t>
+        </is>
+      </c>
+      <c r="I28" s="27" t="inlineStr">
+        <is>
+          <t>x_E = ν_E / Σ ν_j ;  y_E = ν_E·M_E / M</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="6" t="inlineStr"/>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>Somme</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr"/>
+      <c r="G29" s="6" t="inlineStr"/>
+      <c r="H29" s="6" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>ν_E (moles d'atomes par motif)</t>
+        </is>
+      </c>
+      <c r="C30" s="24">
+        <f>C19</f>
+        <v>1.0</v>
+      </c>
+      <c r="D30" s="24">
+        <f>C20</f>
+        <v>1.0</v>
+      </c>
+      <c r="E30" s="24">
+        <f>SUM(C30:D30)</f>
+        <v>2.0</v>
+      </c>
+      <c r="F30" s="15" t="inlineStr"/>
+      <c r="G30" s="15" t="inlineStr"/>
+      <c r="H30" s="15" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>x_E (fraction molaire élémentaire, normalisée)</t>
+        </is>
+      </c>
+      <c r="C31" s="26">
+        <f>C30/$E$30</f>
+        <v>0.5</v>
+      </c>
+      <c r="D31" s="26">
+        <f>D30/$E$30</f>
+        <v>0.5</v>
+      </c>
+      <c r="E31" s="24">
+        <f>SUM(C31:D31)</f>
+        <v>1.0</v>
+      </c>
+      <c r="F31" s="15" t="inlineStr"/>
+      <c r="G31" s="15" t="inlineStr"/>
+      <c r="H31" s="15" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>y_E (fraction massique élémentaire)</t>
+        </is>
+      </c>
+      <c r="C32" s="26">
+        <f>C30*Constantes!$C$11/$C$27</f>
+        <v>0.7004476699961344</v>
+      </c>
+      <c r="D32" s="26">
+        <f>D30*Constantes!$C$7/$C$27</f>
+        <v>0.29955233000386566</v>
+      </c>
+      <c r="E32" s="24">
+        <f>SUM(C32:D32)</f>
+        <v>1.0</v>
+      </c>
+      <c r="F32" s="15" t="inlineStr"/>
+      <c r="G32" s="15" t="inlineStr"/>
+      <c r="H32" s="15" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>Attendu : x_Si = x_C = 0.5000 en molaire, y_Si = 0.7005 / y_C = 0.2995 en masse.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="20" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="B34" s="20" t="inlineStr">
+        <is>
+          <t>Étape 3 — le bilan de surface, écrit sur l'azote</t>
+        </is>
+      </c>
+      <c r="I34" s="27" t="inlineStr">
+        <is>
+          <t>B'c = [Y_e,N + B'g·Y_g,N − Y_w,N(1+B'g)] / (Y_w,N − Y_c,N)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="16" customHeight="1">
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Avec Y_c,N = 0 (le char ne contient pas d'azote) et B'g = 0, il ne reste que :</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   B'c = Y_e,N / Y_w,N − 1        (masse nette gazéifiée par unité de masse d'air)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Le gaz à la paroi contient (1 + B'c) fois la masse d'air qui y entre ; l'azote, qui ne se dépose nulle part, s'y trouve dilué d'autant. Si la paroi FIXE de l'oxygène (silice d'oxydation passive), la masse gazéifiée nette est négative : bprime écrête B'c à 0, comme pour tous les matériaux.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>§4 — RÉSULTAT : CE QUI ENTRE DANS LE XML</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>Composition élémentaire</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="inlineStr">
+        <is>
+          <t>Somme</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>après normalisation par le parseur</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="inlineStr"/>
+      <c r="H40" s="6" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>valeur portée dans le XML (sic)</t>
+        </is>
+      </c>
+      <c r="C41" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" s="24">
+        <f>SUM(C41:D41)</f>
+        <v>2.0</v>
+      </c>
+      <c r="F41" s="11" t="inlineStr">
+        <is>
+          <t>x_Si = x_C = 1/2</t>
+        </is>
+      </c>
+      <c r="G41" s="15" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>air — valeur portée dans le XML</t>
+        </is>
+      </c>
+      <c r="C42" s="74" t="inlineStr">
+        <is>
+          <t>N : 0.79</t>
+        </is>
+      </c>
+      <c r="D42" s="74" t="inlineStr">
+        <is>
+          <t>O : 0.21</t>
+        </is>
+      </c>
+      <c r="E42" s="15" t="inlineStr"/>
+      <c r="F42" s="15" t="inlineStr"/>
+      <c r="G42" s="15" t="inlineStr"/>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>§5 — CONTRÔLES ET VALIDATION CROISÉE</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="20" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="B45" s="20" t="inlineStr">
+        <is>
+          <t>Contrôle 1 — plateau d'oxydation ACTIVE, indépendant de la pression</t>
+        </is>
+      </c>
+      <c r="I45" s="27" t="inlineStr">
+        <is>
+          <t>SiC + O2 → SiO(g) + CO : un SiC gazéifié par O2 consommé</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>Tout l'oxygène de l'air part en SiO et CO, la paroi reste du SiC nu. Chaque O2 (2 atomes d'oxygène) emporte un motif SiC : la masse ablatée par unité de masse d'air vaut y_O · M_SiC / (2·M_O).</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="35" t="inlineStr">
+        <is>
+          <t>B'c attendu sur le plateau</t>
+        </is>
+      </c>
+      <c r="C47" s="71">
+        <f>C21*$C$27/(2*Constantes!$C$9)</f>
+        <v>0.2918571303790834</v>
+      </c>
+      <c r="I47" s="12" t="inlineStr">
+        <is>
+          <t>table : 0.2920 à 1 atm entre 1975 et 2200 K ; 0.2919 à 0.001 atm, 1600 K</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="20" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="B48" s="20" t="inlineStr">
+        <is>
+          <t>Contrôle 2 — oxydation PASSIVE à basse température</t>
+        </is>
+      </c>
+      <c r="I48" s="27" t="inlineStr">
+        <is>
+          <t>SiC + O2 → SiO2(s) + C(gr) : la paroi fixe l'oxygène</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="30" customHeight="1">
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Le gaz à la paroi est de l'azote pur : Y_w,N = 1, donc B'c = Y_e,N − 1 &lt; 0 (prise de masse), écrêté à 0. C'est la couche de silice protectrice qui fait l'intérêt du SiC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="35" t="inlineStr">
+        <is>
+          <t>B'c brut (avant écrêtage) à 300 K</t>
+        </is>
+      </c>
+      <c r="C50" s="46">
+        <f>C22/1-1</f>
+        <v>-0.23290921795842312</v>
+      </c>
+      <c r="I50" s="12" t="inlineStr">
+        <is>
+          <t>prise de masse = masse d'oxygène fixée</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="20" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="B51" s="20" t="inlineStr">
+        <is>
+          <t>Contrôle 3 — pourquoi PAS -char-elem Si : comparaison sur trois points calculés</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>Point (T_w, P)</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>phases à la paroi</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>B'c suivi N</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
+        <is>
+          <t>B'c suivi Si</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="inlineStr">
+        <is>
+          <t>B'c suivi C</t>
+        </is>
+      </c>
+      <c r="G52" s="6" t="inlineStr"/>
+      <c r="H52" s="6" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>2100 K, 1 atm</t>
+        </is>
+      </c>
+      <c r="C53" s="72" t="inlineStr">
+        <is>
+          <t>SiC</t>
+        </is>
+      </c>
+      <c r="D53" s="21" t="n">
+        <v>0.292</v>
+      </c>
+      <c r="E53" s="21" t="n">
+        <v>0.292</v>
+      </c>
+      <c r="F53" s="21" t="n">
+        <v>0.292</v>
+      </c>
+      <c r="G53" s="15" t="inlineStr"/>
+      <c r="H53" s="15" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>2600 K, 1 atm</t>
+        </is>
+      </c>
+      <c r="C54" s="72" t="inlineStr">
+        <is>
+          <t>SiC + Si(L)</t>
+        </is>
+      </c>
+      <c r="D54" s="21" t="n">
+        <v>0.2583</v>
+      </c>
+      <c r="E54" s="21" t="n">
+        <v>0.1506</v>
+      </c>
+      <c r="F54" s="21" t="n">
+        <v>0.6108</v>
+      </c>
+      <c r="G54" s="15" t="inlineStr"/>
+      <c r="H54" s="15" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>2500 K, 0.001 atm</t>
+        </is>
+      </c>
+      <c r="C55" s="72" t="inlineStr">
+        <is>
+          <t>C(gr) (résidu)</t>
+        </is>
+      </c>
+      <c r="D55" s="21" t="n">
+        <v>185.4</v>
+      </c>
+      <c r="E55" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" s="21" t="n">
+        <v>4.312</v>
+      </c>
+      <c r="G55" s="15" t="inlineStr"/>
+      <c r="H55" s="15" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="B56" s="12" t="inlineStr">
+        <is>
+          <t>Les trois suivis coïncident tant que le SiC est la seule phase condensée. Dès qu'un autre solide reste à la paroi, un suivi sur un seul élément du char suppose à tort que l'autre part avec lui dans le rapport 1:1 : avec Si liquide résiduel, le suivi sur Si sous-estime (0.15) et le suivi sur C surestime (0.61) ; avec un résidu de carbone, le suivi sur Si tombe à 0 alors que le SiC se décompose. Le suivi sur N donne la masse réellement injectée dans la couche limite, celle qu'attend le bilan d'énergie de surface.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="18" customHeight="1">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>§6 — SENSIBILITÉ — régimes physiques (à 1 atm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>Régime</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>T_w [K]</t>
+        </is>
+      </c>
+      <c r="D59" s="6" t="inlineStr">
+        <is>
+          <t>Phases condensées</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="inlineStr">
+        <is>
+          <t>Espèces gazeuses dominantes</t>
+        </is>
+      </c>
+      <c r="F59" s="6" t="inlineStr">
+        <is>
+          <t>Mécanisme</t>
+        </is>
+      </c>
+      <c r="G59" s="6" t="inlineStr"/>
+      <c r="H59" s="6" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>oxydation passive</t>
+        </is>
+      </c>
+      <c r="C60" s="72" t="inlineStr">
+        <is>
+          <t>300 – 1625</t>
+        </is>
+      </c>
+      <c r="D60" s="72" t="inlineStr">
+        <is>
+          <t>SiC + SiO2 + C(gr)</t>
+        </is>
+      </c>
+      <c r="E60" s="72" t="inlineStr">
+        <is>
+          <t>N2</t>
+        </is>
+      </c>
+      <c r="F60" s="11" t="inlineStr">
+        <is>
+          <t>SiC + O2 → SiO2 + C ; B'c = 0</t>
+        </is>
+      </c>
+      <c r="G60" s="15" t="inlineStr"/>
+      <c r="H60" s="15" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>transition passive → active</t>
+        </is>
+      </c>
+      <c r="C61" s="72" t="inlineStr">
+        <is>
+          <t>1650 – 1950</t>
+        </is>
+      </c>
+      <c r="D61" s="72" t="inlineStr">
+        <is>
+          <t>SiC + SiO2</t>
+        </is>
+      </c>
+      <c r="E61" s="72" t="inlineStr">
+        <is>
+          <t>N2, CO, SiO</t>
+        </is>
+      </c>
+      <c r="F61" s="11" t="inlineStr">
+        <is>
+          <t>SiC + 2 SiO2 → 3 SiO + CO ; B'c 0 → 0.17</t>
+        </is>
+      </c>
+      <c r="G61" s="15" t="inlineStr"/>
+      <c r="H61" s="15" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>oxydation active</t>
+        </is>
+      </c>
+      <c r="C62" s="72" t="inlineStr">
+        <is>
+          <t>1975 – 2200</t>
+        </is>
+      </c>
+      <c r="D62" s="72" t="inlineStr">
+        <is>
+          <t>SiC</t>
+        </is>
+      </c>
+      <c r="E62" s="72" t="inlineStr">
+        <is>
+          <t>N2, CO, SiO</t>
+        </is>
+      </c>
+      <c r="F62" s="11" t="inlineStr">
+        <is>
+          <t>SiC + O2 → SiO + CO ; B'c = 0.292</t>
+        </is>
+      </c>
+      <c r="G62" s="15" t="inlineStr"/>
+      <c r="H62" s="15" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>oxydation + silicium liquide</t>
+        </is>
+      </c>
+      <c r="C63" s="72" t="inlineStr">
+        <is>
+          <t>2225 – 3000</t>
+        </is>
+      </c>
+      <c r="D63" s="72" t="inlineStr">
+        <is>
+          <t>SiC + Si(L)</t>
+        </is>
+      </c>
+      <c r="E63" s="72" t="inlineStr">
+        <is>
+          <t>N2, CO, SiO, Si, Si2C</t>
+        </is>
+      </c>
+      <c r="F63" s="11" t="inlineStr">
+        <is>
+          <t>SiC + O → Si(L) + CO ; B'c 0.29 → 1.7</t>
+        </is>
+      </c>
+      <c r="G63" s="15" t="inlineStr"/>
+      <c r="H63" s="15" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>sublimation</t>
+        </is>
+      </c>
+      <c r="C64" s="72" t="inlineStr">
+        <is>
+          <t>3025 – 3100</t>
+        </is>
+      </c>
+      <c r="D64" s="72" t="inlineStr">
+        <is>
+          <t>SiC</t>
+        </is>
+      </c>
+      <c r="E64" s="72" t="inlineStr">
+        <is>
+          <t>SiC2, Si2C, Si</t>
+        </is>
+      </c>
+      <c r="F64" s="11" t="inlineStr">
+        <is>
+          <t>SiC ⇌ Si + SiC2 + Si2C ; B'c 2.3 → 13.5</t>
+        </is>
+      </c>
+      <c r="G64" s="15" t="inlineStr"/>
+      <c r="H64" s="15" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>sublimation totale</t>
+        </is>
+      </c>
+      <c r="C65" s="72" t="inlineStr">
+        <is>
+          <t>≥ 3125</t>
+        </is>
+      </c>
+      <c r="D65" s="72" t="inlineStr">
+        <is>
+          <t>gaz seul</t>
+        </is>
+      </c>
+      <c r="E65" s="72" t="inlineStr">
+        <is>
+          <t>Si, SiC2, Si2C</t>
+        </is>
+      </c>
+      <c r="F65" s="11" t="inlineStr">
+        <is>
+          <t>plus de phase condensée : B'c = 200 (plafond)</t>
+        </is>
+      </c>
+      <c r="G65" s="15" t="inlineStr"/>
+      <c r="H65" s="15" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="B66" s="12" t="inlineStr">
+        <is>
+          <t>La pression décale TOUTES les transitions : à 0.001 atm l'oxydation devient active dès 1500 K et le SiC se décompose en laissant un résidu de carbone dès 2350 K ; à 1000 atm la silice (liquide) protège jusqu'à ~2700 K. Assemblage retenu en chaque point : sic_bprime/sic_bprime_phases.csv.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="18" customHeight="1">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>§7 — RÉPONSE MATÉRIAU (n'entre PAS dans le XML)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="35" t="inlineStr">
+        <is>
+          <t>couplage k = B'g / B'c</t>
+        </is>
+      </c>
+      <c r="C69" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="I69" s="12" t="inlineStr">
+        <is>
+          <t>pas de pyrolyse interne — comme le graphite et la silice</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="35" t="inlineStr">
+        <is>
+          <t>récession par unité de flux sur le plateau actif, B'c/ρ [m³/kg]</t>
+        </is>
+      </c>
+      <c r="C70" s="41">
+        <f>C21*$C$27/(2*Constantes!$C$9)/C23</f>
+        <v>9.092122441715994e-05</v>
+      </c>
+      <c r="I70" s="12" t="inlineStr">
+        <is>
+          <t>ṡ = B'c·ṁe/ρ — valable tant que la paroi reste du SiC nu</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="12" t="inlineStr">
+        <is>
+          <t>Hors du régime actif la paroi porte un autre solide (SiO2, Si liquide, carbone) : B'c reste la masse gazéifiée, mais la récession du SiC n'en découle plus directement — le solide résiduel s'accumule, coule ou s'écaille, ce que le modèle d'équilibre ne décrit pas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="18" customHeight="1">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>§8 — BLOC XML</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" s="29" t="inlineStr">
+        <is>
+          <t>&lt;mixture thermo_db="NASA-9"&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    &lt;species&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        N O NO N2 O2</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        C C2 C3 CN CO CO2</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        Si Si2 Si3 SiO SiO2 SiN Si2N SiC SiC2 Si2C</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        C(gr) Si(cr) Si(L) SiC(b) SiC(L)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        SiO2(a-qz) SiO2(b-qz) SiO2(b-crt) SiO2(L)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    &lt;/species&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    &lt;element_compositions default="air"&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="B83" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        &lt;composition name="air"&gt;N:0.79, O:0.21&lt;/composition&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="B84" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        &lt;composition name="sic"&gt;Si:1.0, C:1.0&lt;/composition&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="B85" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    &lt;/element_compositions&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="B86" s="29" t="inlineStr">
+        <is>
+          <t>&lt;/mixture&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="16" customHeight="1">
+      <c r="B88" s="5" t="inlineStr">
+        <is>
+          <t>bprime -T &lt;Tw&gt; -P &lt;P&gt; -b 0.0 -m sic-air -bl air -char sic -char-elem N   (point par point, cf. sic_bprime.py)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="45">
+    <mergeCell ref="B85:I85"/>
+    <mergeCell ref="A25:I25"/>
+    <mergeCell ref="B75:I75"/>
+    <mergeCell ref="B81:I81"/>
+    <mergeCell ref="A18:I18"/>
+    <mergeCell ref="B66:I66"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="B15:H15"/>
+    <mergeCell ref="B46:I46"/>
+    <mergeCell ref="A12:I12"/>
+    <mergeCell ref="B51:H51"/>
+    <mergeCell ref="B71:I71"/>
+    <mergeCell ref="B45:H45"/>
+    <mergeCell ref="B56:I56"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="B26:H26"/>
+    <mergeCell ref="B86:I86"/>
+    <mergeCell ref="B77:I77"/>
+    <mergeCell ref="A5:I5"/>
+    <mergeCell ref="B16:H16"/>
+    <mergeCell ref="B88:I88"/>
+    <mergeCell ref="B82:I82"/>
+    <mergeCell ref="A68:I68"/>
+    <mergeCell ref="B78:I78"/>
+    <mergeCell ref="A44:I44"/>
+    <mergeCell ref="B48:H48"/>
+    <mergeCell ref="B37:I37"/>
+    <mergeCell ref="A58:I58"/>
+    <mergeCell ref="A39:I39"/>
+    <mergeCell ref="B49:I49"/>
+    <mergeCell ref="B84:I84"/>
+    <mergeCell ref="B74:I74"/>
+    <mergeCell ref="B14:H14"/>
+    <mergeCell ref="A73:I73"/>
+    <mergeCell ref="B83:I83"/>
+    <mergeCell ref="B13:H13"/>
+    <mergeCell ref="B33:I33"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="B36:I36"/>
+    <mergeCell ref="B80:I80"/>
+    <mergeCell ref="B76:I76"/>
+    <mergeCell ref="B79:I79"/>
+    <mergeCell ref="B34:H34"/>
+    <mergeCell ref="B35:I35"/>
+    <mergeCell ref="B28:H28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Ajoute les tables B' du molybdène (Mo, TZM) et l'onglet correspondant
- data/mixtures/mo-air.xml : Mo-N-O, oxydes gazeux jusqu'à Mo5O15,
  phases condensées Mo(cr,L), MoO2(cr), MoO3(cr,L).
- mo_bprime.py : deux tables au format des autres matériaux.
  Équilibre complet (borne basse : MoO2 solide fixe l'oxygène, B'c = 0
  jusqu'à ~2350 K à 1 atm) et surface nue sans oxydes condensés (borne
  haute : limite de diffusion Mo + 3/2 O2 -> MoO3, B'c = 0.466).
  Suivi sur N ; les 4725 points d'équilibre sont stables.
- README : choix des deux tables, table à retenir par plage de Tw, limites.
- Classeur : onglet Molybdène, ligne de synthèse, contrôle dans
  verification_xlsx.py (644 formules, 0 erreur).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TcAV8aPzoBRqLK16FKxnci
</commit_message>
<xml_diff>
--- a/mise_en_donnees_xlsx/mise_en_donnees_materiaux.xlsx
+++ b/mise_en_donnees_xlsx/mise_en_donnees_materiaux.xlsx
@@ -18,6 +18,7 @@
     <sheet name="Carbone" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Silice" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="SiC" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Molybdène" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,7 +27,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="9">
+  <numFmts count="10">
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="0.00000"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
@@ -36,6 +37,7 @@
     <numFmt numFmtId="170" formatCode="0.000000"/>
     <numFmt numFmtId="171" formatCode="0.00000000"/>
     <numFmt numFmtId="172" formatCode="0.0000000"/>
+    <numFmt numFmtId="173" formatCode="0.###"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -179,7 +181,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -281,6 +283,10 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="7" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="173" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -647,7 +653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:I56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4.5" customWidth="1" min="1" max="1"/>
@@ -678,7 +684,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Fichier(s) XML : data/mixtures/ — 10 matériaux, 18 fichiers de mélange</t>
+          <t>Fichier(s) XML : data/mixtures/ — 11 matériaux, 19 fichiers de mélange</t>
         </is>
       </c>
     </row>
@@ -1055,97 +1061,106 @@
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="12" t="inlineStr">
-        <is>
-          <t>Les colonnes « gaz » sont des liens vers la ligne « valeur portée dans le XML » de chaque onglet. Le graphite, la silice et le SiC n'ont pas de gaz de pyrolyse (k = 0). TACOT et CPh70 portent RIGOUREUSEMENT la même composition : leurs fichiers XML sont identiques, seul k les distingue — c'est la démonstration de l'onglet CPh70.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Molybdène (TZM)</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G21" s="10" t="inlineStr">
+        <is>
+          <t>Mo:1.0</t>
+        </is>
+      </c>
+      <c r="H21" s="8">
+        <f>'Molybdène'!C53</f>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>Les colonnes « gaz » sont des liens vers la ligne « valeur portée dans le XML » de chaque onglet. Le graphite, la silice, le SiC et le molybdène n'ont pas de gaz de pyrolyse (k = 0). TACOT et CPh70 portent RIGOUREUSEMENT la même composition : leurs fichiers XML sont identiques, seul k les distingue — c'est la démonstration de l'onglet CPh70.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>§3 — LES TROIS SEULES DONNÉES QUE CONSOMME LE CALCUL</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="6" t="inlineStr">
+    <row r="25">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>Composition</t>
         </is>
       </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>Rôle dans le bilan</t>
         </is>
       </c>
-      <c r="E24" s="6" t="inlineStr">
+      <c r="E25" s="6" t="inlineStr">
         <is>
           <t>Option</t>
         </is>
       </c>
-      <c r="F24" s="6" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr">
         <is>
           <t>Comment on l'obtient</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr"/>
-      <c r="H24" s="6" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>bord de couche limite</t>
-        </is>
-      </c>
-      <c r="D25" s="7" t="inlineStr">
-        <is>
-          <t>Y_e</t>
-        </is>
-      </c>
-      <c r="E25" s="14" t="inlineStr">
-        <is>
-          <t>-bl</t>
-        </is>
-      </c>
-      <c r="F25" s="11" t="inlineStr">
-        <is>
-          <t>l'atmosphère : air N:0.79 O:0.21 · Mars · Titan…</t>
-        </is>
-      </c>
-      <c r="G25" s="15" t="inlineStr"/>
-      <c r="H25" s="15" t="inlineStr"/>
+      <c r="G25" s="6" t="inlineStr"/>
+      <c r="H25" s="6" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="B26" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>gaz de pyrolyse</t>
+          <t>bord de couche limite</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>Y_g</t>
+          <t>Y_e</t>
         </is>
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
-          <t>-py</t>
+          <t>-bl</t>
         </is>
       </c>
       <c r="F26" s="11" t="inlineStr">
         <is>
-          <t>c'est TOUT l'objet de ce classeur — quatre routes possibles, §4</t>
+          <t>l'atmosphère : air N:0.79 O:0.21 · Mars · Titan…</t>
         </is>
       </c>
       <c r="G26" s="15" t="inlineStr"/>
@@ -1153,127 +1168,125 @@
     </row>
     <row r="27">
       <c r="B27" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>char</t>
+          <t>gaz de pyrolyse</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>Y_c</t>
+          <t>Y_g</t>
         </is>
       </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
-          <t>-char + -char-elem</t>
+          <t>-py</t>
         </is>
       </c>
       <c r="F27" s="11" t="inlineStr">
         <is>
-          <t>C:1.0 si tous les constituants carbonisent vers le carbone ; sinon pondérer par les masses de char</t>
+          <t>c'est TOUT l'objet de ce classeur — quatre routes possibles, §4</t>
         </is>
       </c>
       <c r="G27" s="15" t="inlineStr"/>
       <c r="H27" s="15" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="B28" s="12" t="inlineStr">
+      <c r="B28" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>char</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>Y_c</t>
+        </is>
+      </c>
+      <c r="E28" s="14" t="inlineStr">
+        <is>
+          <t>-char + -char-elem</t>
+        </is>
+      </c>
+      <c r="F28" s="11" t="inlineStr">
+        <is>
+          <t>C:1.0 si tous les constituants carbonisent vers le carbone ; sinon pondérer par les masses de char</t>
+        </is>
+      </c>
+      <c r="G28" s="15" t="inlineStr"/>
+      <c r="H28" s="15" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="B29" s="12" t="inlineStr">
         <is>
           <t>Plus T, P et B'g. Rien d'autre : cf. src/apps/bprime.cpp:304-330. Sans -char/-char-elem, bprime utilise un char de carbone pur intégré ; les deux options vont toujours ensemble.</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="4" t="inlineStr">
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>§4 — LES QUATRE ROUTES DE CALCUL DU GAZ DE PYROLYSE</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="B31" s="6" t="inlineStr">
+    <row r="32">
+      <c r="B32" s="6" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="C31" s="6" t="inlineStr">
+      <c r="C32" s="6" t="inlineStr">
         <is>
           <t>Matériau</t>
         </is>
       </c>
-      <c r="D31" s="6" t="inlineStr">
+      <c r="D32" s="6" t="inlineStr">
         <is>
           <t>Donnée primaire</t>
         </is>
       </c>
-      <c r="E31" s="6" t="inlineStr">
+      <c r="E32" s="6" t="inlineStr">
         <is>
           <t>Passage à l'élémentaire</t>
         </is>
       </c>
-      <c r="F31" s="6" t="inlineStr">
+      <c r="F32" s="6" t="inlineStr">
         <is>
           <t>Point critique</t>
         </is>
       </c>
-      <c r="G31" s="6" t="inlineStr"/>
-      <c r="H31" s="6" t="inlineStr"/>
-    </row>
-    <row r="32" ht="28" customHeight="1">
-      <c r="B32" s="16" t="inlineStr">
-        <is>
-          <t>A — sommation atomique</t>
-        </is>
-      </c>
-      <c r="C32" s="17" t="inlineStr">
-        <is>
-          <t>TACOT, CPh70</t>
-        </is>
-      </c>
-      <c r="D32" s="17" t="inlineStr">
-        <is>
-          <t>spéciation moléculaire mesurée (7 espèces)</t>
-        </is>
-      </c>
-      <c r="E32" s="18" t="inlineStr">
-        <is>
-          <t>n_E = Σ_j ν_E,j · x_j</t>
-        </is>
-      </c>
-      <c r="F32" s="19" t="inlineStr">
-        <is>
-          <t>la renormalisation : somme réelle des colonnes (100.30), pas les totaux imprimés (100.0)</t>
-        </is>
-      </c>
-      <c r="G32" s="15" t="inlineStr"/>
-      <c r="H32" s="15" t="inlineStr"/>
+      <c r="G32" s="6" t="inlineStr"/>
+      <c r="H32" s="6" t="inlineStr"/>
     </row>
     <row r="33" ht="28" customHeight="1">
       <c r="B33" s="16" t="inlineStr">
         <is>
-          <t>B — conversion directe</t>
+          <t>A — sommation atomique</t>
         </is>
       </c>
       <c r="C33" s="17" t="inlineStr">
         <is>
-          <t>ZURAM</t>
+          <t>TACOT, CPh70</t>
         </is>
       </c>
       <c r="D33" s="17" t="inlineStr">
         <is>
-          <t>composition élémentaire MASSIQUE mesurée</t>
+          <t>spéciation moléculaire mesurée (7 espèces)</t>
         </is>
       </c>
       <c r="E33" s="18" t="inlineStr">
         <is>
-          <t>x_E = (y_E/M_E) / Σ (y_j/M_j)</t>
+          <t>n_E = Σ_j ν_E,j · x_j</t>
         </is>
       </c>
       <c r="F33" s="19" t="inlineStr">
         <is>
-          <t>traçabilité limitée à 3 décimales ; la source primaire VKI n'est pas publique</t>
+          <t>la renormalisation : somme réelle des colonnes (100.30), pas les totaux imprimés (100.0)</t>
         </is>
       </c>
       <c r="G33" s="15" t="inlineStr"/>
@@ -1282,27 +1295,27 @@
     <row r="34" ht="28" customHeight="1">
       <c r="B34" s="16" t="inlineStr">
         <is>
-          <t>C — fermeture élémentaire</t>
+          <t>B — conversion directe</t>
         </is>
       </c>
       <c r="C34" s="17" t="inlineStr">
         <is>
-          <t>SC-1008</t>
+          <t>ZURAM</t>
         </is>
       </c>
       <c r="D34" s="17" t="inlineStr">
         <is>
-          <t>motif chimique idéalisé + rendement en char</t>
+          <t>composition élémentaire MASSIQUE mesurée</t>
         </is>
       </c>
       <c r="E34" s="18" t="inlineStr">
         <is>
-          <t>n_E(gaz) = n_E(résine) − n_E(char)</t>
+          <t>x_E = (y_E/M_E) / Σ (y_j/M_j)</t>
         </is>
       </c>
       <c r="F34" s="19" t="inlineStr">
         <is>
-          <t>le rendement en char entre DANS la chaîne : ±0.05 sur Y déplace le carbone de ~12 %</t>
+          <t>traçabilité limitée à 3 décimales ; la source primaire VKI n'est pas publique</t>
         </is>
       </c>
       <c r="G34" s="15" t="inlineStr"/>
@@ -1311,27 +1324,27 @@
     <row r="35" ht="28" customHeight="1">
       <c r="B35" s="16" t="inlineStr">
         <is>
-          <t>D — fermeture sur DEUX constituants</t>
+          <t>C — fermeture élémentaire</t>
         </is>
       </c>
       <c r="C35" s="17" t="inlineStr">
         <is>
-          <t>Liège/phénolique</t>
+          <t>SC-1008</t>
         </is>
       </c>
       <c r="D35" s="17" t="inlineStr">
         <is>
-          <t>analyses des deux constituants + rendements</t>
+          <t>motif chimique idéalisé + rendement en char</t>
         </is>
       </c>
       <c r="E35" s="18" t="inlineStr">
         <is>
-          <t>n_E(gaz) = Σ_i [n_E(i) − n_E(char,i)]</t>
+          <t>n_E(gaz) = n_E(résine) − n_E(char)</t>
         </is>
       </c>
       <c r="F35" s="19" t="inlineStr">
         <is>
-          <t>le renfort pyrolyse : le rapport renfort/résine entre dans la table B'</t>
+          <t>le rendement en char entre DANS la chaîne : ±0.05 sur Y déplace le carbone de ~12 %</t>
         </is>
       </c>
       <c r="G35" s="15" t="inlineStr"/>
@@ -1340,85 +1353,93 @@
     <row r="36" ht="28" customHeight="1">
       <c r="B36" s="16" t="inlineStr">
         <is>
-          <t>E — stœchiométrie directe</t>
+          <t>D — fermeture sur DEUX constituants</t>
         </is>
       </c>
       <c r="C36" s="17" t="inlineStr">
         <is>
-          <t>Carbone, Silice, SiC</t>
+          <t>Liège/phénolique</t>
         </is>
       </c>
       <c r="D36" s="17" t="inlineStr">
         <is>
-          <t>la formule du solide</t>
+          <t>analyses des deux constituants + rendements</t>
         </is>
       </c>
       <c r="E36" s="18" t="inlineStr">
         <is>
-          <t>aucun gaz de pyrolyse (B'g = 0)</t>
+          <t>n_E(gaz) = Σ_i [n_E(i) − n_E(char,i)]</t>
         </is>
       </c>
       <c r="F36" s="19" t="inlineStr">
         <is>
-          <t>le char EST le matériau ; -char-elem Si pour la silice, N pour le SiC (char non congruent)</t>
+          <t>le renfort pyrolyse : le rapport renfort/résine entre dans la table B'</t>
         </is>
       </c>
       <c r="G36" s="15" t="inlineStr"/>
       <c r="H36" s="15" t="inlineStr"/>
     </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="4" t="inlineStr">
+    <row r="37" ht="28" customHeight="1">
+      <c r="B37" s="16" t="inlineStr">
+        <is>
+          <t>E — stœchiométrie directe</t>
+        </is>
+      </c>
+      <c r="C37" s="17" t="inlineStr">
+        <is>
+          <t>Carbone, Silice, SiC, Mo</t>
+        </is>
+      </c>
+      <c r="D37" s="17" t="inlineStr">
+        <is>
+          <t>la formule du solide</t>
+        </is>
+      </c>
+      <c r="E37" s="18" t="inlineStr">
+        <is>
+          <t>aucun gaz de pyrolyse (B'g = 0)</t>
+        </is>
+      </c>
+      <c r="F37" s="19" t="inlineStr">
+        <is>
+          <t>le char EST le matériau ; -char-elem Si pour la silice, N pour le SiC (char non congruent)</t>
+        </is>
+      </c>
+      <c r="G37" s="15" t="inlineStr"/>
+      <c r="H37" s="15" t="inlineStr"/>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="4" t="inlineStr">
         <is>
           <t>§5 — CE QUI N'ENTRE PAS DANS LE XML</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="B39" s="6" t="inlineStr">
+    <row r="40">
+      <c r="B40" s="6" t="inlineStr">
         <is>
           <t>Donnée</t>
         </is>
       </c>
-      <c r="C39" s="6" t="inlineStr">
+      <c r="C40" s="6" t="inlineStr">
         <is>
           <t>Dans le XML ?</t>
         </is>
       </c>
-      <c r="D39" s="6" t="inlineStr">
+      <c r="D40" s="6" t="inlineStr">
         <is>
           <t>Où elle sert vraiment</t>
         </is>
       </c>
-      <c r="E39" s="6" t="inlineStr"/>
-      <c r="F39" s="6" t="inlineStr"/>
-      <c r="G39" s="6" t="inlineStr"/>
-      <c r="H39" s="6" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="B40" s="7" t="inlineStr">
-        <is>
-          <t>masse volumique ρ_v, ρ_c</t>
-        </is>
-      </c>
-      <c r="C40" s="13" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="D40" s="11" t="inlineStr">
-        <is>
-          <t>solveur de réponse matériau ; récession ṡ = B'c·ṁe/ρ_c</t>
-        </is>
-      </c>
-      <c r="E40" s="15" t="inlineStr"/>
-      <c r="F40" s="15" t="inlineStr"/>
-      <c r="G40" s="15" t="inlineStr"/>
-      <c r="H40" s="15" t="inlineStr"/>
+      <c r="E40" s="6" t="inlineStr"/>
+      <c r="F40" s="6" t="inlineStr"/>
+      <c r="G40" s="6" t="inlineStr"/>
+      <c r="H40" s="6" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>porosité</t>
+          <t>masse volumique ρ_v, ρ_c</t>
         </is>
       </c>
       <c r="C41" s="13" t="inlineStr">
@@ -1428,7 +1449,7 @@
       </c>
       <c r="D41" s="11" t="inlineStr">
         <is>
-          <t>conduction, perméabilité</t>
+          <t>solveur de réponse matériau ; récession ṡ = B'c·ṁe/ρ_c</t>
         </is>
       </c>
       <c r="E41" s="15" t="inlineStr"/>
@@ -1439,17 +1460,17 @@
     <row r="42">
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>rapport fibres/résine</t>
+          <t>porosité</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
         <is>
-          <t>non *</t>
+          <t>non</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>fixe la QUANTITÉ de gaz (donc B'g), pas sa composition</t>
+          <t>conduction, perméabilité</t>
         </is>
       </c>
       <c r="E42" s="15" t="inlineStr"/>
@@ -1460,7 +1481,7 @@
     <row r="43">
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>rendement en char</t>
+          <t>rapport fibres/résine</t>
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr">
@@ -1470,7 +1491,7 @@
       </c>
       <c r="D43" s="11" t="inlineStr">
         <is>
-          <t>idem — mais il entre dans le CALCUL du gaz pour les routes C et D</t>
+          <t>fixe la QUANTITÉ de gaz (donc B'g), pas sa composition</t>
         </is>
       </c>
       <c r="E43" s="15" t="inlineStr"/>
@@ -1481,17 +1502,17 @@
     <row r="44">
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>cinétique de pyrolyse</t>
+          <t>rendement en char</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
-          <t>non</t>
+          <t>non *</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>fixe B'g au cours du temps</t>
+          <t>idem — mais il entre dans le CALCUL du gaz pour les routes C et D</t>
         </is>
       </c>
       <c r="E44" s="15" t="inlineStr"/>
@@ -1500,109 +1521,130 @@
       <c r="H44" s="15" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="B45" s="12" t="inlineStr">
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>cinétique de pyrolyse</t>
+        </is>
+      </c>
+      <c r="C45" s="13" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="D45" s="11" t="inlineStr">
+        <is>
+          <t>fixe B'g au cours du temps</t>
+        </is>
+      </c>
+      <c r="E45" s="15" t="inlineStr"/>
+      <c r="F45" s="15" t="inlineStr"/>
+      <c r="G45" s="15" t="inlineStr"/>
+      <c r="H45" s="15" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="B46" s="12" t="inlineStr">
         <is>
           <t>* sauf si les constituants donnent des chars de compositions élémentaires DIFFÉRENTES (fibres de silice + résine phénolique), ou si le renfort pyrolyse (liège) : le rapport entre alors dans Y_c et/ou Y_g, et la table change. Le bilan de masse de surface est écrit sur des fractions massiques élémentaires, donc normalisées : les grandeurs VOLUMIQUES n'y ont structurellement aucune place.</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="4" t="inlineStr">
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="4" t="inlineStr">
         <is>
           <t>§6 — RECETTE POUR UN NOUVEAU MATÉRIAU</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="B48" s="5" t="inlineStr">
-        <is>
-          <t>Atmosphère → composition -bl (air, Mars, Titan…).</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>Résine → composition du gaz de pyrolyse par l'une des quatre routes du §4 → composition -py.</t>
+          <t>Atmosphère → composition -bl (air, Mars, Titan…).</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>Char → C:1.0 si tous les constituants carbonisent vers le carbone ; sinon pondérer par les masses de char de chaque constituant.</t>
+          <t>Résine → composition du gaz de pyrolyse par l'une des quatre routes du §4 → composition -py.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>Espèces → tous les produits attendus des éléments présents, PLUS la ou les phases condensées.</t>
+          <t>Char → C:1.0 si tous les constituants carbonisent vers le carbone ; sinon pondérer par les masses de char de chaque constituant.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>Vérifier : checkmix (noms, phases), puis un run court.</t>
+          <t>Espèces → tous les produits attendus des éléments présents, PLUS la ou les phases condensées.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>Vérifier : checkmix (noms, phases), puis un run court.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="B53" s="5" t="inlineStr">
+      <c r="B54" s="5" t="inlineStr">
         <is>
           <t>Contrôler la physique : à 300 K et B'g = 0 dans l'air, un char carboné doit donner B'c ≈ 0.0874 (limite C + O2 → CO2, indépendante de la pression). Une valeur ≈ 200 signale l'absence de C(gr). Pour un char multi-élément susceptible de laisser un autre solide à la paroi (SiC), suivre le bilan sur N (-char-elem N).</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="30" customHeight="1">
-      <c r="B55" s="5" t="inlineStr">
-        <is>
-          <t>Documents de référence du dépôt : tacot_bprime/mise_en_donnees_xml.md (mécanique du fichier XML et règles du parseur) · resine_tacot.md · zuram_bprime/resine_zuram.md · sc1008_bprime/resine_sc1008.md · cork_bprime/mise_en_donnees_cork.md · tacot_bprime/cph70_vs_tacot.md · carbon_bprime/bprime_carbon_physique.md · sic_bprime/README.md.</t>
+    <row r="56" ht="30" customHeight="1">
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Documents de référence du dépôt : tacot_bprime/mise_en_donnees_xml.md (mécanique du fichier XML et règles du parseur) · resine_tacot.md · zuram_bprime/resine_zuram.md · sc1008_bprime/resine_sc1008.md · cork_bprime/mise_en_donnees_cork.md · tacot_bprime/cph70_vs_tacot.md · carbon_bprime/bprime_carbon_physique.md · sic_bprime/README.md · mo_bprime/README.md.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="22">
     <mergeCell ref="B7:I7"/>
+    <mergeCell ref="B54:I54"/>
+    <mergeCell ref="B22:I22"/>
     <mergeCell ref="A3:I3"/>
+    <mergeCell ref="B46:I46"/>
+    <mergeCell ref="B56:I56"/>
     <mergeCell ref="B52:I52"/>
-    <mergeCell ref="B21:I21"/>
     <mergeCell ref="A2:I2"/>
-    <mergeCell ref="B48:I48"/>
-    <mergeCell ref="A47:I47"/>
     <mergeCell ref="A5:I5"/>
-    <mergeCell ref="A23:I23"/>
     <mergeCell ref="B8:I8"/>
-    <mergeCell ref="A38:I38"/>
     <mergeCell ref="B53:I53"/>
+    <mergeCell ref="B29:I29"/>
     <mergeCell ref="A10:I10"/>
-    <mergeCell ref="B28:I28"/>
+    <mergeCell ref="A31:I31"/>
+    <mergeCell ref="A39:I39"/>
+    <mergeCell ref="A48:I48"/>
     <mergeCell ref="B49:I49"/>
-    <mergeCell ref="A30:I30"/>
-    <mergeCell ref="B55:I55"/>
+    <mergeCell ref="A24:I24"/>
     <mergeCell ref="B6:I6"/>
     <mergeCell ref="B51:I51"/>
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="B45:I45"/>
     <mergeCell ref="B50:I50"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3447,6 +3489,775 @@
     <mergeCell ref="B34:H34"/>
     <mergeCell ref="B35:I35"/>
     <mergeCell ref="B28:H28"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00C55A11"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I70"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4.5" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="72" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Molybdène Mo (TZM) — métal à oxyde VOLATIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Char monoélément dont l'oxyde MoO3 s'évapore : deux tables encadrent la réalité, équilibre complet (borne basse) et surface nue (borne haute)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Fichier(s) XML : data/mixtures/mo-air.xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>§0 — FICHE D'IDENTITÉ</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="35" t="inlineStr">
+        <is>
+          <t>Matériau</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="inlineStr">
+        <is>
+          <t>molybdène ; s'applique au TZM (Mo + 0.5 % Ti, 0.08 % Zr, ~0.02 % C)</t>
+        </is>
+      </c>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>mo_bprime/mo_bprime.py · mo_bprime/README.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="35" t="inlineStr">
+        <is>
+          <t>Système chimique</t>
+        </is>
+      </c>
+      <c r="C7" s="30" t="inlineStr">
+        <is>
+          <t>Mo-N-O : 5 espèces d'air + Mo, MoO, MoO2, MoO3 et polymères Mo2O6…Mo5O15 + 5 phases condensées</t>
+        </is>
+      </c>
+      <c r="I7" s="12" t="inlineStr">
+        <is>
+          <t>18 espèces au total</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="35" t="inlineStr">
+        <is>
+          <t>Phases condensées</t>
+        </is>
+      </c>
+      <c r="C8" s="30" t="inlineStr">
+        <is>
+          <t>Mo(cr), Mo(L) · MoO2(cr) · MoO3(cr), MoO3(L)</t>
+        </is>
+      </c>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>toutes présentes dans nasa9.dat</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="35" t="inlineStr">
+        <is>
+          <t>Binaire</t>
+        </is>
+      </c>
+      <c r="C9" s="30" t="inlineStr">
+        <is>
+          <t>bprime généralisé : -char mo -char-elem N</t>
+        </is>
+      </c>
+      <c r="I9" s="12" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="B10" s="35" t="inlineStr">
+        <is>
+          <t>Compositions du XML</t>
+        </is>
+      </c>
+      <c r="C10" s="30" t="inlineStr">
+        <is>
+          <t>air (-bl) · mo (char, -char)</t>
+        </is>
+      </c>
+      <c r="I10" s="12" t="inlineStr"/>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>§1 — HYPOTHÈSES</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="A13" s="20" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Le char est le métal pur, Mo:1.0 ; les additions du TZM sont ignorées.</t>
+        </is>
+      </c>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>Ti, Zr et C durcissent l'alliage mais ne changent pas son oxydation, et n'ont pas de données dans la base. Pas de pyrolyse : B'g = 0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="26" customHeight="1">
+      <c r="A14" s="20" t="inlineStr">
+        <is>
+          <t>H2</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Bilan suivi sur N, comme pour le SiC.</t>
+        </is>
+      </c>
+      <c r="I14" s="12" t="inlineStr">
+        <is>
+          <t>B'c = masse nette gazéifiée. Pour un char monoélément, identique au suivi sur Mo tant que seul le métal est condensé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>H3</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>L'équilibre complet est une BORNE BASSE.</t>
+        </is>
+      </c>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>Avec un excès de métal, l'oxygène est fixé en MoO2 solide et B'c = 0 jusqu'à ~2350 K à 1 atm. En réalité MoO3 se forme sur la face externe de l'oxyde, fond à 795 °C et s'évapore : le molybdène s'oxyde vite dès ~1000 K.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="26" customHeight="1">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>La table « surface nue » (sans oxydes condensés) est une BORNE HAUTE.</t>
+        </is>
+      </c>
+      <c r="I16" s="12" t="inlineStr">
+        <is>
+          <t>Tout l'oxygène qui atteint la paroi repart en oxydes gazeux : régime limité par la diffusion dans la couche limite. Conservative au-dessus de ~1000 K, fausse en dessous (cinétique lente).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>§2 — DONNÉES D'ENTRÉE</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="35" t="inlineStr">
+        <is>
+          <t>M_Mo [g/mol]</t>
+        </is>
+      </c>
+      <c r="C19" s="75" t="n">
+        <v>95.95999999999999</v>
+      </c>
+      <c r="I19" s="12" t="inlineStr">
+        <is>
+          <t>data/thermo/elements.xml (masse de Mutation++)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="35" t="inlineStr">
+        <is>
+          <t>fraction massique d'oxygène de l'air</t>
+        </is>
+      </c>
+      <c r="C20" s="50">
+        <f>Constantes!D19</f>
+        <v>0.23290921795842306</v>
+      </c>
+      <c r="I20" s="12" t="inlineStr">
+        <is>
+          <t>y_O calculé au §2 de l'onglet Constantes</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="35" t="inlineStr">
+        <is>
+          <t>masse volumique du TZM [kg/m³]</t>
+        </is>
+      </c>
+      <c r="C21" s="30" t="n">
+        <v>10220</v>
+      </c>
+      <c r="I21" s="12" t="inlineStr">
+        <is>
+          <t>Mo pur : 10 280 kg/m³ — n'entre que dans la récession</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>§3 — CALCUL PAS À PAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="20" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="B24" s="20" t="inlineStr">
+        <is>
+          <t>Étape 1 — composition élémentaire du char : directe</t>
+        </is>
+      </c>
+      <c r="I24" s="27" t="inlineStr">
+        <is>
+          <t>métal pur ⇒ x_Mo = y_Mo = 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="20" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="B25" s="20" t="inlineStr">
+        <is>
+          <t>Étape 2 — réaction limite du régime de diffusion</t>
+        </is>
+      </c>
+      <c r="I25" s="27" t="inlineStr">
+        <is>
+          <t>Mo + 3/2 O2 → MoO3(g)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Chaque molécule d'O2 qui atteint la paroi emporte 2/3 d'atome de molybdène. La masse de Mo gazéifiée par unité de masse d'air vaut donc y_O · M_Mo / (3·M_O), indépendamment de la pression.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="35" t="inlineStr">
+        <is>
+          <t>B'c limite de diffusion (MoO3)</t>
+        </is>
+      </c>
+      <c r="C27" s="71">
+        <f>C20*C19/(3*Constantes!$C$9)</f>
+        <v>0.46565344824239585</v>
+      </c>
+      <c r="I27" s="12" t="inlineStr">
+        <is>
+          <t>table « surface nue » : 0.4657 sur tout le plateau</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="35" t="inlineStr">
+        <is>
+          <t>B'c si l'oxyde gazeux était MoO2</t>
+        </is>
+      </c>
+      <c r="C28" s="71">
+        <f>C20*C19/(2*Constantes!$C$9)</f>
+        <v>0.6984801723635938</v>
+      </c>
+      <c r="I28" s="12" t="inlineStr">
+        <is>
+          <t>borne supérieure du plateau, approchée à haute T quand MoO2 et MoO remplacent MoO3</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>§4 — RÉSULTAT : CE QUI ENTRE DANS LE XML</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>Composition élémentaire</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>Mo</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr"/>
+      <c r="G31" s="6" t="inlineStr"/>
+      <c r="H31" s="6" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>mo — valeur portée dans le XML</t>
+        </is>
+      </c>
+      <c r="C32" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E32" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F32" s="15" t="inlineStr"/>
+      <c r="G32" s="15" t="inlineStr"/>
+      <c r="H32" s="15" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>air — valeur portée dans le XML</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D33" s="44" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="E33" s="44" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="F33" s="15" t="inlineStr"/>
+      <c r="G33" s="15" t="inlineStr"/>
+      <c r="H33" s="15" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>La variante « surface nue » n'est pas un fichier du dépôt : mo_bprime.py l'écrit à la volée en retirant MoO2(cr), MoO3(cr) et MoO3(L) de la liste d'espèces.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>§5 — CONTRÔLES ET VALIDATION CROISÉE</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="35" t="inlineStr">
+        <is>
+          <t>plateau de la table « surface nue »</t>
+        </is>
+      </c>
+      <c r="C37" s="76" t="n">
+        <v>0.4657</v>
+      </c>
+      <c r="I37" s="12" t="inlineStr">
+        <is>
+          <t>à comparer au calcul analytique du §3</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="35" t="inlineStr">
+        <is>
+          <t>écart relatif</t>
+        </is>
+      </c>
+      <c r="C38" s="67">
+        <f>ABS(C37-C27)/C27</f>
+        <v>9.99708211758358e-05</v>
+      </c>
+      <c r="I38" s="12" t="inlineStr">
+        <is>
+          <t>l'arrondi de la table</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="35" t="inlineStr">
+        <is>
+          <t>points instables (critère de force motrice)</t>
+        </is>
+      </c>
+      <c r="C39" s="77" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" s="12" t="inlineStr">
+        <is>
+          <t>table d'équilibre complet, 4725 points — contrôle du script SiC</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>§6 — SENSIBILITÉ — disparition des oxydes condensés (équilibre complet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>P [atm]</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>T_w [K]</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr"/>
+      <c r="E42" s="6" t="inlineStr"/>
+      <c r="F42" s="6" t="inlineStr"/>
+      <c r="G42" s="6" t="inlineStr"/>
+      <c r="H42" s="6" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="B43" s="78" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="C43" s="40" t="n">
+        <v>1875</v>
+      </c>
+      <c r="D43" s="15" t="inlineStr"/>
+      <c r="E43" s="15" t="inlineStr"/>
+      <c r="F43" s="15" t="inlineStr"/>
+      <c r="G43" s="15" t="inlineStr"/>
+      <c r="H43" s="15" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="B44" s="78" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C44" s="40" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D44" s="15" t="inlineStr"/>
+      <c r="E44" s="15" t="inlineStr"/>
+      <c r="F44" s="15" t="inlineStr"/>
+      <c r="G44" s="15" t="inlineStr"/>
+      <c r="H44" s="15" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="B45" s="78" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C45" s="40" t="n">
+        <v>2175</v>
+      </c>
+      <c r="D45" s="15" t="inlineStr"/>
+      <c r="E45" s="15" t="inlineStr"/>
+      <c r="F45" s="15" t="inlineStr"/>
+      <c r="G45" s="15" t="inlineStr"/>
+      <c r="H45" s="15" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="B46" s="78" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" s="40" t="n">
+        <v>2350</v>
+      </c>
+      <c r="D46" s="15" t="inlineStr"/>
+      <c r="E46" s="15" t="inlineStr"/>
+      <c r="F46" s="15" t="inlineStr"/>
+      <c r="G46" s="15" t="inlineStr"/>
+      <c r="H46" s="15" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="B47" s="78" t="n">
+        <v>10</v>
+      </c>
+      <c r="C47" s="40" t="n">
+        <v>2600</v>
+      </c>
+      <c r="D47" s="15" t="inlineStr"/>
+      <c r="E47" s="15" t="inlineStr"/>
+      <c r="F47" s="15" t="inlineStr"/>
+      <c r="G47" s="15" t="inlineStr"/>
+      <c r="H47" s="15" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="B48" s="78" t="n">
+        <v>100</v>
+      </c>
+      <c r="C48" s="40" t="n">
+        <v>2925</v>
+      </c>
+      <c r="D48" s="15" t="inlineStr"/>
+      <c r="E48" s="15" t="inlineStr"/>
+      <c r="F48" s="15" t="inlineStr"/>
+      <c r="G48" s="15" t="inlineStr"/>
+      <c r="H48" s="15" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="B49" s="78" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C49" s="40" t="n">
+        <v>4775</v>
+      </c>
+      <c r="D49" s="15" t="inlineStr"/>
+      <c r="E49" s="15" t="inlineStr"/>
+      <c r="F49" s="15" t="inlineStr"/>
+      <c r="G49" s="15" t="inlineStr"/>
+      <c r="H49" s="15" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>En dessous de ces températures, l'équilibre complet donne B'c = 0 (MoO2 solide) et la surface nue 0.466 : la vérité est entre les deux, fixée par la cinétique. Au-dessus, les deux tables coïncident ; fusion du métal à 2896 K, puis sublimation jusqu'au plafond B'c = 200.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>§7 — RÉPONSE MATÉRIAU (n'entre PAS dans le XML)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="35" t="inlineStr">
+        <is>
+          <t>couplage k = B'g / B'c</t>
+        </is>
+      </c>
+      <c r="C53" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="I53" s="12" t="inlineStr">
+        <is>
+          <t>pas de pyrolyse interne</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="35" t="inlineStr">
+        <is>
+          <t>récession par unité de flux en limite de diffusion, B'c/ρ [m³/kg]</t>
+        </is>
+      </c>
+      <c r="C54" s="41">
+        <f>C27/C21</f>
+        <v>4.556295971060625e-05</v>
+      </c>
+      <c r="I54" s="12" t="inlineStr">
+        <is>
+          <t>ṡ = B'c·ṁe/ρ — borne haute au-dessus de ~1000 K</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="12" t="inlineStr">
+        <is>
+          <t>Dans l'air, le TZM s'emploie revêtu (siliciures de type MoSi2). La table décrit le métal mis à nu par une défaillance du revêtement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="18" customHeight="1">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>§8 — BLOC XML</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="29" t="inlineStr">
+        <is>
+          <t>&lt;mixture thermo_db="NASA-9"&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    &lt;species&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        N O NO N2 O2</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        Mo MoO MoO2 MoO3 Mo2O6 Mo3O9 Mo4O12 Mo5O15</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        Mo(cr) Mo(L) MoO2(cr) MoO3(cr) MoO3(L)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    &lt;/species&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    &lt;element_compositions default="air"&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        &lt;composition name="air"&gt;N:0.79, O:0.21&lt;/composition&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        &lt;composition name="mo"&gt;Mo:1.0&lt;/composition&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    &lt;/element_compositions&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="29" t="inlineStr">
+        <is>
+          <t>&lt;/mixture&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="16" customHeight="1">
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>bprime -T 300:25:5000 -P &lt;P&gt; -b 0.0 -m mo-air -bl air -char mo -char-elem N</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="34">
+    <mergeCell ref="A41:I41"/>
+    <mergeCell ref="B62:I62"/>
+    <mergeCell ref="A18:I18"/>
+    <mergeCell ref="B24:H24"/>
+    <mergeCell ref="B59:I59"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="B15:H15"/>
+    <mergeCell ref="B66:I66"/>
+    <mergeCell ref="A12:I12"/>
+    <mergeCell ref="B58:I58"/>
+    <mergeCell ref="A57:I57"/>
+    <mergeCell ref="B70:I70"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A5:I5"/>
+    <mergeCell ref="A23:I23"/>
+    <mergeCell ref="B16:H16"/>
+    <mergeCell ref="B60:I60"/>
+    <mergeCell ref="B67:I67"/>
+    <mergeCell ref="B25:H25"/>
+    <mergeCell ref="B61:I61"/>
+    <mergeCell ref="A52:I52"/>
+    <mergeCell ref="B34:I34"/>
+    <mergeCell ref="A30:I30"/>
+    <mergeCell ref="B65:I65"/>
+    <mergeCell ref="B14:H14"/>
+    <mergeCell ref="B68:I68"/>
+    <mergeCell ref="B64:I64"/>
+    <mergeCell ref="B13:H13"/>
+    <mergeCell ref="B55:I55"/>
+    <mergeCell ref="A36:I36"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="B63:I63"/>
+    <mergeCell ref="B50:I50"/>
+    <mergeCell ref="B26:I26"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Ajoute la mise en données du bois de chêne et l'onglet Chêne du classeur
Bois de chêne sec, rendement en char 20 % : fermeture élémentaire bois − char
sur l'analyse C 50.0 / H 6.1 / O 43.9 (contrôlée par la reconstruction depuis
les unités de répétition cellulose / xylane / lignine S+G / ellagitanins).
Gaz oak_pyro C:0.221, H:0.536, O:0.243, char C:1.0, k = 4.0.

- data/mixtures/oak-air.xml et oak-pyrogas.xml
- oak_bprime/ : scripts de composition, tables B'c/h_w et h_g, documentation
- onglet Chêne du classeur, vérifié contre oak-air.xml (écart 0.08 %)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XRtNxD16XChjc3GYaFqTeK
</commit_message>
<xml_diff>
--- a/mise_en_donnees_xlsx/mise_en_donnees_materiaux.xlsx
+++ b/mise_en_donnees_xlsx/mise_en_donnees_materiaux.xlsx
@@ -15,10 +15,11 @@
     <sheet name="SC-1008" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="MX-4926" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Liège-phénolique" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Carbone" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Silice" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="SiC" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Molybdène" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Chêne" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Carbone" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Silice" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="SiC" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Molybdène" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -181,7 +182,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -279,11 +280,13 @@
     <xf numFmtId="164" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="7" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="7" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="7" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="173" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -653,7 +656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I56"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4.5" customWidth="1" min="1" max="1"/>
@@ -684,7 +687,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Fichier(s) XML : data/mixtures/ — 11 matériaux, 19 fichiers de mélange</t>
+          <t>Fichier(s) XML : data/mixtures/ — 12 matériaux, 21 fichiers de mélange</t>
         </is>
       </c>
     </row>
@@ -955,239 +958,244 @@
     <row r="18">
       <c r="B18" s="7" t="inlineStr">
         <is>
+          <t>Bois de chêne</t>
+        </is>
+      </c>
+      <c r="C18" s="8">
+        <f>'Chêne'!C67</f>
+        <v>0.221</v>
+      </c>
+      <c r="D18" s="8">
+        <f>'Chêne'!D67</f>
+        <v>0.536</v>
+      </c>
+      <c r="E18" s="8">
+        <f>'Chêne'!E67</f>
+        <v>0.243</v>
+      </c>
+      <c r="F18" s="9">
+        <f>'Chêne'!D67/'Chêne'!E67</f>
+        <v>2.205761316872428</v>
+      </c>
+      <c r="G18" s="10" t="inlineStr">
+        <is>
+          <t>C:1.0</t>
+        </is>
+      </c>
+      <c r="H18" s="8">
+        <f>'Chêne'!C106</f>
+        <v>4.0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="7" t="inlineStr">
+        <is>
           <t>Carbone graphite</t>
         </is>
       </c>
-      <c r="C18" s="11" t="inlineStr">
+      <c r="C19" s="11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
+      <c r="D19" s="11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E18" s="11" t="inlineStr">
+      <c r="E19" s="11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F18" s="11" t="inlineStr">
+      <c r="F19" s="11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G18" s="10" t="inlineStr">
+      <c r="G19" s="10" t="inlineStr">
         <is>
           <t>C:1.0</t>
         </is>
       </c>
-      <c r="H18" s="8">
+      <c r="H19" s="8">
         <f>'Carbone'!C53</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" s="7" t="inlineStr">
+    <row r="20">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>Silice SiO2</t>
         </is>
       </c>
-      <c r="C19" s="11" t="inlineStr">
+      <c r="C20" s="11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D19" s="11" t="inlineStr">
+      <c r="D20" s="11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
+      <c r="E20" s="11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F19" s="11" t="inlineStr">
+      <c r="F20" s="11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G19" s="10" t="inlineStr">
+      <c r="G20" s="10" t="inlineStr">
         <is>
           <t>Si:1.0, O:2.0</t>
         </is>
       </c>
-      <c r="H19" s="8">
+      <c r="H20" s="8">
         <f>'Silice'!C46</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="7" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Carbure de silicium SiC</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
+      <c r="C21" s="11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D20" s="11" t="inlineStr">
+      <c r="D21" s="11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E20" s="11" t="inlineStr">
+      <c r="E21" s="11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F20" s="11" t="inlineStr">
+      <c r="F21" s="11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G20" s="10" t="inlineStr">
+      <c r="G21" s="10" t="inlineStr">
         <is>
           <t>Si:1.0, C:1.0</t>
         </is>
       </c>
-      <c r="H20" s="8">
+      <c r="H21" s="8">
         <f>'SiC'!C69</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="21">
-      <c r="B21" s="7" t="inlineStr">
+    <row r="22">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>Molybdène (TZM)</t>
         </is>
       </c>
-      <c r="C21" s="11" t="inlineStr">
+      <c r="C22" s="11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D21" s="11" t="inlineStr">
+      <c r="D22" s="11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E21" s="11" t="inlineStr">
+      <c r="E22" s="11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F21" s="11" t="inlineStr">
+      <c r="F22" s="11" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G21" s="10" t="inlineStr">
+      <c r="G22" s="10" t="inlineStr">
         <is>
           <t>Mo:1.0</t>
         </is>
       </c>
-      <c r="H21" s="8">
+      <c r="H22" s="8">
         <f>'Molybdène'!C53</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="12" t="inlineStr">
+    <row r="23">
+      <c r="B23" s="12" t="inlineStr">
         <is>
           <t>Les colonnes « gaz » sont des liens vers la ligne « valeur portée dans le XML » de chaque onglet. Le graphite, la silice, le SiC et le molybdène n'ont pas de gaz de pyrolyse (k = 0). TACOT et CPh70 portent RIGOUREUSEMENT la même composition : leurs fichiers XML sont identiques, seul k les distingue — c'est la démonstration de l'onglet CPh70.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="4" t="inlineStr">
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>§3 — LES TROIS SEULES DONNÉES QUE CONSOMME LE CALCUL</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="B25" s="6" t="inlineStr">
+    <row r="26">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C26" s="6" t="inlineStr">
         <is>
           <t>Composition</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
+      <c r="D26" s="6" t="inlineStr">
         <is>
           <t>Rôle dans le bilan</t>
         </is>
       </c>
-      <c r="E25" s="6" t="inlineStr">
+      <c r="E26" s="6" t="inlineStr">
         <is>
           <t>Option</t>
         </is>
       </c>
-      <c r="F25" s="6" t="inlineStr">
+      <c r="F26" s="6" t="inlineStr">
         <is>
           <t>Comment on l'obtient</t>
         </is>
       </c>
-      <c r="G25" s="6" t="inlineStr"/>
-      <c r="H25" s="6" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>bord de couche limite</t>
-        </is>
-      </c>
-      <c r="D26" s="7" t="inlineStr">
-        <is>
-          <t>Y_e</t>
-        </is>
-      </c>
-      <c r="E26" s="14" t="inlineStr">
-        <is>
-          <t>-bl</t>
-        </is>
-      </c>
-      <c r="F26" s="11" t="inlineStr">
-        <is>
-          <t>l'atmosphère : air N:0.79 O:0.21 · Mars · Titan…</t>
-        </is>
-      </c>
-      <c r="G26" s="15" t="inlineStr"/>
-      <c r="H26" s="15" t="inlineStr"/>
+      <c r="G26" s="6" t="inlineStr"/>
+      <c r="H26" s="6" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="B27" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>gaz de pyrolyse</t>
+          <t>bord de couche limite</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>Y_g</t>
+          <t>Y_e</t>
         </is>
       </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
-          <t>-py</t>
+          <t>-bl</t>
         </is>
       </c>
       <c r="F27" s="11" t="inlineStr">
         <is>
-          <t>c'est TOUT l'objet de ce classeur — quatre routes possibles, §4</t>
+          <t>l'atmosphère : air N:0.79 O:0.21 · Mars · Titan…</t>
         </is>
       </c>
       <c r="G27" s="15" t="inlineStr"/>
@@ -1195,127 +1203,125 @@
     </row>
     <row r="28">
       <c r="B28" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>char</t>
+          <t>gaz de pyrolyse</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Y_c</t>
+          <t>Y_g</t>
         </is>
       </c>
       <c r="E28" s="14" t="inlineStr">
         <is>
-          <t>-char + -char-elem</t>
+          <t>-py</t>
         </is>
       </c>
       <c r="F28" s="11" t="inlineStr">
         <is>
-          <t>C:1.0 si tous les constituants carbonisent vers le carbone ; sinon pondérer par les masses de char</t>
+          <t>c'est TOUT l'objet de ce classeur — quatre routes possibles, §4</t>
         </is>
       </c>
       <c r="G28" s="15" t="inlineStr"/>
       <c r="H28" s="15" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="B29" s="12" t="inlineStr">
+      <c r="B29" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>char</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Y_c</t>
+        </is>
+      </c>
+      <c r="E29" s="14" t="inlineStr">
+        <is>
+          <t>-char + -char-elem</t>
+        </is>
+      </c>
+      <c r="F29" s="11" t="inlineStr">
+        <is>
+          <t>C:1.0 si tous les constituants carbonisent vers le carbone ; sinon pondérer par les masses de char</t>
+        </is>
+      </c>
+      <c r="G29" s="15" t="inlineStr"/>
+      <c r="H29" s="15" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="12" t="inlineStr">
         <is>
           <t>Plus T, P et B'g. Rien d'autre : cf. src/apps/bprime.cpp:304-330. Sans -char/-char-elem, bprime utilise un char de carbone pur intégré ; les deux options vont toujours ensemble.</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="4" t="inlineStr">
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>§4 — LES QUATRE ROUTES DE CALCUL DU GAZ DE PYROLYSE</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="B32" s="6" t="inlineStr">
+    <row r="33">
+      <c r="B33" s="6" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="C32" s="6" t="inlineStr">
+      <c r="C33" s="6" t="inlineStr">
         <is>
           <t>Matériau</t>
         </is>
       </c>
-      <c r="D32" s="6" t="inlineStr">
+      <c r="D33" s="6" t="inlineStr">
         <is>
           <t>Donnée primaire</t>
         </is>
       </c>
-      <c r="E32" s="6" t="inlineStr">
+      <c r="E33" s="6" t="inlineStr">
         <is>
           <t>Passage à l'élémentaire</t>
         </is>
       </c>
-      <c r="F32" s="6" t="inlineStr">
+      <c r="F33" s="6" t="inlineStr">
         <is>
           <t>Point critique</t>
         </is>
       </c>
-      <c r="G32" s="6" t="inlineStr"/>
-      <c r="H32" s="6" t="inlineStr"/>
-    </row>
-    <row r="33" ht="28" customHeight="1">
-      <c r="B33" s="16" t="inlineStr">
-        <is>
-          <t>A — sommation atomique</t>
-        </is>
-      </c>
-      <c r="C33" s="17" t="inlineStr">
-        <is>
-          <t>TACOT, CPh70</t>
-        </is>
-      </c>
-      <c r="D33" s="17" t="inlineStr">
-        <is>
-          <t>spéciation moléculaire mesurée (7 espèces)</t>
-        </is>
-      </c>
-      <c r="E33" s="18" t="inlineStr">
-        <is>
-          <t>n_E = Σ_j ν_E,j · x_j</t>
-        </is>
-      </c>
-      <c r="F33" s="19" t="inlineStr">
-        <is>
-          <t>la renormalisation : somme réelle des colonnes (100.30), pas les totaux imprimés (100.0)</t>
-        </is>
-      </c>
-      <c r="G33" s="15" t="inlineStr"/>
-      <c r="H33" s="15" t="inlineStr"/>
+      <c r="G33" s="6" t="inlineStr"/>
+      <c r="H33" s="6" t="inlineStr"/>
     </row>
     <row r="34" ht="28" customHeight="1">
       <c r="B34" s="16" t="inlineStr">
         <is>
-          <t>B — conversion directe</t>
+          <t>A — sommation atomique</t>
         </is>
       </c>
       <c r="C34" s="17" t="inlineStr">
         <is>
-          <t>ZURAM</t>
+          <t>TACOT, CPh70</t>
         </is>
       </c>
       <c r="D34" s="17" t="inlineStr">
         <is>
-          <t>composition élémentaire MASSIQUE mesurée</t>
+          <t>spéciation moléculaire mesurée (7 espèces)</t>
         </is>
       </c>
       <c r="E34" s="18" t="inlineStr">
         <is>
-          <t>x_E = (y_E/M_E) / Σ (y_j/M_j)</t>
+          <t>n_E = Σ_j ν_E,j · x_j</t>
         </is>
       </c>
       <c r="F34" s="19" t="inlineStr">
         <is>
-          <t>traçabilité limitée à 3 décimales ; la source primaire VKI n'est pas publique</t>
+          <t>la renormalisation : somme réelle des colonnes (100.30), pas les totaux imprimés (100.0)</t>
         </is>
       </c>
       <c r="G34" s="15" t="inlineStr"/>
@@ -1324,27 +1330,27 @@
     <row r="35" ht="28" customHeight="1">
       <c r="B35" s="16" t="inlineStr">
         <is>
-          <t>C — fermeture élémentaire</t>
+          <t>B — conversion directe</t>
         </is>
       </c>
       <c r="C35" s="17" t="inlineStr">
         <is>
-          <t>SC-1008</t>
+          <t>ZURAM</t>
         </is>
       </c>
       <c r="D35" s="17" t="inlineStr">
         <is>
-          <t>motif chimique idéalisé + rendement en char</t>
+          <t>composition élémentaire MASSIQUE mesurée</t>
         </is>
       </c>
       <c r="E35" s="18" t="inlineStr">
         <is>
-          <t>n_E(gaz) = n_E(résine) − n_E(char)</t>
+          <t>x_E = (y_E/M_E) / Σ (y_j/M_j)</t>
         </is>
       </c>
       <c r="F35" s="19" t="inlineStr">
         <is>
-          <t>le rendement en char entre DANS la chaîne : ±0.05 sur Y déplace le carbone de ~12 %</t>
+          <t>traçabilité limitée à 3 décimales ; la source primaire VKI n'est pas publique</t>
         </is>
       </c>
       <c r="G35" s="15" t="inlineStr"/>
@@ -1353,27 +1359,27 @@
     <row r="36" ht="28" customHeight="1">
       <c r="B36" s="16" t="inlineStr">
         <is>
-          <t>D — fermeture sur DEUX constituants</t>
+          <t>C — fermeture élémentaire</t>
         </is>
       </c>
       <c r="C36" s="17" t="inlineStr">
         <is>
-          <t>Liège/phénolique</t>
+          <t>SC-1008, Chêne</t>
         </is>
       </c>
       <c r="D36" s="17" t="inlineStr">
         <is>
-          <t>analyses des deux constituants + rendements</t>
+          <t>motif idéalisé (SC-1008) ou analyse élémentaire (chêne) + rendement en char</t>
         </is>
       </c>
       <c r="E36" s="18" t="inlineStr">
         <is>
-          <t>n_E(gaz) = Σ_i [n_E(i) − n_E(char,i)]</t>
+          <t>n_E(gaz) = n_E(solide) − n_E(char)</t>
         </is>
       </c>
       <c r="F36" s="19" t="inlineStr">
         <is>
-          <t>le renfort pyrolyse : le rapport renfort/résine entre dans la table B'</t>
+          <t>le rendement en char entre DANS la chaîne : ±0.05 sur Y déplace le carbone de ~12 %</t>
         </is>
       </c>
       <c r="G36" s="15" t="inlineStr"/>
@@ -1382,85 +1388,93 @@
     <row r="37" ht="28" customHeight="1">
       <c r="B37" s="16" t="inlineStr">
         <is>
-          <t>E — stœchiométrie directe</t>
+          <t>D — fermeture sur DEUX constituants</t>
         </is>
       </c>
       <c r="C37" s="17" t="inlineStr">
         <is>
-          <t>Carbone, Silice, SiC, Mo</t>
+          <t>Liège/phénolique</t>
         </is>
       </c>
       <c r="D37" s="17" t="inlineStr">
         <is>
-          <t>la formule du solide</t>
+          <t>analyses des deux constituants + rendements</t>
         </is>
       </c>
       <c r="E37" s="18" t="inlineStr">
         <is>
-          <t>aucun gaz de pyrolyse (B'g = 0)</t>
+          <t>n_E(gaz) = Σ_i [n_E(i) − n_E(char,i)]</t>
         </is>
       </c>
       <c r="F37" s="19" t="inlineStr">
         <is>
-          <t>le char EST le matériau ; -char-elem Si pour la silice, N pour le SiC (char non congruent)</t>
+          <t>le renfort pyrolyse : le rapport renfort/résine entre dans la table B'</t>
         </is>
       </c>
       <c r="G37" s="15" t="inlineStr"/>
       <c r="H37" s="15" t="inlineStr"/>
     </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="4" t="inlineStr">
+    <row r="38" ht="28" customHeight="1">
+      <c r="B38" s="16" t="inlineStr">
+        <is>
+          <t>E — stœchiométrie directe</t>
+        </is>
+      </c>
+      <c r="C38" s="17" t="inlineStr">
+        <is>
+          <t>Carbone, Silice, SiC, Mo</t>
+        </is>
+      </c>
+      <c r="D38" s="17" t="inlineStr">
+        <is>
+          <t>la formule du solide</t>
+        </is>
+      </c>
+      <c r="E38" s="18" t="inlineStr">
+        <is>
+          <t>aucun gaz de pyrolyse (B'g = 0)</t>
+        </is>
+      </c>
+      <c r="F38" s="19" t="inlineStr">
+        <is>
+          <t>le char EST le matériau ; -char-elem Si pour la silice, N pour le SiC (char non congruent)</t>
+        </is>
+      </c>
+      <c r="G38" s="15" t="inlineStr"/>
+      <c r="H38" s="15" t="inlineStr"/>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>§5 — CE QUI N'ENTRE PAS DANS LE XML</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="B40" s="6" t="inlineStr">
+    <row r="41">
+      <c r="B41" s="6" t="inlineStr">
         <is>
           <t>Donnée</t>
         </is>
       </c>
-      <c r="C40" s="6" t="inlineStr">
+      <c r="C41" s="6" t="inlineStr">
         <is>
           <t>Dans le XML ?</t>
         </is>
       </c>
-      <c r="D40" s="6" t="inlineStr">
+      <c r="D41" s="6" t="inlineStr">
         <is>
           <t>Où elle sert vraiment</t>
         </is>
       </c>
-      <c r="E40" s="6" t="inlineStr"/>
-      <c r="F40" s="6" t="inlineStr"/>
-      <c r="G40" s="6" t="inlineStr"/>
-      <c r="H40" s="6" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="B41" s="7" t="inlineStr">
-        <is>
-          <t>masse volumique ρ_v, ρ_c</t>
-        </is>
-      </c>
-      <c r="C41" s="13" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="D41" s="11" t="inlineStr">
-        <is>
-          <t>solveur de réponse matériau ; récession ṡ = B'c·ṁe/ρ_c</t>
-        </is>
-      </c>
-      <c r="E41" s="15" t="inlineStr"/>
-      <c r="F41" s="15" t="inlineStr"/>
-      <c r="G41" s="15" t="inlineStr"/>
-      <c r="H41" s="15" t="inlineStr"/>
+      <c r="E41" s="6" t="inlineStr"/>
+      <c r="F41" s="6" t="inlineStr"/>
+      <c r="G41" s="6" t="inlineStr"/>
+      <c r="H41" s="6" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>porosité</t>
+          <t>masse volumique ρ_v, ρ_c</t>
         </is>
       </c>
       <c r="C42" s="13" t="inlineStr">
@@ -1470,7 +1484,7 @@
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>conduction, perméabilité</t>
+          <t>solveur de réponse matériau ; récession ṡ = B'c·ṁe/ρ_c</t>
         </is>
       </c>
       <c r="E42" s="15" t="inlineStr"/>
@@ -1481,17 +1495,17 @@
     <row r="43">
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>rapport fibres/résine</t>
+          <t>porosité</t>
         </is>
       </c>
       <c r="C43" s="13" t="inlineStr">
         <is>
-          <t>non *</t>
+          <t>non</t>
         </is>
       </c>
       <c r="D43" s="11" t="inlineStr">
         <is>
-          <t>fixe la QUANTITÉ de gaz (donc B'g), pas sa composition</t>
+          <t>conduction, perméabilité</t>
         </is>
       </c>
       <c r="E43" s="15" t="inlineStr"/>
@@ -1502,7 +1516,7 @@
     <row r="44">
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>rendement en char</t>
+          <t>rapport fibres/résine</t>
         </is>
       </c>
       <c r="C44" s="13" t="inlineStr">
@@ -1512,7 +1526,7 @@
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>idem — mais il entre dans le CALCUL du gaz pour les routes C et D</t>
+          <t>fixe la QUANTITÉ de gaz (donc B'g), pas sa composition</t>
         </is>
       </c>
       <c r="E44" s="15" t="inlineStr"/>
@@ -1523,17 +1537,17 @@
     <row r="45">
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>cinétique de pyrolyse</t>
+          <t>rendement en char</t>
         </is>
       </c>
       <c r="C45" s="13" t="inlineStr">
         <is>
-          <t>non</t>
+          <t>non *</t>
         </is>
       </c>
       <c r="D45" s="11" t="inlineStr">
         <is>
-          <t>fixe B'g au cours du temps</t>
+          <t>idem — mais il entre dans le CALCUL du gaz pour les routes C et D</t>
         </is>
       </c>
       <c r="E45" s="15" t="inlineStr"/>
@@ -1542,106 +1556,127 @@
       <c r="H45" s="15" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="B46" s="12" t="inlineStr">
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>cinétique de pyrolyse</t>
+        </is>
+      </c>
+      <c r="C46" s="13" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="D46" s="11" t="inlineStr">
+        <is>
+          <t>fixe B'g au cours du temps</t>
+        </is>
+      </c>
+      <c r="E46" s="15" t="inlineStr"/>
+      <c r="F46" s="15" t="inlineStr"/>
+      <c r="G46" s="15" t="inlineStr"/>
+      <c r="H46" s="15" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="B47" s="12" t="inlineStr">
         <is>
           <t>* sauf si les constituants donnent des chars de compositions élémentaires DIFFÉRENTES (fibres de silice + résine phénolique), ou si le renfort pyrolyse (liège) : le rapport entre alors dans Y_c et/ou Y_g, et la table change. Le bilan de masse de surface est écrit sur des fractions massiques élémentaires, donc normalisées : les grandeurs VOLUMIQUES n'y ont structurellement aucune place.</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="4" t="inlineStr">
+    <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="4" t="inlineStr">
         <is>
           <t>§6 — RECETTE POUR UN NOUVEAU MATÉRIAU</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="B49" s="5" t="inlineStr">
-        <is>
-          <t>Atmosphère → composition -bl (air, Mars, Titan…).</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>Résine → composition du gaz de pyrolyse par l'une des quatre routes du §4 → composition -py.</t>
+          <t>Atmosphère → composition -bl (air, Mars, Titan…).</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>Char → C:1.0 si tous les constituants carbonisent vers le carbone ; sinon pondérer par les masses de char de chaque constituant.</t>
+          <t>Résine → composition du gaz de pyrolyse par l'une des quatre routes du §4 → composition -py.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>Espèces → tous les produits attendus des éléments présents, PLUS la ou les phases condensées.</t>
+          <t>Char → C:1.0 si tous les constituants carbonisent vers le carbone ; sinon pondérer par les masses de char de chaque constituant.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="20" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>Vérifier : checkmix (noms, phases), puis un run court.</t>
+          <t>Espèces → tous les produits attendus des éléments présents, PLUS la ou les phases condensées.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Vérifier : checkmix (noms, phases), puis un run court.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="B54" s="5" t="inlineStr">
+      <c r="B55" s="5" t="inlineStr">
         <is>
           <t>Contrôler la physique : à 300 K et B'g = 0 dans l'air, un char carboné doit donner B'c ≈ 0.0874 (limite C + O2 → CO2, indépendante de la pression). Une valeur ≈ 200 signale l'absence de C(gr). Pour un char multi-élément susceptible de laisser un autre solide à la paroi (SiC), suivre le bilan sur N (-char-elem N).</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="30" customHeight="1">
-      <c r="B56" s="5" t="inlineStr">
-        <is>
-          <t>Documents de référence du dépôt : tacot_bprime/mise_en_donnees_xml.md (mécanique du fichier XML et règles du parseur) · resine_tacot.md · zuram_bprime/resine_zuram.md · sc1008_bprime/resine_sc1008.md · cork_bprime/mise_en_donnees_cork.md · tacot_bprime/cph70_vs_tacot.md · carbon_bprime/bprime_carbon_physique.md · sic_bprime/README.md · mo_bprime/README.md.</t>
+    <row r="57" ht="30" customHeight="1">
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>Documents de référence du dépôt : tacot_bprime/mise_en_donnees_xml.md (mécanique du fichier XML et règles du parseur) · resine_tacot.md · zuram_bprime/resine_zuram.md · sc1008_bprime/resine_sc1008.md · cork_bprime/mise_en_donnees_cork.md · oak_bprime/mise_en_donnees_chene.md · tacot_bprime/cph70_vs_tacot.md · carbon_bprime/bprime_carbon_physique.md · sic_bprime/README.md · mo_bprime/README.md.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="A25:I25"/>
     <mergeCell ref="B7:I7"/>
+    <mergeCell ref="B47:I47"/>
     <mergeCell ref="B54:I54"/>
-    <mergeCell ref="B22:I22"/>
     <mergeCell ref="A3:I3"/>
-    <mergeCell ref="B46:I46"/>
-    <mergeCell ref="B56:I56"/>
     <mergeCell ref="B52:I52"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A5:I5"/>
+    <mergeCell ref="A32:I32"/>
+    <mergeCell ref="B23:I23"/>
+    <mergeCell ref="B57:I57"/>
     <mergeCell ref="B8:I8"/>
     <mergeCell ref="B53:I53"/>
-    <mergeCell ref="B29:I29"/>
     <mergeCell ref="A10:I10"/>
-    <mergeCell ref="A31:I31"/>
-    <mergeCell ref="A39:I39"/>
-    <mergeCell ref="A48:I48"/>
-    <mergeCell ref="B49:I49"/>
-    <mergeCell ref="A24:I24"/>
+    <mergeCell ref="A40:I40"/>
+    <mergeCell ref="B30:I30"/>
+    <mergeCell ref="A49:I49"/>
+    <mergeCell ref="B55:I55"/>
     <mergeCell ref="B6:I6"/>
     <mergeCell ref="B51:I51"/>
     <mergeCell ref="A1:I1"/>
@@ -1652,6 +1687,846 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00404040"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I67"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4.5" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="72" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Carbone graphite — ablateur non pyrolysant</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Cas dégénéré : le solide EST le char, il n'y a pas de gaz de pyrolyse · sert de cas de référence physique aux autres onglets</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Fichier(s) XML : data/mixtures/carbon-air.xml</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>§0 — FICHE D'IDENTITÉ</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="35" t="inlineStr">
+        <is>
+          <t>Matériau</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="inlineStr">
+        <is>
+          <t>graphite pur (carbone massif)</t>
+        </is>
+      </c>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>carbon_bprime/bprime_carbon_physique.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="35" t="inlineStr">
+        <is>
+          <t>Renfort / résine</t>
+        </is>
+      </c>
+      <c r="C7" s="30" t="inlineStr">
+        <is>
+          <t>sans objet — matériau monolithique</t>
+        </is>
+      </c>
+      <c r="I7" s="12" t="inlineStr">
+        <is>
+          <t>aucune pyrolyse interne</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="35" t="inlineStr">
+        <is>
+          <t>Système chimique</t>
+        </is>
+      </c>
+      <c r="C8" s="30" t="inlineStr">
+        <is>
+          <t>C-N-O : 5 espèces d'air + 3 formes gazeuses du carbone + CO, CO2, CN + C(gr)</t>
+        </is>
+      </c>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>12 espèces au total</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="35" t="inlineStr">
+        <is>
+          <t>Compositions du XML</t>
+        </is>
+      </c>
+      <c r="C9" s="30" t="inlineStr">
+        <is>
+          <t>air (-bl) · pyro = C:1.0 (-py, et définit le char)</t>
+        </is>
+      </c>
+      <c r="I9" s="12" t="inlineStr"/>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>§1 — HYPOTHÈSES</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Pas de pyrolyse interne : B'g = 0.</t>
+        </is>
+      </c>
+      <c r="I12" s="12" t="inlineStr">
+        <is>
+          <t>Il n'y a pas de résine à décomposer. Toute la masse injectée vient de la surface, d'où le nom de « cas dégénéré ».</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="A13" s="20" t="inlineStr">
+        <is>
+          <t>H2</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Le char est le matériau lui-même : carbone pur, C:1.0.</t>
+        </is>
+      </c>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>Aucune fermeture élémentaire à faire — c'est la seule mise en données du dépôt où la composition ne se CALCULE pas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="26" customHeight="1">
+      <c r="A14" s="20" t="inlineStr">
+        <is>
+          <t>H3</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Équilibre thermochimique à la paroi, char infini.</t>
+        </is>
+      </c>
+      <c r="I14" s="12" t="inlineStr">
+        <is>
+          <t>Le solveur ajoute δ = max(200, 100·B'g) de carbone élémentaire à la composition du bord de couche limite avant de normaliser, puis calcule l'équilibre multiphase.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>C(gr) est indispensable dans la liste d'espèces.</t>
+        </is>
+      </c>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>Sans phase condensée, C3 gazeux domine dès 300 K, Y_w,C → 1 et B'c ≈ 200 — non physique. C'est le contrôle du §5, valable pour TOUS les onglets carbonés.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>§2 — DONNÉES D'ENTRÉE</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="35" t="inlineStr">
+        <is>
+          <t>bord de couche limite</t>
+        </is>
+      </c>
+      <c r="C18" s="30" t="inlineStr">
+        <is>
+          <t>air : N:0.79, O:0.21 (molaire)</t>
+        </is>
+      </c>
+      <c r="I18" s="12" t="inlineStr">
+        <is>
+          <t>cf. onglet Constantes §2</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="35" t="inlineStr">
+        <is>
+          <t>fraction massique d'oxygène de l'air</t>
+        </is>
+      </c>
+      <c r="C19" s="50">
+        <f>Constantes!D19</f>
+        <v>0.23290921795842306</v>
+      </c>
+      <c r="I19" s="12" t="inlineStr">
+        <is>
+          <t>y_O calculé au §2 de l'onglet Constantes</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="35" t="inlineStr">
+        <is>
+          <t>masse volumique du graphite [kg/m³]</t>
+        </is>
+      </c>
+      <c r="C20" s="30" t="n">
+        <v>1800</v>
+      </c>
+      <c r="I20" s="12" t="inlineStr">
+        <is>
+          <t>ordre de grandeur (1600-2200 selon la qualité) — n'entre que dans la récession</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>§3 — CALCUL PAS À PAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="20" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="B23" s="20" t="inlineStr">
+        <is>
+          <t>Étape 1 — composition élémentaire du char : directe</t>
+        </is>
+      </c>
+      <c r="I23" s="27" t="inlineStr">
+        <is>
+          <t>le solide est du carbone pur ⇒ x_C = 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="6" t="inlineStr"/>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>Somme</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr"/>
+      <c r="H24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>char (= le matériau)</t>
+        </is>
+      </c>
+      <c r="C25" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="24">
+        <f>SUM(C25:E25)</f>
+        <v>1.0</v>
+      </c>
+      <c r="G25" s="15" t="inlineStr"/>
+      <c r="H25" s="15" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="20" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="B26" s="20" t="inlineStr">
+        <is>
+          <t>Étape 2 — gaz de pyrolyse : il n'y en a pas</t>
+        </is>
+      </c>
+      <c r="I26" s="27" t="inlineStr">
+        <is>
+          <t>B'g = 0 dans toutes les commandes bprime de ce matériau</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>La composition nommée `pyro` du XML vaut néanmoins C:1.0. Ce n'est pas une incohérence : elle sert d'argument à `-py` (le parseur exige une composition valide) et définit le char. Comme elle est appelée avec -b 0.0, elle ne contribue à rien.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="20" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="B28" s="20" t="inlineStr">
+        <is>
+          <t>Étape 3 — le bilan de surface se réduit à une expression fermée</t>
+        </is>
+      </c>
+      <c r="I28" s="27" t="inlineStr">
+        <is>
+          <t>B'c = [Y_e,C + B'g·Y_g,C − Y_w,C(1+B'g)] / (Y_w,C − Y_c,C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="16" customHeight="1">
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Avec Y_c,C = 1 (char de carbone pur), Y_e,C = 0 (l'air ne contient pas de carbone) et B'g = 0, il ne reste que :</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   B'c = − Y_w,C / (Y_w,C − 1) = Y_w,C / (1 − Y_w,C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>La seule inconnue est Y_w,C, la fraction massique de carbone dans le gaz d'équilibre à la paroi — c'est elle que le solveur multiphase calcule à (T_w, P).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>§4 — RÉSULTAT : CE QUI ENTRE DANS LE XML</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>Composition élémentaire (fractions molaires)</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>Somme</t>
+        </is>
+      </c>
+      <c r="G34" s="6" t="inlineStr"/>
+      <c r="H34" s="6" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>pyro / char — valeur portée dans le XML</t>
+        </is>
+      </c>
+      <c r="C35" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E35" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F35" s="15" t="inlineStr"/>
+      <c r="G35" s="15" t="inlineStr"/>
+      <c r="H35" s="15" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>air — valeur portée dans le XML</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D36" s="44" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="E36" s="44" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="F36" s="24">
+        <f>D36+E36</f>
+        <v>1.0</v>
+      </c>
+      <c r="G36" s="15" t="inlineStr"/>
+      <c r="H36" s="15" t="inlineStr"/>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>§5 — CONTRÔLES ET VALIDATION CROISÉE</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="20" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="B39" s="20" t="inlineStr">
+        <is>
+          <t>Contrôle de recette valable pour TOUS les matériaux carbonés du dépôt</t>
+        </is>
+      </c>
+      <c r="I39" s="27" t="inlineStr">
+        <is>
+          <t>à 300 K, B'g = 0 : régime d'oxydation basse température, C(gr) + O2 → CO2</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>À 300 K tout l'oxygène de l'air est consommé en CO2. Chaque O2 (2 atomes d'oxygène) emporte un atome de carbone : la masse de carbone ablatée par unité de masse d'air vaut donc y_O · M_C / (2·M_O). Ce nombre ne dépend PAS de la pression.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="35" t="inlineStr">
+        <is>
+          <t>B'c attendu à 300 K, 1 atm</t>
+        </is>
+      </c>
+      <c r="C41" s="74">
+        <f>C19*Constantes!$C$7/(2*Constantes!$C$9)</f>
+        <v>0.08742648343329643</v>
+      </c>
+      <c r="I41" s="12" t="inlineStr">
+        <is>
+          <t>attendu 0.0874 — valeur obtenue par bprime sur carbon-air, cork-air, tacot-air…</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="35" t="inlineStr">
+        <is>
+          <t>B'c obtenu si C(gr) manque dans &lt;species&gt;</t>
+        </is>
+      </c>
+      <c r="C42" s="31" t="inlineStr">
+        <is>
+          <t>≈ 200</t>
+        </is>
+      </c>
+      <c r="I42" s="12" t="inlineStr">
+        <is>
+          <t>signature sans ambiguïté d'une liste d'espèces incomplète : Y_w,C → 1 et B'c sature sur son plafond interne</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>§6 — SENSIBILITÉ — régimes physiques (à 1 atm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>Régime</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>T_w [K]</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="inlineStr">
+        <is>
+          <t>Phase stable</t>
+        </is>
+      </c>
+      <c r="E45" s="6" t="inlineStr">
+        <is>
+          <t>Espèce gazeuse dominante</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>Mécanisme</t>
+        </is>
+      </c>
+      <c r="G45" s="6" t="inlineStr"/>
+      <c r="H45" s="6" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="B46" s="7" t="inlineStr">
+        <is>
+          <t>faible ablation</t>
+        </is>
+      </c>
+      <c r="C46" s="75" t="inlineStr">
+        <is>
+          <t>300 – 700</t>
+        </is>
+      </c>
+      <c r="D46" s="75" t="inlineStr">
+        <is>
+          <t>C(gr)</t>
+        </is>
+      </c>
+      <c r="E46" s="75" t="inlineStr">
+        <is>
+          <t>CO2, O2, N2</t>
+        </is>
+      </c>
+      <c r="F46" s="11" t="inlineStr">
+        <is>
+          <t>C(gr) + O2 → CO2</t>
+        </is>
+      </c>
+      <c r="G46" s="15" t="inlineStr"/>
+      <c r="H46" s="15" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>oxydation active</t>
+        </is>
+      </c>
+      <c r="C47" s="75" t="inlineStr">
+        <is>
+          <t>700 – 3500</t>
+        </is>
+      </c>
+      <c r="D47" s="75" t="inlineStr">
+        <is>
+          <t>C(gr)</t>
+        </is>
+      </c>
+      <c r="E47" s="75" t="inlineStr">
+        <is>
+          <t>CO, N2, CN</t>
+        </is>
+      </c>
+      <c r="F47" s="11" t="inlineStr">
+        <is>
+          <t>C(gr) + O → CO ; Boudouard C(gr) + CO2 → 2 CO</t>
+        </is>
+      </c>
+      <c r="G47" s="15" t="inlineStr"/>
+      <c r="H47" s="15" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>sublimation</t>
+        </is>
+      </c>
+      <c r="C48" s="75" t="inlineStr">
+        <is>
+          <t>3500 – 4000</t>
+        </is>
+      </c>
+      <c r="D48" s="75" t="inlineStr">
+        <is>
+          <t>C(gr) + gaz</t>
+        </is>
+      </c>
+      <c r="E48" s="75" t="inlineStr">
+        <is>
+          <t>CO, CN, C3</t>
+        </is>
+      </c>
+      <c r="F48" s="11" t="inlineStr">
+        <is>
+          <t>C(gr) ⇌ C, C2, C3</t>
+        </is>
+      </c>
+      <c r="G48" s="15" t="inlineStr"/>
+      <c r="H48" s="15" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>sublimation totale</t>
+        </is>
+      </c>
+      <c r="C49" s="75" t="inlineStr">
+        <is>
+          <t>&gt; 4000</t>
+        </is>
+      </c>
+      <c r="D49" s="75" t="inlineStr">
+        <is>
+          <t>gaz seul</t>
+        </is>
+      </c>
+      <c r="E49" s="75" t="inlineStr">
+        <is>
+          <t>C, C2, C3</t>
+        </is>
+      </c>
+      <c r="F49" s="11" t="inlineStr">
+        <is>
+          <t>plus de phase condensée : B'c ≫ 1</t>
+        </is>
+      </c>
+      <c r="G49" s="15" t="inlineStr"/>
+      <c r="H49" s="15" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>À haute pression les mêmes régimes sont décalés vers des températures plus élevées (la sublimation est retardée, effet Clausius-Clapeyron), tandis que les réactions d'oxydation sont favorisées. La table B' est donc une SURFACE B'c(T_w, P), tracée comme un faisceau de 25 isobares de 10⁻³ à 10³ atm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>§7 — RÉPONSE MATÉRIAU (n'entre PAS dans le XML)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="35" t="inlineStr">
+        <is>
+          <t>couplage k = B'g / B'c</t>
+        </is>
+      </c>
+      <c r="C53" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="I53" s="12" t="inlineStr">
+        <is>
+          <t>aucun gaz de pyrolyse — le graphite est le seul matériau du classeur à k = 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" s="35" t="inlineStr">
+        <is>
+          <t>récession par unité de flux, B'c/ρ_c à 300 K [m³/kg]</t>
+        </is>
+      </c>
+      <c r="C54" s="41">
+        <f>C19*Constantes!$C$7/(2*Constantes!$C$9)/C20</f>
+        <v>4.857026857405357e-05</v>
+      </c>
+      <c r="I54" s="12" t="inlineStr">
+        <is>
+          <t>ṡ = B'c·ṁe/ρ_c</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>§8 — BLOC XML</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="29" t="inlineStr">
+        <is>
+          <t>&lt;mixture thermo_db="NASA-9"&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    &lt;species&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        N O NO N2 O2 C C2 C3 CN CO CO2 C(gr)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    &lt;/species&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    &lt;element_compositions default="air"&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        &lt;composition name="air"&gt;N:0.79, O:0.21&lt;/composition&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        &lt;composition name="pyro"&gt;C:1.0&lt;/composition&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    &lt;/element_compositions&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="29" t="inlineStr">
+        <is>
+          <t>&lt;/mixture&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="16" customHeight="1">
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>bprime -T 300:25:5000 -P &lt;P&gt; -b 0.0 -m carbon-air -bl air -py pyro</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="36">
+    <mergeCell ref="B62:I62"/>
+    <mergeCell ref="A56:I56"/>
+    <mergeCell ref="B59:I59"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="B15:H15"/>
+    <mergeCell ref="B31:I31"/>
+    <mergeCell ref="B27:I27"/>
+    <mergeCell ref="B58:I58"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="B26:H26"/>
+    <mergeCell ref="A33:I33"/>
+    <mergeCell ref="A5:I5"/>
+    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="B60:I60"/>
+    <mergeCell ref="B67:I67"/>
+    <mergeCell ref="A22:I22"/>
+    <mergeCell ref="B61:I61"/>
+    <mergeCell ref="B57:I57"/>
+    <mergeCell ref="A38:I38"/>
+    <mergeCell ref="A52:I52"/>
+    <mergeCell ref="B29:I29"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="B39:H39"/>
+    <mergeCell ref="A44:I44"/>
+    <mergeCell ref="B65:I65"/>
+    <mergeCell ref="B23:H23"/>
+    <mergeCell ref="B40:I40"/>
+    <mergeCell ref="B14:H14"/>
+    <mergeCell ref="B30:I30"/>
+    <mergeCell ref="A11:I11"/>
+    <mergeCell ref="B64:I64"/>
+    <mergeCell ref="B13:H13"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="B63:I63"/>
+    <mergeCell ref="B50:I50"/>
+    <mergeCell ref="B28:H28"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="000070C0"/>
@@ -2192,7 +3067,7 @@
           <t>ρ_char [kg/m³]</t>
         </is>
       </c>
-      <c r="C47" s="73">
+      <c r="C47" s="76">
         <f>C20</f>
         <v>2200.0</v>
       </c>
@@ -2318,7 +3193,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="007030A0"/>
@@ -2857,12 +3732,12 @@
           <t>air — valeur portée dans le XML</t>
         </is>
       </c>
-      <c r="C42" s="74" t="inlineStr">
+      <c r="C42" s="77" t="inlineStr">
         <is>
           <t>N : 0.79</t>
         </is>
       </c>
-      <c r="D42" s="74" t="inlineStr">
+      <c r="D42" s="77" t="inlineStr">
         <is>
           <t>O : 0.21</t>
         </is>
@@ -2908,7 +3783,7 @@
           <t>B'c attendu sur le plateau</t>
         </is>
       </c>
-      <c r="C47" s="71">
+      <c r="C47" s="74">
         <f>C21*$C$27/(2*Constantes!$C$9)</f>
         <v>0.2918571303790834</v>
       </c>
@@ -3005,7 +3880,7 @@
           <t>2100 K, 1 atm</t>
         </is>
       </c>
-      <c r="C53" s="72" t="inlineStr">
+      <c r="C53" s="75" t="inlineStr">
         <is>
           <t>SiC</t>
         </is>
@@ -3028,7 +3903,7 @@
           <t>2600 K, 1 atm</t>
         </is>
       </c>
-      <c r="C54" s="72" t="inlineStr">
+      <c r="C54" s="75" t="inlineStr">
         <is>
           <t>SiC + Si(L)</t>
         </is>
@@ -3051,7 +3926,7 @@
           <t>2500 K, 0.001 atm</t>
         </is>
       </c>
-      <c r="C55" s="72" t="inlineStr">
+      <c r="C55" s="75" t="inlineStr">
         <is>
           <t>C(gr) (résidu)</t>
         </is>
@@ -3117,17 +3992,17 @@
           <t>oxydation passive</t>
         </is>
       </c>
-      <c r="C60" s="72" t="inlineStr">
+      <c r="C60" s="75" t="inlineStr">
         <is>
           <t>300 – 1625</t>
         </is>
       </c>
-      <c r="D60" s="72" t="inlineStr">
+      <c r="D60" s="75" t="inlineStr">
         <is>
           <t>SiC + SiO2 + C(gr)</t>
         </is>
       </c>
-      <c r="E60" s="72" t="inlineStr">
+      <c r="E60" s="75" t="inlineStr">
         <is>
           <t>N2</t>
         </is>
@@ -3146,17 +4021,17 @@
           <t>transition passive → active</t>
         </is>
       </c>
-      <c r="C61" s="72" t="inlineStr">
+      <c r="C61" s="75" t="inlineStr">
         <is>
           <t>1650 – 1950</t>
         </is>
       </c>
-      <c r="D61" s="72" t="inlineStr">
+      <c r="D61" s="75" t="inlineStr">
         <is>
           <t>SiC + SiO2</t>
         </is>
       </c>
-      <c r="E61" s="72" t="inlineStr">
+      <c r="E61" s="75" t="inlineStr">
         <is>
           <t>N2, CO, SiO</t>
         </is>
@@ -3175,17 +4050,17 @@
           <t>oxydation active</t>
         </is>
       </c>
-      <c r="C62" s="72" t="inlineStr">
+      <c r="C62" s="75" t="inlineStr">
         <is>
           <t>1975 – 2200</t>
         </is>
       </c>
-      <c r="D62" s="72" t="inlineStr">
+      <c r="D62" s="75" t="inlineStr">
         <is>
           <t>SiC</t>
         </is>
       </c>
-      <c r="E62" s="72" t="inlineStr">
+      <c r="E62" s="75" t="inlineStr">
         <is>
           <t>N2, CO, SiO</t>
         </is>
@@ -3204,17 +4079,17 @@
           <t>oxydation + silicium liquide</t>
         </is>
       </c>
-      <c r="C63" s="72" t="inlineStr">
+      <c r="C63" s="75" t="inlineStr">
         <is>
           <t>2225 – 3000</t>
         </is>
       </c>
-      <c r="D63" s="72" t="inlineStr">
+      <c r="D63" s="75" t="inlineStr">
         <is>
           <t>SiC + Si(L)</t>
         </is>
       </c>
-      <c r="E63" s="72" t="inlineStr">
+      <c r="E63" s="75" t="inlineStr">
         <is>
           <t>N2, CO, SiO, Si, Si2C</t>
         </is>
@@ -3233,17 +4108,17 @@
           <t>sublimation</t>
         </is>
       </c>
-      <c r="C64" s="72" t="inlineStr">
+      <c r="C64" s="75" t="inlineStr">
         <is>
           <t>3025 – 3100</t>
         </is>
       </c>
-      <c r="D64" s="72" t="inlineStr">
+      <c r="D64" s="75" t="inlineStr">
         <is>
           <t>SiC</t>
         </is>
       </c>
-      <c r="E64" s="72" t="inlineStr">
+      <c r="E64" s="75" t="inlineStr">
         <is>
           <t>SiC2, Si2C, Si</t>
         </is>
@@ -3262,17 +4137,17 @@
           <t>sublimation totale</t>
         </is>
       </c>
-      <c r="C65" s="72" t="inlineStr">
+      <c r="C65" s="75" t="inlineStr">
         <is>
           <t>≥ 3125</t>
         </is>
       </c>
-      <c r="D65" s="72" t="inlineStr">
+      <c r="D65" s="75" t="inlineStr">
         <is>
           <t>gaz seul</t>
         </is>
       </c>
-      <c r="E65" s="72" t="inlineStr">
+      <c r="E65" s="75" t="inlineStr">
         <is>
           <t>Si, SiC2, Si2C</t>
         </is>
@@ -3494,7 +4369,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00C55A11"/>
@@ -3708,7 +4583,7 @@
           <t>M_Mo [g/mol]</t>
         </is>
       </c>
-      <c r="C19" s="75" t="n">
+      <c r="C19" s="71" t="n">
         <v>95.95999999999999</v>
       </c>
       <c r="I19" s="12" t="inlineStr">
@@ -3802,7 +4677,7 @@
           <t>B'c limite de diffusion (MoO3)</t>
         </is>
       </c>
-      <c r="C27" s="71">
+      <c r="C27" s="74">
         <f>C20*C19/(3*Constantes!$C$9)</f>
         <v>0.46565344824239585</v>
       </c>
@@ -3818,7 +4693,7 @@
           <t>B'c si l'oxyde gazeux était MoO2</t>
         </is>
       </c>
-      <c r="C28" s="71">
+      <c r="C28" s="74">
         <f>C20*C19/(2*Constantes!$C$9)</f>
         <v>0.6984801723635938</v>
       </c>
@@ -3924,7 +4799,7 @@
           <t>plateau de la table « surface nue »</t>
         </is>
       </c>
-      <c r="C37" s="76" t="n">
+      <c r="C37" s="78" t="n">
         <v>0.4657</v>
       </c>
       <c r="I37" s="12" t="inlineStr">
@@ -3955,7 +4830,7 @@
           <t>points instables (critère de force motrice)</t>
         </is>
       </c>
-      <c r="C39" s="77" t="n">
+      <c r="C39" s="79" t="n">
         <v>0</v>
       </c>
       <c r="I39" s="12" t="inlineStr">
@@ -3989,7 +4864,7 @@
       <c r="H42" s="6" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="B43" s="78" t="n">
+      <c r="B43" s="80" t="n">
         <v>0.001</v>
       </c>
       <c r="C43" s="40" t="n">
@@ -4002,7 +4877,7 @@
       <c r="H43" s="15" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="B44" s="78" t="n">
+      <c r="B44" s="80" t="n">
         <v>0.01</v>
       </c>
       <c r="C44" s="40" t="n">
@@ -4015,7 +4890,7 @@
       <c r="H44" s="15" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="B45" s="78" t="n">
+      <c r="B45" s="80" t="n">
         <v>0.1</v>
       </c>
       <c r="C45" s="40" t="n">
@@ -4028,7 +4903,7 @@
       <c r="H45" s="15" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="B46" s="78" t="n">
+      <c r="B46" s="80" t="n">
         <v>1</v>
       </c>
       <c r="C46" s="40" t="n">
@@ -4041,7 +4916,7 @@
       <c r="H46" s="15" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="B47" s="78" t="n">
+      <c r="B47" s="80" t="n">
         <v>10</v>
       </c>
       <c r="C47" s="40" t="n">
@@ -4054,7 +4929,7 @@
       <c r="H47" s="15" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="B48" s="78" t="n">
+      <c r="B48" s="80" t="n">
         <v>100</v>
       </c>
       <c r="C48" s="40" t="n">
@@ -4067,7 +4942,7 @@
       <c r="H48" s="15" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="B49" s="78" t="n">
+      <c r="B49" s="80" t="n">
         <v>1000</v>
       </c>
       <c r="C49" s="40" t="n">
@@ -16510,11 +17385,11 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="00404040"/>
+    <tabColor rgb="007F6000"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I67"/>
+  <dimension ref="A1:I122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4.5" customWidth="1" min="1" max="1"/>
@@ -16531,21 +17406,21 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Carbone graphite — ablateur non pyrolysant</t>
+          <t>Bois de chêne — ablateur pyrolysant à un seul constituant</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cas dégénéré : le solide EST le char, il n'y a pas de gaz de pyrolyse · sert de cas de référence physique aux autres onglets</t>
+          <t>Le cas le plus simple des ablateurs pyrolysants : TOUT le solide pyrolyse, sans résine ni renfort inerte — une seule fermeture élémentaire bois − char</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Fichier(s) XML : data/mixtures/carbon-air.xml</t>
+          <t>Fichier(s) XML : data/mixtures/oak-air.xml · oak-pyrogas.xml</t>
         </is>
       </c>
     </row>
@@ -16564,784 +17439,1950 @@
       </c>
       <c r="C6" s="30" t="inlineStr">
         <is>
-          <t>graphite pur (carbone massif)</t>
+          <t>bois de chêne massif (Quercus robur / Q. petraea), SEC, sans résine</t>
         </is>
       </c>
       <c r="I6" s="12" t="inlineStr">
         <is>
-          <t>carbon_bprime/bprime_carbon_physique.md</t>
+          <t>feuillu — à ne pas confondre avec le liège (Q. suber)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="35" t="inlineStr">
         <is>
-          <t>Renfort / résine</t>
+          <t>Constituants</t>
         </is>
       </c>
       <c r="C7" s="30" t="inlineStr">
         <is>
-          <t>sans objet — matériau monolithique</t>
+          <t>cellulose 43 / hémicelluloses 22 / lignine S+G 25 / ellagitanins 8 %</t>
         </is>
       </c>
       <c r="I7" s="12" t="inlineStr">
         <is>
-          <t>aucune pyrolyse interne</t>
+          <t>IL PYROLYSE ENTIÈREMENT : 80 % du bois part en gaz</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="35" t="inlineStr">
         <is>
-          <t>Système chimique</t>
+          <t>Rendement en char</t>
         </is>
       </c>
       <c r="C8" s="30" t="inlineStr">
         <is>
-          <t>C-N-O : 5 espèces d'air + 3 formes gazeuses du carbone + CO, CO2, CN + C(gr)</t>
+          <t>20 % en masse</t>
         </is>
       </c>
       <c r="I8" s="12" t="inlineStr">
         <is>
-          <t>12 espèces au total</t>
+          <t>donnée de l'énoncé</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="35" t="inlineStr">
         <is>
+          <t>Unité de répétition globale</t>
+        </is>
+      </c>
+      <c r="C9" s="30" t="inlineStr">
+        <is>
+          <t>C6H8.7O3.95 — soit CH1.45O0.66 par atome de carbone</t>
+        </is>
+      </c>
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>calculée à l'étape 5 du §3</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="35" t="inlineStr">
+        <is>
+          <t>Sources</t>
+        </is>
+      </c>
+      <c r="C10" s="30" t="inlineStr">
+        <is>
+          <t>oak_bprime/mise_en_donnees_chene.md · oak_pyrolysis_data.py</t>
+        </is>
+      </c>
+      <c r="I10" s="12" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="B11" s="35" t="inlineStr">
+        <is>
           <t>Compositions du XML</t>
         </is>
       </c>
-      <c r="C9" s="30" t="inlineStr">
-        <is>
-          <t>air (-bl) · pyro = C:1.0 (-py, et définit le char)</t>
-        </is>
-      </c>
-      <c r="I9" s="12" t="inlineStr"/>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="C11" s="30" t="inlineStr">
+        <is>
+          <t>air (-bl) · oak_pyro (-py) · oak_char (-char, -char-elem C)</t>
+        </is>
+      </c>
+      <c r="I11" s="12" t="inlineStr"/>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>§1 — HYPOTHÈSES</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="26" customHeight="1">
-      <c r="A12" s="20" t="inlineStr">
-        <is>
-          <t>H1</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Pas de pyrolyse interne : B'g = 0.</t>
-        </is>
-      </c>
-      <c r="I12" s="12" t="inlineStr">
-        <is>
-          <t>Il n'y a pas de résine à décomposer. Toute la masse injectée vient de la surface, d'où le nom de « cas dégénéré ».</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="26" customHeight="1">
-      <c r="A13" s="20" t="inlineStr">
-        <is>
-          <t>H2</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Le char est le matériau lui-même : carbone pur, C:1.0.</t>
-        </is>
-      </c>
-      <c r="I13" s="12" t="inlineStr">
-        <is>
-          <t>Aucune fermeture élémentaire à faire — c'est la seule mise en données du dépôt où la composition ne se CALCULE pas.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="26" customHeight="1">
       <c r="A14" s="20" t="inlineStr">
         <is>
-          <t>H3</t>
+          <t>H1</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Équilibre thermochimique à la paroi, char infini.</t>
+          <t>UN SEUL CONSTITUANT, QUI PYROLYSE ENTIÈREMENT. Gaz = bois − char, sans mélange de gaz.</t>
         </is>
       </c>
       <c r="I14" s="12" t="inlineStr">
         <is>
-          <t>Le solveur ajoute δ = max(200, 100·B'g) de carbone élémentaire à la composition du bord de couche limite avant de normaliser, puis calcule l'équilibre multiphase.</t>
+          <t>Route C (fermeture élémentaire), mais partant d'une ANALYSE élémentaire et non d'un motif idéalisé. Pas de rapport renfort/résine : contrairement au liège, rien d'autre que le rendement en char ne pondère le gaz.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="26" customHeight="1">
       <c r="A15" s="20" t="inlineStr">
         <is>
+          <t>H2</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Bois SEC. L'humidité (8-12 % dans un bois stabilisé à l'air) n'est pas comptée.</t>
+        </is>
+      </c>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>Elle partirait intégralement en vapeur d'eau, donc dans le gaz : le §6 chiffre la variante (gaz plus riche en H et O, k plus grand).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="26" customHeight="1">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>H3</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Analyse élémentaire du chêne retenue : C 50.0 / H 6.1 / O 43.9 % masse (littérature, sec sans cendres).</t>
+        </is>
+      </c>
+      <c r="I16" s="12" t="inlineStr">
+        <is>
+          <t>PROVENANCE À CONFIRMER : valeurs usuelles pour le bois de chêne, non vérifiées sur une source primaire accessible. Le contrôle biochimique du §5 les retrouve à 0.4 point près. L'azote (0.1-0.3 %) est négligé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="26" customHeight="1">
+      <c r="A17" s="20" t="inlineStr">
+        <is>
           <t>H4</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>C(gr) est indispensable dans la liste d'espèces.</t>
-        </is>
-      </c>
-      <c r="I15" s="12" t="inlineStr">
-        <is>
-          <t>Sans phase condensée, C3 gazeux domine dès 300 K, Y_w,C → 1 et B'c ≈ 200 — non physique. C'est le contrôle du §5, valable pour TOUS les onglets carbonés.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Rendement en char : 20 % en masse du bois sec.</t>
+        </is>
+      </c>
+      <c r="I17" s="12" t="inlineStr">
+        <is>
+          <t>Donnée de l'énoncé. C'est LE paramètre du calcul : il fixe à la fois le carbone du gaz et le couplage k (§6). Le contrôle par additivité des constituants donne 22 %.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="26" customHeight="1">
+      <c r="A18" s="20" t="inlineStr">
+        <is>
+          <t>H5</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Le bois carbonise vers du carbone pur ⇒ char C:1.0.</t>
+        </is>
+      </c>
+      <c r="I18" s="12" t="inlineStr">
+        <is>
+          <t>Un charbon de bois réel retient H et O (d'autant plus que la carbonisation est froide) : le §5 chiffre la variante — et rappelle qu'il faut alors RETIRER ces atomes du gaz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="26" customHeight="1">
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t>H6</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Le couplage stationnaire se calcule sur les MASSES : k = (1 − y)/y = 4.0.</t>
+        </is>
+      </c>
+      <c r="I19" s="12" t="inlineStr">
+        <is>
+          <t>L'identité k = (ρ_v − ρ_c)/ρ_c suppose un volume constant ; le bois se rétracte en carbonisant (retrait volumique typiquement 30-50 %).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>§2 — DONNÉES D'ENTRÉE</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="35" t="inlineStr">
-        <is>
-          <t>bord de couche limite</t>
-        </is>
-      </c>
-      <c r="C18" s="30" t="inlineStr">
-        <is>
-          <t>air : N:0.79, O:0.21 (molaire)</t>
-        </is>
-      </c>
-      <c r="I18" s="12" t="inlineStr">
-        <is>
-          <t>cf. onglet Constantes §2</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="35" t="inlineStr">
-        <is>
-          <t>fraction massique d'oxygène de l'air</t>
-        </is>
-      </c>
-      <c r="C19" s="50">
-        <f>Constantes!D19</f>
-        <v>0.23290921795842306</v>
-      </c>
-      <c r="I19" s="12" t="inlineStr">
-        <is>
-          <t>y_O calculé au §2 de l'onglet Constantes</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="35" t="inlineStr">
-        <is>
-          <t>masse volumique du graphite [kg/m³]</t>
-        </is>
-      </c>
-      <c r="C20" s="30" t="n">
-        <v>1800</v>
-      </c>
-      <c r="I20" s="12" t="inlineStr">
-        <is>
-          <t>ordre de grandeur (1600-2200 selon la qualité) — n'entre que dans la récession</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="20" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="B22" s="20" t="inlineStr">
+        <is>
+          <t>Analyse élémentaire du chêne — valeurs de littérature (RETENUES)</t>
+        </is>
+      </c>
+      <c r="I22" s="27" t="inlineStr">
+        <is>
+          <t>% masse, sec sans cendres</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="6" t="inlineStr"/>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>Somme</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr"/>
+      <c r="H23" s="6" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>chêne [% masse]</t>
+        </is>
+      </c>
+      <c r="C24" s="69" t="n">
+        <v>50</v>
+      </c>
+      <c r="D24" s="69" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="E24" s="69" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="F24" s="9">
+        <f>SUM(C24:E24)</f>
+        <v>100.0</v>
+      </c>
+      <c r="G24" s="15" t="inlineStr"/>
+      <c r="H24" s="15" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>La somme vaut 100 % : l'étape 1 renormalise quand même, pour qu'une analyse mesurée (qui ne somme jamais exactement à 100) puisse être collée ici telle quelle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="20" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="B27" s="20" t="inlineStr">
+        <is>
+          <t>Constituants biochimiques du chêne et leurs unités de répétition (sert au contrôle du §5)</t>
+        </is>
+      </c>
+      <c r="I27" s="27" t="inlineStr">
+        <is>
+          <t>M_i = Σ_E ν_E,i · M_E</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>Constituant — unité de répétition</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>% masse</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>ν_C</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>ν_H</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>ν_O</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>M [g/mol]</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>rendement en char</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>cellulose — C6H10O5 (anhydroglucose)</t>
+        </is>
+      </c>
+      <c r="C29" s="36" t="n">
+        <v>43</v>
+      </c>
+      <c r="D29" s="40" t="n">
+        <v>6</v>
+      </c>
+      <c r="E29" s="40" t="n">
+        <v>10</v>
+      </c>
+      <c r="F29" s="40" t="n">
+        <v>5</v>
+      </c>
+      <c r="G29" s="9">
+        <f>D29*Constantes!$C$7+E29*Constantes!$C$8+F29*Constantes!$C$9</f>
+        <v>162.14100000000002</v>
+      </c>
+      <c r="H29" s="36" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>hémicelluloses — C5H8O4 (anhydroxylose, glucuronoxylane)</t>
+        </is>
+      </c>
+      <c r="C30" s="36" t="n">
+        <v>22</v>
+      </c>
+      <c r="D30" s="40" t="n">
+        <v>5</v>
+      </c>
+      <c r="E30" s="40" t="n">
+        <v>8</v>
+      </c>
+      <c r="F30" s="40" t="n">
+        <v>4</v>
+      </c>
+      <c r="G30" s="9">
+        <f>D30*Constantes!$C$7+E30*Constantes!$C$8+F30*Constantes!$C$9</f>
+        <v>132.115</v>
+      </c>
+      <c r="H30" s="36" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>lignine S — C11H14O4 (alcool sinapylique)</t>
+        </is>
+      </c>
+      <c r="C31" s="36" t="n">
+        <v>16</v>
+      </c>
+      <c r="D31" s="40" t="n">
+        <v>11</v>
+      </c>
+      <c r="E31" s="40" t="n">
+        <v>14</v>
+      </c>
+      <c r="F31" s="40" t="n">
+        <v>4</v>
+      </c>
+      <c r="G31" s="9">
+        <f>D31*Constantes!$C$7+E31*Constantes!$C$8+F31*Constantes!$C$9</f>
+        <v>210.22899999999998</v>
+      </c>
+      <c r="H31" s="36" t="n">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>lignine G — C10H12O3 (alcool coniférylique)</t>
+        </is>
+      </c>
+      <c r="C32" s="36" t="n">
+        <v>9</v>
+      </c>
+      <c r="D32" s="40" t="n">
+        <v>10</v>
+      </c>
+      <c r="E32" s="40" t="n">
+        <v>12</v>
+      </c>
+      <c r="F32" s="40" t="n">
+        <v>3</v>
+      </c>
+      <c r="G32" s="9">
+        <f>D32*Constantes!$C$7+E32*Constantes!$C$8+F32*Constantes!$C$9</f>
+        <v>180.20299999999997</v>
+      </c>
+      <c r="H32" s="36" t="n">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>tanins — C41H26O26 (vescalagine, ellagitanin)</t>
+        </is>
+      </c>
+      <c r="C33" s="36" t="n">
+        <v>8</v>
+      </c>
+      <c r="D33" s="40" t="n">
+        <v>41</v>
+      </c>
+      <c r="E33" s="40" t="n">
+        <v>26</v>
+      </c>
+      <c r="F33" s="40" t="n">
+        <v>26</v>
+      </c>
+      <c r="G33" s="9">
+        <f>D33*Constantes!$C$7+E33*Constantes!$C$8+F33*Constantes!$C$9</f>
+        <v>934.633</v>
+      </c>
+      <c r="H33" s="36" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>SOMME des parts</t>
+        </is>
+      </c>
+      <c r="C34" s="9">
+        <f>SUM(C29:C33)</f>
+        <v>98.0</v>
+      </c>
+      <c r="D34" s="15" t="inlineStr"/>
+      <c r="E34" s="15" t="inlineStr"/>
+      <c r="F34" s="15" t="inlineStr"/>
+      <c r="G34" s="15" t="inlineStr"/>
+      <c r="H34" s="15" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>Les parts somment à 98 % : le complément (cendres ~0.4 %, groupes acétyles des hémicelluloses, extractibles mineurs) n'est pas de la matière C/H/O identifiée. On renormalise sur les 98 % déclarés. La lignine de feuillu est répartie en 16 % S + 9 % G en masse, soit S/G = 1.52 en moles. Les rendements en char par constituant (dernière colonne) sont des ordres de grandeur d'ATG lente sous inerte — ils servent au contrôle B du §5, pas au calcul du XML.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="35" t="inlineStr">
+        <is>
+          <t>rendement en char du bois sec</t>
+        </is>
+      </c>
+      <c r="C37" s="71" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I37" s="12" t="inlineStr">
+        <is>
+          <t>hypothèse H4 — donnée de l'énoncé</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="35" t="inlineStr">
+        <is>
+          <t>ρ vierge [kg/m³]</t>
+        </is>
+      </c>
+      <c r="C38" s="30" t="n">
+        <v>700</v>
+      </c>
+      <c r="I38" s="12" t="inlineStr">
+        <is>
+          <t>chêne sec, ordre de grandeur 650-750 kg/m³ — n'entre PAS dans le XML</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="35" t="inlineStr">
+        <is>
+          <t>V_char / V_vierge (retrait volumique)</t>
+        </is>
+      </c>
+      <c r="C39" s="72" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="I39" s="12" t="inlineStr">
+        <is>
+          <t>HYPOTHÈSE, non mesurée ici — à remplacer par une mesure (§7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="4" t="inlineStr">
         <is>
           <t>§3 — CALCUL PAS À PAS</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="20" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="20" t="inlineStr">
         <is>
           <t>&gt;</t>
         </is>
       </c>
-      <c r="B23" s="20" t="inlineStr">
-        <is>
-          <t>Étape 1 — composition élémentaire du char : directe</t>
-        </is>
-      </c>
-      <c r="I23" s="27" t="inlineStr">
-        <is>
-          <t>le solide est du carbone pur ⇒ x_C = 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="6" t="inlineStr"/>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="B42" s="20" t="inlineStr">
+        <is>
+          <t>Étape 1 — renormaliser l'analyse élémentaire du chêne à 100 %</t>
+        </is>
+      </c>
+      <c r="I42" s="27" t="inlineStr">
+        <is>
+          <t>w_E = w_E,brut / Σ w_j,brut</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="6" t="inlineStr"/>
+      <c r="C43" s="6" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="inlineStr">
+      <c r="D43" s="6" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="F24" s="6" t="inlineStr">
+      <c r="F43" s="6" t="inlineStr">
         <is>
           <t>Somme</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr"/>
-      <c r="H24" s="6" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>char (= le matériau)</t>
-        </is>
-      </c>
-      <c r="C25" s="44" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" s="24">
-        <f>SUM(C25:E25)</f>
-        <v>1.0</v>
-      </c>
-      <c r="G25" s="15" t="inlineStr"/>
-      <c r="H25" s="15" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="20" t="inlineStr">
+      <c r="G43" s="6" t="inlineStr"/>
+      <c r="H43" s="6" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>chêne renormalisé [% masse]</t>
+        </is>
+      </c>
+      <c r="C44" s="9">
+        <f>C24/$F$24*100</f>
+        <v>50.0</v>
+      </c>
+      <c r="D44" s="9">
+        <f>D24/$F$24*100</f>
+        <v>6.1</v>
+      </c>
+      <c r="E44" s="9">
+        <f>E24/$F$24*100</f>
+        <v>43.9</v>
+      </c>
+      <c r="F44" s="9">
+        <f>SUM(C44:E44)</f>
+        <v>100.0</v>
+      </c>
+      <c r="G44" s="15" t="inlineStr"/>
+      <c r="H44" s="15" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="20" t="inlineStr">
         <is>
           <t>&gt;</t>
         </is>
       </c>
-      <c r="B26" s="20" t="inlineStr">
-        <is>
-          <t>Étape 2 — gaz de pyrolyse : il n'y en a pas</t>
-        </is>
-      </c>
-      <c r="I26" s="27" t="inlineStr">
-        <is>
-          <t>B'g = 0 dans toutes les commandes bprime de ce matériau</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="30" customHeight="1">
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>La composition nommée `pyro` du XML vaut néanmoins C:1.0. Ce n'est pas une incohérence : elle sert d'argument à `-py` (le parseur exige une composition valide) et définit le char. Comme elle est appelée avec -b 0.0, elle ne contribue à rien.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="20" t="inlineStr">
-        <is>
-          <t>&gt;</t>
-        </is>
-      </c>
-      <c r="B28" s="20" t="inlineStr">
-        <is>
-          <t>Étape 3 — le bilan de surface se réduit à une expression fermée</t>
-        </is>
-      </c>
-      <c r="I28" s="27" t="inlineStr">
-        <is>
-          <t>B'c = [Y_e,C + B'g·Y_g,C − Y_w,C(1+B'g)] / (Y_w,C − Y_c,C)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="16" customHeight="1">
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>Avec Y_c,C = 1 (char de carbone pur), Y_e,C = 0 (l'air ne contient pas de carbone) et B'g = 0, il ne reste que :</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="B30" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   B'c = − Y_w,C / (Y_w,C − 1) = Y_w,C / (1 − Y_w,C)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>La seule inconnue est Y_w,C, la fraction massique de carbone dans le gaz d'équilibre à la paroi — c'est elle que le solveur multiphase calcule à (T_w, P).</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>§4 — RÉSULTAT : CE QUI ENTRE DANS LE XML</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="6" t="inlineStr">
-        <is>
-          <t>Composition élémentaire (fractions molaires)</t>
-        </is>
-      </c>
-      <c r="C34" s="6" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D34" s="6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E34" s="6" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="inlineStr">
-        <is>
-          <t>Somme</t>
-        </is>
-      </c>
-      <c r="G34" s="6" t="inlineStr"/>
-      <c r="H34" s="6" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="B35" s="7" t="inlineStr">
-        <is>
-          <t>pyro / char — valeur portée dans le XML</t>
-        </is>
-      </c>
-      <c r="C35" s="44" t="n">
-        <v>1</v>
-      </c>
-      <c r="D35" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E35" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F35" s="15" t="inlineStr"/>
-      <c r="G35" s="15" t="inlineStr"/>
-      <c r="H35" s="15" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="B36" s="7" t="inlineStr">
-        <is>
-          <t>air — valeur portée dans le XML</t>
-        </is>
-      </c>
-      <c r="C36" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D36" s="44" t="n">
-        <v>0.79</v>
-      </c>
-      <c r="E36" s="44" t="n">
-        <v>0.21</v>
-      </c>
-      <c r="F36" s="24">
-        <f>D36+E36</f>
-        <v>1.0</v>
-      </c>
-      <c r="G36" s="15" t="inlineStr"/>
-      <c r="H36" s="15" t="inlineStr"/>
-    </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>§5 — CONTRÔLES ET VALIDATION CROISÉE</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="20" t="inlineStr">
-        <is>
-          <t>&gt;</t>
-        </is>
-      </c>
-      <c r="B39" s="20" t="inlineStr">
-        <is>
-          <t>Contrôle de recette valable pour TOUS les matériaux carbonés du dépôt</t>
-        </is>
-      </c>
-      <c r="I39" s="27" t="inlineStr">
-        <is>
-          <t>à 300 K, B'g = 0 : régime d'oxydation basse température, C(gr) + O2 → CO2</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="30" customHeight="1">
-      <c r="B40" s="5" t="inlineStr">
-        <is>
-          <t>À 300 K tout l'oxygène de l'air est consommé en CO2. Chaque O2 (2 atomes d'oxygène) emporte un atome de carbone : la masse de carbone ablatée par unité de masse d'air vaut donc y_O · M_C / (2·M_O). Ce nombre ne dépend PAS de la pression.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="B41" s="35" t="inlineStr">
-        <is>
-          <t>B'c attendu à 300 K, 1 atm</t>
-        </is>
-      </c>
-      <c r="C41" s="71">
-        <f>C19*Constantes!$C$7/(2*Constantes!$C$9)</f>
-        <v>0.08742648343329643</v>
-      </c>
-      <c r="I41" s="12" t="inlineStr">
-        <is>
-          <t>attendu 0.0874 — valeur obtenue par bprime sur carbon-air, cork-air, tacot-air…</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="B42" s="35" t="inlineStr">
-        <is>
-          <t>B'c obtenu si C(gr) manque dans &lt;species&gt;</t>
-        </is>
-      </c>
-      <c r="C42" s="31" t="inlineStr">
-        <is>
-          <t>≈ 200</t>
-        </is>
-      </c>
-      <c r="I42" s="12" t="inlineStr">
-        <is>
-          <t>signature sans ambiguïté d'une liste d'espèces incomplète : Y_w,C → 1 et B'c sature sur son plafond interne</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>§6 — SENSIBILITÉ — régimes physiques (à 1 atm)</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="B45" s="6" t="inlineStr">
-        <is>
-          <t>Régime</t>
-        </is>
-      </c>
-      <c r="C45" s="6" t="inlineStr">
-        <is>
-          <t>T_w [K]</t>
-        </is>
-      </c>
-      <c r="D45" s="6" t="inlineStr">
-        <is>
-          <t>Phase stable</t>
-        </is>
-      </c>
-      <c r="E45" s="6" t="inlineStr">
-        <is>
-          <t>Espèce gazeuse dominante</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="inlineStr">
-        <is>
-          <t>Mécanisme</t>
-        </is>
-      </c>
-      <c r="G45" s="6" t="inlineStr"/>
-      <c r="H45" s="6" t="inlineStr"/>
+      <c r="B45" s="20" t="inlineStr">
+        <is>
+          <t>Étape 2 — bilan de masse sur 100 g de bois sec</t>
+        </is>
+      </c>
+      <c r="I45" s="27" t="inlineStr">
+        <is>
+          <t>m_char = 100 · y ;  m_gaz = 100 · (1 − y)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
-      <c r="B46" s="7" t="inlineStr">
-        <is>
-          <t>faible ablation</t>
-        </is>
-      </c>
-      <c r="C46" s="72" t="inlineStr">
-        <is>
-          <t>300 – 700</t>
-        </is>
-      </c>
-      <c r="D46" s="72" t="inlineStr">
-        <is>
-          <t>C(gr)</t>
-        </is>
-      </c>
-      <c r="E46" s="72" t="inlineStr">
-        <is>
-          <t>CO2, O2, N2</t>
-        </is>
-      </c>
-      <c r="F46" s="11" t="inlineStr">
-        <is>
-          <t>C(gr) + O2 → CO2</t>
-        </is>
-      </c>
-      <c r="G46" s="15" t="inlineStr"/>
-      <c r="H46" s="15" t="inlineStr"/>
+      <c r="B46" s="6" t="inlineStr"/>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>masse [g]</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>rendement char</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>char [g]</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>gaz [g]</t>
+        </is>
+      </c>
+      <c r="G46" s="6" t="inlineStr"/>
+      <c r="H46" s="6" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>oxydation active</t>
-        </is>
-      </c>
-      <c r="C47" s="72" t="inlineStr">
-        <is>
-          <t>700 – 3500</t>
-        </is>
-      </c>
-      <c r="D47" s="72" t="inlineStr">
-        <is>
-          <t>C(gr)</t>
-        </is>
-      </c>
-      <c r="E47" s="72" t="inlineStr">
-        <is>
-          <t>CO, N2, CN</t>
-        </is>
-      </c>
-      <c r="F47" s="11" t="inlineStr">
-        <is>
-          <t>C(gr) + O → CO ; Boudouard C(gr) + CO2 → 2 CO</t>
-        </is>
+          <t>bois sec</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="D47" s="24">
+        <f>$C$37</f>
+        <v>0.2</v>
+      </c>
+      <c r="E47" s="9">
+        <f>C47*D47</f>
+        <v>20.0</v>
+      </c>
+      <c r="F47" s="9">
+        <f>C47-E47</f>
+        <v>80.0</v>
       </c>
       <c r="G47" s="15" t="inlineStr"/>
       <c r="H47" s="15" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="B48" s="7" t="inlineStr">
-        <is>
-          <t>sublimation</t>
-        </is>
-      </c>
-      <c r="C48" s="72" t="inlineStr">
-        <is>
-          <t>3500 – 4000</t>
-        </is>
-      </c>
-      <c r="D48" s="72" t="inlineStr">
-        <is>
-          <t>C(gr) + gaz</t>
-        </is>
-      </c>
-      <c r="E48" s="72" t="inlineStr">
-        <is>
-          <t>CO, CN, C3</t>
-        </is>
-      </c>
-      <c r="F48" s="11" t="inlineStr">
-        <is>
-          <t>C(gr) ⇌ C, C2, C3</t>
-        </is>
-      </c>
-      <c r="G48" s="15" t="inlineStr"/>
-      <c r="H48" s="15" t="inlineStr"/>
+      <c r="A48" s="20" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="B48" s="20" t="inlineStr">
+        <is>
+          <t>Étape 3 — fermeture élémentaire : aucun atome n'est créé</t>
+        </is>
+      </c>
+      <c r="I48" s="27" t="inlineStr">
+        <is>
+          <t>n_E(gaz) = n_E(bois) − n_E(char)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="B49" s="7" t="inlineStr">
-        <is>
-          <t>sublimation totale</t>
-        </is>
-      </c>
-      <c r="C49" s="72" t="inlineStr">
-        <is>
-          <t>&gt; 4000</t>
-        </is>
-      </c>
-      <c r="D49" s="72" t="inlineStr">
-        <is>
-          <t>gaz seul</t>
-        </is>
-      </c>
-      <c r="E49" s="72" t="inlineStr">
-        <is>
-          <t>C, C2, C3</t>
-        </is>
-      </c>
-      <c r="F49" s="11" t="inlineStr">
-        <is>
-          <t>plus de phase condensée : B'c ≫ 1</t>
-        </is>
-      </c>
-      <c r="G49" s="15" t="inlineStr"/>
-      <c r="H49" s="15" t="inlineStr"/>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>Moles d'atomes</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="E49" s="6" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t>Somme</t>
+        </is>
+      </c>
+      <c r="G49" s="6" t="inlineStr"/>
+      <c r="H49" s="6" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="B50" s="12" t="inlineStr">
-        <is>
-          <t>À haute pression les mêmes régimes sont décalés vers des températures plus élevées (la sublimation est retardée, effet Clausius-Clapeyron), tandis que les réactions d'oxydation sont favorisées. La table B' est donc une SURFACE B'c(T_w, P), tracée comme un faisceau de 25 isobares de 10⁻³ à 10³ atm.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="4" t="inlineStr">
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>bois — atomes du solide vierge</t>
+        </is>
+      </c>
+      <c r="C50" s="26">
+        <f>$C$47*C44/100/Constantes!$C$7</f>
+        <v>4.162850720173175</v>
+      </c>
+      <c r="D50" s="26">
+        <f>$C$47*D44/100/Constantes!$C$8</f>
+        <v>6.051587301587301</v>
+      </c>
+      <c r="E50" s="26">
+        <f>$C$47*E44/100/Constantes!$C$9</f>
+        <v>2.743921495093443</v>
+      </c>
+      <c r="F50" s="26">
+        <f>SUM(C50:E50)</f>
+        <v>12.958359516853918</v>
+      </c>
+      <c r="G50" s="15" t="inlineStr"/>
+      <c r="H50" s="15" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>bois — atomes du char (C pur)</t>
+        </is>
+      </c>
+      <c r="C51" s="26">
+        <f>$E$47/Constantes!$C$7</f>
+        <v>1.6651402880692698</v>
+      </c>
+      <c r="D51" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" s="26">
+        <f>SUM(C51:E51)</f>
+        <v>1.6651402880692698</v>
+      </c>
+      <c r="G51" s="15" t="inlineStr"/>
+      <c r="H51" s="15" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="B52" s="13" t="inlineStr">
+        <is>
+          <t>GAZ = bois − char</t>
+        </is>
+      </c>
+      <c r="C52" s="26">
+        <f>C50-C51</f>
+        <v>2.497710432103905</v>
+      </c>
+      <c r="D52" s="26">
+        <f>D50-D51</f>
+        <v>6.051587301587301</v>
+      </c>
+      <c r="E52" s="26">
+        <f>E50-E51</f>
+        <v>2.743921495093443</v>
+      </c>
+      <c r="F52" s="26">
+        <f>SUM(C52:E52)</f>
+        <v>11.29321922878465</v>
+      </c>
+      <c r="G52" s="15" t="inlineStr"/>
+      <c r="H52" s="15" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="B53" s="12" t="inlineStr">
+        <is>
+          <t>Le char ne prend que du carbone : tout l'hydrogène et tout l'oxygène du bois passent dans le gaz. Le char emporte 1.665 des 4.163 moles de carbone, soit 40 % du carbone du bois.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="20" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="B54" s="20" t="inlineStr">
+        <is>
+          <t>Étape 4 — normaliser</t>
+        </is>
+      </c>
+      <c r="I54" s="27" t="inlineStr">
+        <is>
+          <t>x_E = n_E / Σ n_j ;  y_E = x_E·M_E / Σ x_j·M_j</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="6" t="inlineStr"/>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F55" s="6" t="inlineStr">
+        <is>
+          <t>Somme</t>
+        </is>
+      </c>
+      <c r="G55" s="6" t="inlineStr">
+        <is>
+          <t>M par atome [g/mol]</t>
+        </is>
+      </c>
+      <c r="H55" s="6" t="inlineStr">
+        <is>
+          <t>H/O</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>x_E (fraction molaire élémentaire)</t>
+        </is>
+      </c>
+      <c r="C56" s="26">
+        <f>C52/$F$52</f>
+        <v>0.2211690379424878</v>
+      </c>
+      <c r="D56" s="26">
+        <f>D52/$F$52</f>
+        <v>0.5358602519787052</v>
+      </c>
+      <c r="E56" s="26">
+        <f>E52/$F$52</f>
+        <v>0.24297071007880694</v>
+      </c>
+      <c r="F56" s="24">
+        <f>SUM(C56:E56)</f>
+        <v>1.0</v>
+      </c>
+      <c r="G56" s="24">
+        <f>C56*Constantes!$C$7+D56*Constantes!$C$8+E56*Constantes!$C$9</f>
+        <v>7.0838968392725885</v>
+      </c>
+      <c r="H56" s="24">
+        <f>D56/E56</f>
+        <v>2.2054520555374775</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>y_E (fraction massique élémentaire)</t>
+        </is>
+      </c>
+      <c r="C57" s="24">
+        <f>C56*Constantes!$C$7/$G$56</f>
+        <v>0.37500000000000006</v>
+      </c>
+      <c r="D57" s="24">
+        <f>D56*Constantes!$C$8/$G$56</f>
+        <v>0.07625</v>
+      </c>
+      <c r="E57" s="24">
+        <f>E56*Constantes!$C$9/$G$56</f>
+        <v>0.54875</v>
+      </c>
+      <c r="F57" s="24">
+        <f>SUM(C57:E57)</f>
+        <v>1.0</v>
+      </c>
+      <c r="G57" s="15" t="inlineStr"/>
+      <c r="H57" s="15" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="B58" s="12" t="inlineStr">
+        <is>
+          <t>H/O = 2.2 : trois fois plus bas que les phénoliques (5.9-6.8) et deux fois plus bas que le liège (4.9). C'est le gaz le plus OXYGÉNÉ du dépôt — le bois est pour les deux tiers des polysaccharides, eux-mêmes à H/O = 2. Plus d'oxygène dans le gaz de pyrolyse, c'est plus d'oxydant disponible à la paroi pour le char.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="20" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="B59" s="20" t="inlineStr">
+        <is>
+          <t>Étape 5 — unité de répétition globale du bois (ramenée à 6 atomes de carbone)</t>
+        </is>
+      </c>
+      <c r="I59" s="27" t="inlineStr">
+        <is>
+          <t>ν_E = 6 · (w_E/M_E) / (w_C/M_C)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="6" t="inlineStr"/>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>ν_C</t>
+        </is>
+      </c>
+      <c r="D60" s="6" t="inlineStr">
+        <is>
+          <t>ν_H</t>
+        </is>
+      </c>
+      <c r="E60" s="6" t="inlineStr">
+        <is>
+          <t>ν_O</t>
+        </is>
+      </c>
+      <c r="F60" s="6" t="inlineStr">
+        <is>
+          <t>M [g/mol]</t>
+        </is>
+      </c>
+      <c r="G60" s="6" t="inlineStr">
+        <is>
+          <t>H/C</t>
+        </is>
+      </c>
+      <c r="H60" s="6" t="inlineStr">
+        <is>
+          <t>O/C</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>bois de chêne — C6HxOy</t>
+        </is>
+      </c>
+      <c r="C61" s="73" t="n">
+        <v>6</v>
+      </c>
+      <c r="D61" s="9">
+        <f>6*(D44/Constantes!$C$8)/(C44/Constantes!$C$7)</f>
+        <v>8.72227380952381</v>
+      </c>
+      <c r="E61" s="9">
+        <f>6*(E44/Constantes!$C$9)/(C44/Constantes!$C$7)</f>
+        <v>3.9548689293080814</v>
+      </c>
+      <c r="F61" s="49">
+        <f>C61*Constantes!$C$7+D61*Constantes!$C$8+E61*Constantes!$C$9</f>
+        <v>144.132</v>
+      </c>
+      <c r="G61" s="24">
+        <f>D61/C61</f>
+        <v>1.4537123015873015</v>
+      </c>
+      <c r="H61" s="24">
+        <f>E61/C61</f>
+        <v>0.6591448215513469</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="12" t="inlineStr">
+        <is>
+          <t>Attendu C6H8.72O3.95 (M = 144.1 g/mol), soit CH1.45O0.66 : l'anhydroglucose C6H10O5 (cellulose) « enrichi en carbone » par la lignine. Cette unité n'entre pas dans le XML — c'est la même information que l'analyse élémentaire, écrite en motif.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="18" customHeight="1">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>§4 — RÉSULTAT : CE QUI ENTRE DANS LE XML</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>Composition élémentaire (fractions molaires)</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D65" s="6" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="E65" s="6" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F65" s="6" t="inlineStr">
+        <is>
+          <t>Somme</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="7" t="inlineStr">
+        <is>
+          <t>calcul — chaîne complète ci-dessus</t>
+        </is>
+      </c>
+      <c r="C66" s="26">
+        <f>C56</f>
+        <v>0.2211690379424878</v>
+      </c>
+      <c r="D66" s="26">
+        <f>D56</f>
+        <v>0.5358602519787052</v>
+      </c>
+      <c r="E66" s="26">
+        <f>E56</f>
+        <v>0.24297071007880694</v>
+      </c>
+      <c r="F66" s="24">
+        <f>SUM(C66:E66)</f>
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>valeur portée dans le XML (oak_pyro)</t>
+        </is>
+      </c>
+      <c r="C67" s="42" t="n">
+        <v>0.221</v>
+      </c>
+      <c r="D67" s="42" t="n">
+        <v>0.536</v>
+      </c>
+      <c r="E67" s="42" t="n">
+        <v>0.243</v>
+      </c>
+      <c r="F67" s="24">
+        <f>SUM(C67:E67)</f>
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>écart relatif |calcul − XML| / XML</t>
+        </is>
+      </c>
+      <c r="C68" s="43">
+        <f>ABS(C66-C67)/C67</f>
+        <v>0.000764877567818068</v>
+      </c>
+      <c r="D68" s="43">
+        <f>ABS(D66-D67)/D67</f>
+        <v>0.00026072392032610886</v>
+      </c>
+      <c r="E68" s="43">
+        <f>ABS(E66-E67)/E67</f>
+        <v>0.00012053465511544931</v>
+      </c>
+      <c r="F68" s="15" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>Char (oak_char)</t>
+        </is>
+      </c>
+      <c r="C69" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D69" s="6" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="E69" s="6" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F69" s="6" t="inlineStr"/>
+      <c r="G69" s="6" t="inlineStr"/>
+      <c r="H69" s="6" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="B70" s="7" t="inlineStr">
+        <is>
+          <t>composition du XML</t>
+        </is>
+      </c>
+      <c r="C70" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D70" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E70" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F70" s="15" t="inlineStr"/>
+      <c r="G70" s="15" t="inlineStr"/>
+      <c r="H70" s="15" t="inlineStr"/>
+    </row>
+    <row r="72" ht="18" customHeight="1">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t>§5 — CONTRÔLES ET VALIDATION CROISÉE</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="20" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="B73" s="20" t="inlineStr">
+        <is>
+          <t>Contrôle A — reconstruire le chêne depuis ses unités de répétition (traçable ligne à ligne)</t>
+        </is>
+      </c>
+      <c r="I73" s="27" t="inlineStr">
+        <is>
+          <t>w_E = Σ_i (part_i / Σ parts) · (ν_E,i·M_E / M_i)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" s="6" t="inlineStr"/>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D74" s="6" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="E74" s="6" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F74" s="6" t="inlineStr">
+        <is>
+          <t>Somme</t>
+        </is>
+      </c>
+      <c r="G74" s="6" t="inlineStr">
+        <is>
+          <t>écart / littérature [points]</t>
+        </is>
+      </c>
+      <c r="H74" s="6" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>chêne reconstruit [% masse]</t>
+        </is>
+      </c>
+      <c r="C75" s="9">
+        <f>SUMPRODUCT($C$29:$C$33,D29:D33/$G$29:$G$33)*Constantes!$C$7/$C$34*100</f>
+        <v>50.38950994879695</v>
+      </c>
+      <c r="D75" s="9">
+        <f>SUMPRODUCT($C$29:$C$33,E29:E33/$G$29:$G$33)*Constantes!$C$8/$C$34*100</f>
+        <v>6.039320485528451</v>
+      </c>
+      <c r="E75" s="9">
+        <f>SUMPRODUCT($C$29:$C$33,F29:F33/$G$29:$G$33)*Constantes!$C$9/$C$34*100</f>
+        <v>43.571169565674595</v>
+      </c>
+      <c r="F75" s="9">
+        <f>SUM(C75:E75)</f>
+        <v>100.0</v>
+      </c>
+      <c r="G75" s="9">
+        <f>MAX(ABS(C75-C44),ABS(D75-D44),ABS(E75-E44))</f>
+        <v>0.3895099487969489</v>
+      </c>
+      <c r="H75" s="15" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="B76" s="7" t="inlineStr">
+        <is>
+          <t>⇒ gaz de pyrolyse avec le chêne reconstruit (x_E)</t>
+        </is>
+      </c>
+      <c r="C76" s="24">
+        <f>(100*C75/$F$75/Constantes!$C$7-$E$47/Constantes!$C$7)/(100*C75/$F$75/Constantes!$C$7-$E$47/Constantes!$C$7+100*D75/$F$75/Constantes!$C$8+100*E75/$F$75/Constantes!$C$9)</f>
+        <v>0.2250033721577044</v>
+      </c>
+      <c r="D76" s="24">
+        <f>(100*D75/$F$75/Constantes!$C$8)/(100*C75/$F$75/Constantes!$C$7-$E$47/Constantes!$C$7+100*D75/$F$75/Constantes!$C$8+100*E75/$F$75/Constantes!$C$9)</f>
+        <v>0.5328096006041946</v>
+      </c>
+      <c r="E76" s="24">
+        <f>(100*E75/$F$75/Constantes!$C$9)/(100*C75/$F$75/Constantes!$C$7-$E$47/Constantes!$C$7+100*D75/$F$75/Constantes!$C$8+100*E75/$F$75/Constantes!$C$9)</f>
+        <v>0.24218702723810098</v>
+      </c>
+      <c r="F76" s="24">
+        <f>SUM(C76:E76)</f>
+        <v>1.0</v>
+      </c>
+      <c r="G76" s="15" t="inlineStr"/>
+      <c r="H76" s="15" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="B77" s="12" t="inlineStr">
+        <is>
+          <t>Attendu C 50.39 / H 6.04 / O 43.57, soit un gaz C:0.225 / H:0.533 / O:0.242. La reconstruction retombe sur l'analyse de littérature à 0.4 point près — bien mieux que pour le liège (4 points sur C) : l'unité dominante, l'anhydroglucose, est exacte, et il n'y a pas de subérine dont l'unité serait incertaine. L'écart sur le gaz (0.004 sur x_C) est négligeable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="20" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="B78" s="20" t="inlineStr">
+        <is>
+          <t>Contrôle B — rendement en char par additivité des constituants</t>
+        </is>
+      </c>
+      <c r="I78" s="27" t="inlineStr">
+        <is>
+          <t>y = Σ_i part_i · y_i / Σ parts</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" s="35" t="inlineStr">
+        <is>
+          <t>y_chêne par additivité</t>
+        </is>
+      </c>
+      <c r="C79" s="70">
+        <f>SUMPRODUCT($C$29:$C$33,$H$29:$H$33)/$C$34</f>
+        <v>0.21989795918367344</v>
+      </c>
+      <c r="I79" s="12" t="inlineStr">
+        <is>
+          <t>attendu 22.0 % — contre 20 % retenus : les deux voies sont COHÉRENTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" s="12" t="inlineStr">
+        <is>
+          <t>La cellulose, qui pèse 43 %, se dépolymérise en lévoglucosane et laisse peu de char ; la lignine et les tanins, aromatiques, en laissent le plus. Le rendement réel dépend fortement de la vitesse de chauffe : 20 % correspond à une pyrolyse lente, une pyrolyse flash descend vers 10-15 %.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="20" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="B81" s="20" t="inlineStr">
+        <is>
+          <t>Contrôle C — variante : char retenant H et O (char multi-élément)</t>
+        </is>
+      </c>
+      <c r="I81" s="27" t="inlineStr">
+        <is>
+          <t>n_E(char) = m_char · w_E,char / M_E ;  n_E(gaz) = n_E(bois) − n_E(char)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>char supposé [% masse]</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D82" s="6" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="E82" s="6" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F82" s="6" t="inlineStr">
+        <is>
+          <t>Somme</t>
+        </is>
+      </c>
+      <c r="G82" s="6" t="inlineStr"/>
+      <c r="H82" s="6" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="B83" s="7" t="inlineStr">
+        <is>
+          <t>hypothèse de travail</t>
+        </is>
+      </c>
+      <c r="C83" s="36" t="n">
+        <v>90</v>
+      </c>
+      <c r="D83" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="E83" s="36" t="n">
+        <v>8</v>
+      </c>
+      <c r="F83" s="9">
+        <f>SUM(C83:E83)</f>
+        <v>100.0</v>
+      </c>
+      <c r="G83" s="15" t="inlineStr"/>
+      <c r="H83" s="15" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="B84" s="7" t="inlineStr">
+        <is>
+          <t>moles d'atomes du char</t>
+        </is>
+      </c>
+      <c r="C84" s="26">
+        <f>$E$47*C83/100/Constantes!$C$7</f>
+        <v>1.498626259262343</v>
+      </c>
+      <c r="D84" s="26">
+        <f>$E$47*D83/100/Constantes!$C$8</f>
+        <v>0.39682539682539686</v>
+      </c>
+      <c r="E84" s="26">
+        <f>$E$47*E83/100/Constantes!$C$9</f>
+        <v>0.10000625039064942</v>
+      </c>
+      <c r="F84" s="26">
+        <f>SUM(C84:E84)</f>
+        <v>1.995457906478389</v>
+      </c>
+      <c r="G84" s="15" t="inlineStr"/>
+      <c r="H84" s="15" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="B85" s="7" t="inlineStr">
+        <is>
+          <t>⇒ oak_char multi-élément (x_E)</t>
+        </is>
+      </c>
+      <c r="C85" s="24">
+        <f>C84/$F$84</f>
+        <v>0.7510187282813391</v>
+      </c>
+      <c r="D85" s="24">
+        <f>D84/$F$84</f>
+        <v>0.19886432860200978</v>
+      </c>
+      <c r="E85" s="24">
+        <f>E84/$F$84</f>
+        <v>0.050116943116651255</v>
+      </c>
+      <c r="F85" s="24">
+        <f>SUM(C85:E85)</f>
+        <v>1.0</v>
+      </c>
+      <c r="G85" s="15" t="inlineStr"/>
+      <c r="H85" s="15" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="B86" s="7" t="inlineStr">
+        <is>
+          <t>⇒ gaz cohérent (x_E)</t>
+        </is>
+      </c>
+      <c r="C86" s="24">
+        <f>(C50-C84)/($F$50-$F$84)</f>
+        <v>0.2430218345104322</v>
+      </c>
+      <c r="D86" s="24">
+        <f>(D50-D84)/($F$50-$F$84)</f>
+        <v>0.5158088712034152</v>
+      </c>
+      <c r="E86" s="24">
+        <f>(E50-E84)/($F$50-$F$84)</f>
+        <v>0.24116929428615272</v>
+      </c>
+      <c r="F86" s="24">
+        <f>SUM(C86:E86)</f>
+        <v>1.0000000000000002</v>
+      </c>
+      <c r="G86" s="15" t="inlineStr"/>
+      <c r="H86" s="15" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="B87" s="12" t="inlineStr">
+        <is>
+          <t>Attendu char C:0.751, H:0.199, O:0.050 et gaz C:0.243, H:0.516, O:0.241. `-char-elem C` reste valable. Un char qui retient H et O laisse PLUS de carbone au gaz (x_C +0.022) : c'est automatique dans la fermeture élémentaire, pas si l'on recopie deux compositions de sources différentes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="18" customHeight="1">
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <t>§6 — SENSIBILITÉ</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="20" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="B90" s="20" t="inlineStr">
+        <is>
+          <t>Au rendement en char — LE paramètre du calcul</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="B91" s="6" t="inlineStr">
+        <is>
+          <t>y testé</t>
+        </is>
+      </c>
+      <c r="C91" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D91" s="6" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="E91" s="6" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F91" s="6" t="inlineStr"/>
+      <c r="G91" s="6" t="inlineStr">
+        <is>
+          <t>k = (1−y)/y</t>
+        </is>
+      </c>
+      <c r="H91" s="6" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="B92" s="28" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C92" s="24">
+        <f>($C$50-100*B92/Constantes!$C$7)/(($C$50-100*B92/Constantes!$C$7)+$D$50+$E$50)</f>
+        <v>0.2746444354050527</v>
+      </c>
+      <c r="D92" s="24">
+        <f>$D$50/(($C$50-100*B92/Constantes!$C$7)+$D$50+$E$50)</f>
+        <v>0.4990674928885301</v>
+      </c>
+      <c r="E92" s="24">
+        <f>$E$50/(($C$50-100*B92/Constantes!$C$7)+$D$50+$E$50)</f>
+        <v>0.2262880717064173</v>
+      </c>
+      <c r="F92" s="15" t="inlineStr"/>
+      <c r="G92" s="24">
+        <f>(1-B92)/B92</f>
+        <v>9.0</v>
+      </c>
+      <c r="H92" s="15" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="B93" s="28" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C93" s="24">
+        <f>($C$50-100*B93/Constantes!$C$7)/(($C$50-100*B93/Constantes!$C$7)+$D$50+$E$50)</f>
+        <v>0.24885728970795523</v>
+      </c>
+      <c r="D93" s="24">
+        <f>$D$50/(($C$50-100*B93/Constantes!$C$7)+$D$50+$E$50)</f>
+        <v>0.516809861983042</v>
+      </c>
+      <c r="E93" s="24">
+        <f>$E$50/(($C$50-100*B93/Constantes!$C$7)+$D$50+$E$50)</f>
+        <v>0.23433284830900278</v>
+      </c>
+      <c r="F93" s="15" t="inlineStr"/>
+      <c r="G93" s="24">
+        <f>(1-B93)/B93</f>
+        <v>5.666666666666667</v>
+      </c>
+      <c r="H93" s="15" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="B94" s="28" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C94" s="24">
+        <f>($C$50-100*B94/Constantes!$C$7)/(($C$50-100*B94/Constantes!$C$7)+$D$50+$E$50)</f>
+        <v>0.2211690379424878</v>
+      </c>
+      <c r="D94" s="24">
+        <f>$D$50/(($C$50-100*B94/Constantes!$C$7)+$D$50+$E$50)</f>
+        <v>0.5358602519787052</v>
+      </c>
+      <c r="E94" s="24">
+        <f>$E$50/(($C$50-100*B94/Constantes!$C$7)+$D$50+$E$50)</f>
+        <v>0.24297071007880694</v>
+      </c>
+      <c r="F94" s="15" t="inlineStr"/>
+      <c r="G94" s="24">
+        <f>(1-B94)/B94</f>
+        <v>4.0</v>
+      </c>
+      <c r="H94" s="15" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="B95" s="28" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C95" s="24">
+        <f>($C$50-100*B95/Constantes!$C$7)/(($C$50-100*B95/Constantes!$C$7)+$D$50+$E$50)</f>
+        <v>0.19136140111610234</v>
+      </c>
+      <c r="D95" s="24">
+        <f>$D$50/(($C$50-100*B95/Constantes!$C$7)+$D$50+$E$50)</f>
+        <v>0.5563688457029199</v>
+      </c>
+      <c r="E95" s="24">
+        <f>$E$50/(($C$50-100*B95/Constantes!$C$7)+$D$50+$E$50)</f>
+        <v>0.25226975318097794</v>
+      </c>
+      <c r="F95" s="15" t="inlineStr"/>
+      <c r="G95" s="24">
+        <f>(1-B95)/B95</f>
+        <v>3.0</v>
+      </c>
+      <c r="H95" s="15" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="B96" s="28" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C96" s="24">
+        <f>($C$50-100*B96/Constantes!$C$7)/(($C$50-100*B96/Constantes!$C$7)+$D$50+$E$50)</f>
+        <v>0.15918135429060362</v>
+      </c>
+      <c r="D96" s="24">
+        <f>$D$50/(($C$50-100*B96/Constantes!$C$7)+$D$50+$E$50)</f>
+        <v>0.5785097322889425</v>
+      </c>
+      <c r="E96" s="24">
+        <f>$E$50/(($C$50-100*B96/Constantes!$C$7)+$D$50+$E$50)</f>
+        <v>0.26230891342045404</v>
+      </c>
+      <c r="F96" s="15" t="inlineStr"/>
+      <c r="G96" s="24">
+        <f>(1-B96)/B96</f>
+        <v>2.3333333333333335</v>
+      </c>
+      <c r="H96" s="15" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="B97" s="12" t="inlineStr">
+        <is>
+          <t>±5 points de rendement déplacent le carbone du gaz de ∓0.03 et k de 3.0 à 5.7. Comme pour le liège, le rendement pèse bien plus sur la QUANTITÉ de gaz (k) que sur sa composition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="20" t="inlineStr">
+        <is>
+          <t>&gt;</t>
+        </is>
+      </c>
+      <c r="B98" s="20" t="inlineStr">
+        <is>
+          <t>À l'humidité du bois — l'eau part entièrement dans le gaz</t>
+        </is>
+      </c>
+      <c r="I98" s="27" t="inlineStr">
+        <is>
+          <t>m_eau = 100·h/(1−h) ;  n_H += 2·n_eau ;  n_O += n_eau</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="B99" s="6" t="inlineStr">
+        <is>
+          <t>humidité h (base humide)</t>
+        </is>
+      </c>
+      <c r="C99" s="6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D99" s="6" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="E99" s="6" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="F99" s="6" t="inlineStr">
+        <is>
+          <t>char / bois humide</t>
+        </is>
+      </c>
+      <c r="G99" s="6" t="inlineStr">
+        <is>
+          <t>k = m_gaz/m_char</t>
+        </is>
+      </c>
+      <c r="H99" s="6" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="B100" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="C100" s="24">
+        <f>$C$52/($C$52+($D$52+2*(100*B100/(1-B100)/(2*Constantes!$C$8+Constantes!$C$9)))+($E$52+(100*B100/(1-B100)/(2*Constantes!$C$8+Constantes!$C$9))))</f>
+        <v>0.2211690379424878</v>
+      </c>
+      <c r="D100" s="24">
+        <f>($D$52+2*(100*B100/(1-B100)/(2*Constantes!$C$8+Constantes!$C$9)))/($C$52+($D$52+2*(100*B100/(1-B100)/(2*Constantes!$C$8+Constantes!$C$9)))+($E$52+(100*B100/(1-B100)/(2*Constantes!$C$8+Constantes!$C$9))))</f>
+        <v>0.5358602519787052</v>
+      </c>
+      <c r="E100" s="24">
+        <f>($E$52+(100*B100/(1-B100)/(2*Constantes!$C$8+Constantes!$C$9)))/($C$52+($D$52+2*(100*B100/(1-B100)/(2*Constantes!$C$8+Constantes!$C$9)))+($E$52+(100*B100/(1-B100)/(2*Constantes!$C$8+Constantes!$C$9))))</f>
+        <v>0.24297071007880694</v>
+      </c>
+      <c r="F100" s="24">
+        <f>$E$47/(100+100*B100/(1-B100))</f>
+        <v>0.2</v>
+      </c>
+      <c r="G100" s="24">
+        <f>($F$47+100*B100/(1-B100))/$E$47</f>
+        <v>4.0</v>
+      </c>
+      <c r="H100" s="15" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="B101" s="28" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="C101" s="24">
+        <f>$C$52/($C$52+($D$52+2*(100*B101/(1-B101)/(2*Constantes!$C$8+Constantes!$C$9)))+($E$52+(100*B101/(1-B101)/(2*Constantes!$C$8+Constantes!$C$9))))</f>
+        <v>0.19603280752539232</v>
+      </c>
+      <c r="D101" s="24">
+        <f>($D$52+2*(100*B101/(1-B101)/(2*Constantes!$C$8+Constantes!$C$9)))/($C$52+($D$52+2*(100*B101/(1-B101)/(2*Constantes!$C$8+Constantes!$C$9)))+($E$52+(100*B101/(1-B101)/(2*Constantes!$C$8+Constantes!$C$9))))</f>
+        <v>0.5507266193971219</v>
+      </c>
+      <c r="E101" s="24">
+        <f>($E$52+(100*B101/(1-B101)/(2*Constantes!$C$8+Constantes!$C$9)))/($C$52+($D$52+2*(100*B101/(1-B101)/(2*Constantes!$C$8+Constantes!$C$9)))+($E$52+(100*B101/(1-B101)/(2*Constantes!$C$8+Constantes!$C$9))))</f>
+        <v>0.2532405730774859</v>
+      </c>
+      <c r="F101" s="24">
+        <f>$E$47/(100+100*B101/(1-B101))</f>
+        <v>0.184</v>
+      </c>
+      <c r="G101" s="24">
+        <f>($F$47+100*B101/(1-B101))/$E$47</f>
+        <v>4.434782608695652</v>
+      </c>
+      <c r="H101" s="15" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="B102" s="28" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="C102" s="24">
+        <f>$C$52/($C$52+($D$52+2*(100*B102/(1-B102)/(2*Constantes!$C$8+Constantes!$C$9)))+($E$52+(100*B102/(1-B102)/(2*Constantes!$C$8+Constantes!$C$9))))</f>
+        <v>0.18414188018509986</v>
+      </c>
+      <c r="D102" s="24">
+        <f>($D$52+2*(100*B102/(1-B102)/(2*Constantes!$C$8+Constantes!$C$9)))/($C$52+($D$52+2*(100*B102/(1-B102)/(2*Constantes!$C$8+Constantes!$C$9)))+($E$52+(100*B102/(1-B102)/(2*Constantes!$C$8+Constantes!$C$9))))</f>
+        <v>0.5577592926282782</v>
+      </c>
+      <c r="E102" s="24">
+        <f>($E$52+(100*B102/(1-B102)/(2*Constantes!$C$8+Constantes!$C$9)))/($C$52+($D$52+2*(100*B102/(1-B102)/(2*Constantes!$C$8+Constantes!$C$9)))+($E$52+(100*B102/(1-B102)/(2*Constantes!$C$8+Constantes!$C$9))))</f>
+        <v>0.2580988271866221</v>
+      </c>
+      <c r="F102" s="24">
+        <f>$E$47/(100+100*B102/(1-B102))</f>
+        <v>0.176</v>
+      </c>
+      <c r="G102" s="24">
+        <f>($F$47+100*B102/(1-B102))/$E$47</f>
+        <v>4.681818181818182</v>
+      </c>
+      <c r="H102" s="15" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="B103" s="12" t="inlineStr">
+        <is>
+          <t>Un bois stabilisé à l'air (12 %) donne un gaz C:0.184 et k = 4.68 : l'effet sur la composition dépasse celui de ±5 points de rendement. Préciser « sec » ou « à X % d'humidité » dans l'énoncé.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="18" customHeight="1">
+      <c r="A105" s="4" t="inlineStr">
         <is>
           <t>§7 — RÉPONSE MATÉRIAU (n'entre PAS dans le XML)</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="B53" s="35" t="inlineStr">
-        <is>
-          <t>couplage k = B'g / B'c</t>
-        </is>
-      </c>
-      <c r="C53" s="70" t="n">
-        <v>0</v>
-      </c>
-      <c r="I53" s="12" t="inlineStr">
-        <is>
-          <t>aucun gaz de pyrolyse — le graphite est le seul matériau du classeur à k = 0</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="B54" s="35" t="inlineStr">
-        <is>
-          <t>récession par unité de flux, B'c/ρ_c à 300 K [m³/kg]</t>
-        </is>
-      </c>
-      <c r="C54" s="41">
-        <f>C19*Constantes!$C$7/(2*Constantes!$C$9)/C20</f>
-        <v>4.857026857405357e-05</v>
-      </c>
-      <c r="I54" s="12" t="inlineStr">
-        <is>
-          <t>ṡ = B'c·ṁe/ρ_c</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="18" customHeight="1">
-      <c r="A56" s="4" t="inlineStr">
+    <row r="106">
+      <c r="B106" s="35" t="inlineStr">
+        <is>
+          <t>k = B'g/B'c = m_gaz / m_char = (1 − y)/y</t>
+        </is>
+      </c>
+      <c r="C106" s="46">
+        <f>F47/E47</f>
+        <v>4.0</v>
+      </c>
+      <c r="I106" s="12" t="inlineStr">
+        <is>
+          <t>attendu 4.0 — le même que le liège/phénolique, QUINZE FOIS le TACOT (0.273)</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="B107" s="35" t="inlineStr">
+        <is>
+          <t>ρ char [kg/m³] = y · ρ_v / (V_char/V_v)</t>
+        </is>
+      </c>
+      <c r="C107" s="45">
+        <f>$C$37*C38/C39</f>
+        <v>254.54545454545453</v>
+      </c>
+      <c r="I107" s="12" t="inlineStr">
+        <is>
+          <t>≈ 255 kg/m³ avec le retrait supposé — à MESURER</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="B108" s="35" t="inlineStr">
+        <is>
+          <t>k si l'on prenait les densités : (ρ_v − ρ_c)/ρ_c</t>
+        </is>
+      </c>
+      <c r="C108" s="46">
+        <f>(C38-C107)/C107</f>
+        <v>1.7500000000000002</v>
+      </c>
+      <c r="I108" s="12" t="inlineStr">
+        <is>
+          <t>1.75 — plus de deux fois trop peu : l'identité suppose un volume constant</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="B109" s="12" t="inlineStr">
+        <is>
+          <t>Conséquences pratiques : (1) balayer B'g jusqu'à ~10 (les tables oak_bprime vont à B'g = 5 et le balayage du point de fonctionnement à 10) ; (2) la récession se lit sur la ρ_char MESURÉE, pas sur 0.20·ρ_v = 140 kg/m³ ; (3) le gaz porte plus d'oxygène que de carbone (O/C = 1.10) : au-dessus de ~1500 K il OXYDE le char, et B'c CROÎT avec B'g (1 atm, 3000 K : 0.177 à B'g = 0, 0.79 à B'g = 5) — l'inverse du liège, dont le soufflage protège le char. Point de fonctionnement à 1 atm : B'c = 0.127 / 0.213 / 0.430 à 1000 / 2000 / 3000 K (oak_bprime).</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="18" customHeight="1">
+      <c r="A111" s="4" t="inlineStr">
         <is>
           <t>§8 — BLOC XML</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="B57" s="29" t="inlineStr">
+    <row r="112">
+      <c r="B112" s="29" t="inlineStr">
         <is>
           <t>&lt;mixture thermo_db="NASA-9"&gt;</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="B58" s="29" t="inlineStr">
+    <row r="113">
+      <c r="B113" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">    &lt;species&gt;</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="B59" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        N O NO N2 O2 C C2 C3 CN CO CO2 C(gr)</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="B60" s="29" t="inlineStr">
+    <row r="114">
+      <c r="B114" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">       C H O N CH4 CN CO CO2 C2 C2H C2H2,acetylene C3 C4 C4H2,butadiyne C5</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="B115" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">       HCN H2 H2O N2 CH2OH CNN CNC CNCOCN C6H6 HNC C(gr)</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="B116" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">    &lt;/species&gt;</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="B61" s="29" t="inlineStr">
+    <row r="117">
+      <c r="B117" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">    &lt;element_compositions default="air"&gt;</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="B62" s="29" t="inlineStr">
+    <row r="118">
+      <c r="B118" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">        &lt;composition name="air"&gt;N:0.79, O:0.21&lt;/composition&gt;</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="B63" s="29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">        &lt;composition name="pyro"&gt;C:1.0&lt;/composition&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="B64" s="29" t="inlineStr">
+    <row r="119">
+      <c r="B119" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        &lt;composition name="oak_pyro"&gt;C:0.221, H:0.536, O:0.243&lt;/composition&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="B120" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        &lt;composition name="oak_char"&gt;C:1.0&lt;/composition&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="B121" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">    &lt;/element_compositions&gt;</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="B65" s="29" t="inlineStr">
+    <row r="122">
+      <c r="B122" s="29" t="inlineStr">
         <is>
           <t>&lt;/mixture&gt;</t>
         </is>
       </c>
     </row>
-    <row r="67" ht="16" customHeight="1">
-      <c r="B67" s="5" t="inlineStr">
-        <is>
-          <t>bprime -T 300:25:5000 -P &lt;P&gt; -b 0.0 -m carbon-air -bl air -py pyro</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="36">
+  <mergeCells count="52">
+    <mergeCell ref="B97:I97"/>
+    <mergeCell ref="A41:I41"/>
     <mergeCell ref="B62:I62"/>
-    <mergeCell ref="A56:I56"/>
-    <mergeCell ref="B59:I59"/>
+    <mergeCell ref="B25:I25"/>
+    <mergeCell ref="B109:I109"/>
+    <mergeCell ref="A89:I89"/>
+    <mergeCell ref="B121:I121"/>
+    <mergeCell ref="B115:I115"/>
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="B15:H15"/>
-    <mergeCell ref="B31:I31"/>
-    <mergeCell ref="B27:I27"/>
+    <mergeCell ref="A105:I105"/>
+    <mergeCell ref="B122:I122"/>
+    <mergeCell ref="A21:I21"/>
+    <mergeCell ref="B45:H45"/>
     <mergeCell ref="B58:I58"/>
     <mergeCell ref="A2:I2"/>
-    <mergeCell ref="B26:H26"/>
-    <mergeCell ref="A33:I33"/>
+    <mergeCell ref="B77:I77"/>
     <mergeCell ref="A5:I5"/>
-    <mergeCell ref="A17:I17"/>
-    <mergeCell ref="B60:I60"/>
-    <mergeCell ref="B67:I67"/>
-    <mergeCell ref="A22:I22"/>
-    <mergeCell ref="B61:I61"/>
-    <mergeCell ref="B57:I57"/>
-    <mergeCell ref="A38:I38"/>
-    <mergeCell ref="A52:I52"/>
-    <mergeCell ref="B29:I29"/>
-    <mergeCell ref="B12:H12"/>
-    <mergeCell ref="B39:H39"/>
-    <mergeCell ref="A44:I44"/>
-    <mergeCell ref="B65:I65"/>
-    <mergeCell ref="B23:H23"/>
-    <mergeCell ref="B40:I40"/>
+    <mergeCell ref="B117:I117"/>
+    <mergeCell ref="B120:I120"/>
+    <mergeCell ref="B16:H16"/>
+    <mergeCell ref="B54:H54"/>
+    <mergeCell ref="B90:H90"/>
+    <mergeCell ref="B59:H59"/>
+    <mergeCell ref="B81:H81"/>
+    <mergeCell ref="A72:I72"/>
+    <mergeCell ref="B119:I119"/>
+    <mergeCell ref="B22:H22"/>
+    <mergeCell ref="B53:I53"/>
+    <mergeCell ref="B116:I116"/>
+    <mergeCell ref="B18:H18"/>
+    <mergeCell ref="B27:H27"/>
+    <mergeCell ref="B87:I87"/>
+    <mergeCell ref="A13:I13"/>
+    <mergeCell ref="B103:I103"/>
+    <mergeCell ref="A111:I111"/>
+    <mergeCell ref="B112:I112"/>
+    <mergeCell ref="B48:H48"/>
+    <mergeCell ref="B42:H42"/>
+    <mergeCell ref="B118:I118"/>
+    <mergeCell ref="B98:H98"/>
+    <mergeCell ref="A64:I64"/>
     <mergeCell ref="B14:H14"/>
-    <mergeCell ref="B30:I30"/>
-    <mergeCell ref="A11:I11"/>
-    <mergeCell ref="B64:I64"/>
-    <mergeCell ref="B13:H13"/>
+    <mergeCell ref="B17:H17"/>
+    <mergeCell ref="B73:H73"/>
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="B63:I63"/>
-    <mergeCell ref="B50:I50"/>
-    <mergeCell ref="B28:H28"/>
+    <mergeCell ref="B80:I80"/>
+    <mergeCell ref="B78:H78"/>
+    <mergeCell ref="B114:I114"/>
+    <mergeCell ref="B19:H19"/>
+    <mergeCell ref="B35:I35"/>
+    <mergeCell ref="B113:I113"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>